<commit_message>
Update forecast data 2026-05-30_22-19-20
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -1072,7 +1072,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.898064091961442</v>
+        <v>4.898069501238354</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1080,7 +1080,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.892934160761559</v>
+        <v>4.892941165807041</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1088,7 +1088,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.878559249589901</v>
+        <v>4.878679297592601</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1096,7 +1096,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.864557487993167</v>
+        <v>4.864733494956884</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1104,7 +1104,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.859666954539319</v>
+        <v>4.859811251879885</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1112,7 +1112,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.841849868698081</v>
+        <v>4.841976474290608</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1120,7 +1120,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.831419720977332</v>
+        <v>4.831704400688444</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1128,7 +1128,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.834719431712154</v>
+        <v>4.834925291066625</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1136,7 +1136,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.888472683656829</v>
+        <v>4.888517227668712</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1144,7 +1144,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.894167211056487</v>
+        <v>4.89392676157999</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1152,7 +1152,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.898143826681418</v>
+        <v>4.897415545304445</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1160,7 +1160,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.901386658927887</v>
+        <v>4.903541652600095</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1168,7 +1168,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.900558772272453</v>
+        <v>4.903096002719311</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1176,7 +1176,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.876976632350926</v>
+        <v>4.880080449052318</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-05-30_22-50-39
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -357,7 +357,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B102"/>
+  <dimension ref="A1:B103"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" style="1" customWidth="1"/>
@@ -1168,7 +1168,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.903096002719311</v>
+        <v>4.902999083812658</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1176,7 +1176,15 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.880080449052318</v>
+        <v>4.879845562696071</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2">
+      <c r="A103" s="2">
+        <v>46276</v>
+      </c>
+      <c r="B103">
+        <v>4.876751492213141</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-06-01_08-07-57
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -357,7 +357,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B103"/>
+  <dimension ref="A1:B104"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" style="1" customWidth="1"/>
@@ -696,7 +696,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712936785384079</v>
+        <v>4.712932183328753</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -704,7 +704,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711192829760884</v>
+        <v>4.711214563655856</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -712,7 +712,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.719605034084739</v>
+        <v>4.719631215107587</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -720,7 +720,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.705733911676118</v>
+        <v>4.705788348171614</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -728,7 +728,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.693067016141562</v>
+        <v>4.693122066994401</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -736,7 +736,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.677131323477594</v>
+        <v>4.677186854323957</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -744,7 +744,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.672137745020536</v>
+        <v>4.672193377450561</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -752,7 +752,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.685215121991877</v>
+        <v>4.685270647430218</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -760,7 +760,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.700921974918149</v>
+        <v>4.700988042504145</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -768,7 +768,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.704625713474441</v>
+        <v>4.704669446882999</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -776,7 +776,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.693676720613981</v>
+        <v>4.693721369463404</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -784,7 +784,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.663621432144661</v>
+        <v>4.663669910151888</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -792,7 +792,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649509417059265</v>
+        <v>4.649514156344575</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -800,7 +800,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.640995649010753</v>
+        <v>4.641011663601414</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -808,7 +808,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.635962528828301</v>
+        <v>4.635973904235275</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -816,7 +816,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633378674428384</v>
+        <v>4.633404885003799</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -824,7 +824,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.63725580478787</v>
+        <v>4.637260368931736</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -832,7 +832,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634790173944906</v>
+        <v>4.634774691872143</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -840,7 +840,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.628613160456835</v>
+        <v>4.62856922862416</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -848,7 +848,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.624947670339617</v>
+        <v>4.624900243092027</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -856,7 +856,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.600294755880086</v>
+        <v>4.600247727707352</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -864,7 +864,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.581982440933707</v>
+        <v>4.581875965376661</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -872,7 +872,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.564728267345042</v>
+        <v>4.56455378011229</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -880,7 +880,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.528557637989003</v>
+        <v>4.528303373876065</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -888,7 +888,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.528066170974466</v>
+        <v>4.52770752882156</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -896,7 +896,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.541692827851181</v>
+        <v>4.541301475583533</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -904,7 +904,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.560675901016843</v>
+        <v>4.560281886521748</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -912,7 +912,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.594226732615766</v>
+        <v>4.593791606188526</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -920,7 +920,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.615410269900954</v>
+        <v>4.614877485274593</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -928,7 +928,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.689944168702922</v>
+        <v>4.689330727799398</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -936,7 +936,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.726444653908651</v>
+        <v>4.725793412214621</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -944,7 +944,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.791889748975263</v>
+        <v>4.79130453023603</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -952,7 +952,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.821554310149132</v>
+        <v>4.821209003958732</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -960,7 +960,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.819051878725599</v>
+        <v>4.818720284636064</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -968,7 +968,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.828149865804882</v>
+        <v>4.827826790496798</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -976,7 +976,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.863077937699277</v>
+        <v>4.863052559426609</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -984,7 +984,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855448911644942</v>
+        <v>4.855439440747269</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -992,7 +992,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.849034792413009</v>
+        <v>4.849198362396718</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1000,7 +1000,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.827208414082759</v>
+        <v>4.82733459962648</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1008,7 +1008,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.83419655944717</v>
+        <v>4.834357580818274</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1016,7 +1016,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.88433864235864</v>
+        <v>4.884616845429106</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1024,7 +1024,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.913448964807747</v>
+        <v>4.913628600217725</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1032,7 +1032,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.922644104593459</v>
+        <v>4.922823267946093</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1040,7 +1040,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.913047060138272</v>
+        <v>4.91320730767155</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1048,7 +1048,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.894641214494123</v>
+        <v>4.894771719880164</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1056,7 +1056,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.890957409543572</v>
+        <v>4.8911649398165</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1064,7 +1064,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.892791027362668</v>
+        <v>4.889975509872036</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1072,7 +1072,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.898069501238354</v>
+        <v>4.894273340865623</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1080,7 +1080,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.892941165807041</v>
+        <v>4.889510164089134</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1088,7 +1088,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.878679297592601</v>
+        <v>4.876315880921263</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1096,7 +1096,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.864733494956884</v>
+        <v>4.863332075900846</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1104,7 +1104,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.859811251879885</v>
+        <v>4.858908418295761</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1112,7 +1112,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.841976474290608</v>
+        <v>4.842813628993508</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1120,7 +1120,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.831704400688444</v>
+        <v>4.833979577403978</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1128,7 +1128,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.834925291066625</v>
+        <v>4.838314182564192</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1136,7 +1136,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.888517227668712</v>
+        <v>4.885163532372392</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1144,7 +1144,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.89392676157999</v>
+        <v>4.8892399749263</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1152,7 +1152,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.897415545304445</v>
+        <v>4.891253848457051</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1160,7 +1160,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.903541652600095</v>
+        <v>4.898970622779578</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1168,7 +1168,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.902999083812658</v>
+        <v>4.90167478598809</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1176,7 +1176,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.879845562696071</v>
+        <v>4.879668435555153</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1184,7 +1184,15 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.876751492213141</v>
+        <v>4.876511853098584</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2">
+      <c r="A104" s="2">
+        <v>46283</v>
+      </c>
+      <c r="B104">
+        <v>4.87121894085697</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-06-20_12-55-04
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -30,8 +30,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -47,7 +55,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -55,13 +63,31 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -357,22 +383,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B104"/>
+  <dimension ref="A1:B105"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" s="2">
+      <c r="A2" s="3">
         <v>44743</v>
       </c>
       <c r="B2">
@@ -380,7 +406,7 @@
       </c>
     </row>
     <row r="3" spans="1:2">
-      <c r="A3" s="2">
+      <c r="A3" s="3">
         <v>44778</v>
       </c>
       <c r="B3">
@@ -388,7 +414,7 @@
       </c>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4" s="2">
+      <c r="A4" s="3">
         <v>44806</v>
       </c>
       <c r="B4">
@@ -396,7 +422,7 @@
       </c>
     </row>
     <row r="5" spans="1:2">
-      <c r="A5" s="2">
+      <c r="A5" s="3">
         <v>44841</v>
       </c>
       <c r="B5">
@@ -404,7 +430,7 @@
       </c>
     </row>
     <row r="6" spans="1:2">
-      <c r="A6" s="2">
+      <c r="A6" s="3">
         <v>44869</v>
       </c>
       <c r="B6">
@@ -412,7 +438,7 @@
       </c>
     </row>
     <row r="7" spans="1:2">
-      <c r="A7" s="2">
+      <c r="A7" s="3">
         <v>44897</v>
       </c>
       <c r="B7">
@@ -420,7 +446,7 @@
       </c>
     </row>
     <row r="8" spans="1:2">
-      <c r="A8" s="2">
+      <c r="A8" s="3">
         <v>44932</v>
       </c>
       <c r="B8">
@@ -428,7 +454,7 @@
       </c>
     </row>
     <row r="9" spans="1:2">
-      <c r="A9" s="2">
+      <c r="A9" s="3">
         <v>44960</v>
       </c>
       <c r="B9">
@@ -436,7 +462,7 @@
       </c>
     </row>
     <row r="10" spans="1:2">
-      <c r="A10" s="2">
+      <c r="A10" s="3">
         <v>44988</v>
       </c>
       <c r="B10">
@@ -444,7 +470,7 @@
       </c>
     </row>
     <row r="11" spans="1:2">
-      <c r="A11" s="2">
+      <c r="A11" s="3">
         <v>45016</v>
       </c>
       <c r="B11">
@@ -452,7 +478,7 @@
       </c>
     </row>
     <row r="12" spans="1:2">
-      <c r="A12" s="2">
+      <c r="A12" s="3">
         <v>45051</v>
       </c>
       <c r="B12">
@@ -460,7 +486,7 @@
       </c>
     </row>
     <row r="13" spans="1:2">
-      <c r="A13" s="2">
+      <c r="A13" s="3">
         <v>45079</v>
       </c>
       <c r="B13">
@@ -468,7 +494,7 @@
       </c>
     </row>
     <row r="14" spans="1:2">
-      <c r="A14" s="2">
+      <c r="A14" s="3">
         <v>45107</v>
       </c>
       <c r="B14">
@@ -476,7 +502,7 @@
       </c>
     </row>
     <row r="15" spans="1:2">
-      <c r="A15" s="2">
+      <c r="A15" s="3">
         <v>45142</v>
       </c>
       <c r="B15">
@@ -484,7 +510,7 @@
       </c>
     </row>
     <row r="16" spans="1:2">
-      <c r="A16" s="2">
+      <c r="A16" s="3">
         <v>45170</v>
       </c>
       <c r="B16">
@@ -492,7 +518,7 @@
       </c>
     </row>
     <row r="17" spans="1:2">
-      <c r="A17" s="2">
+      <c r="A17" s="3">
         <v>45205</v>
       </c>
       <c r="B17">
@@ -500,7 +526,7 @@
       </c>
     </row>
     <row r="18" spans="1:2">
-      <c r="A18" s="2">
+      <c r="A18" s="3">
         <v>45233</v>
       </c>
       <c r="B18">
@@ -508,7 +534,7 @@
       </c>
     </row>
     <row r="19" spans="1:2">
-      <c r="A19" s="2">
+      <c r="A19" s="3">
         <v>45261</v>
       </c>
       <c r="B19">
@@ -516,7 +542,7 @@
       </c>
     </row>
     <row r="20" spans="1:2">
-      <c r="A20" s="2">
+      <c r="A20" s="3">
         <v>45296</v>
       </c>
       <c r="B20">
@@ -524,7 +550,7 @@
       </c>
     </row>
     <row r="21" spans="1:2">
-      <c r="A21" s="2">
+      <c r="A21" s="3">
         <v>45324</v>
       </c>
       <c r="B21">
@@ -532,7 +558,7 @@
       </c>
     </row>
     <row r="22" spans="1:2">
-      <c r="A22" s="2">
+      <c r="A22" s="3">
         <v>45352</v>
       </c>
       <c r="B22">
@@ -540,7 +566,7 @@
       </c>
     </row>
     <row r="23" spans="1:2">
-      <c r="A23" s="2">
+      <c r="A23" s="3">
         <v>45387</v>
       </c>
       <c r="B23">
@@ -548,7 +574,7 @@
       </c>
     </row>
     <row r="24" spans="1:2">
-      <c r="A24" s="2">
+      <c r="A24" s="3">
         <v>45415</v>
       </c>
       <c r="B24">
@@ -556,7 +582,7 @@
       </c>
     </row>
     <row r="25" spans="1:2">
-      <c r="A25" s="2">
+      <c r="A25" s="3">
         <v>45443</v>
       </c>
       <c r="B25">
@@ -564,7 +590,7 @@
       </c>
     </row>
     <row r="26" spans="1:2">
-      <c r="A26" s="2">
+      <c r="A26" s="3">
         <v>45478</v>
       </c>
       <c r="B26">
@@ -572,7 +598,7 @@
       </c>
     </row>
     <row r="27" spans="1:2">
-      <c r="A27" s="2">
+      <c r="A27" s="3">
         <v>45506</v>
       </c>
       <c r="B27">
@@ -580,7 +606,7 @@
       </c>
     </row>
     <row r="28" spans="1:2">
-      <c r="A28" s="2">
+      <c r="A28" s="3">
         <v>45541</v>
       </c>
       <c r="B28">
@@ -588,7 +614,7 @@
       </c>
     </row>
     <row r="29" spans="1:2">
-      <c r="A29" s="2">
+      <c r="A29" s="3">
         <v>45569</v>
       </c>
       <c r="B29">
@@ -596,7 +622,7 @@
       </c>
     </row>
     <row r="30" spans="1:2">
-      <c r="A30" s="2">
+      <c r="A30" s="3">
         <v>45597</v>
       </c>
       <c r="B30">
@@ -604,7 +630,7 @@
       </c>
     </row>
     <row r="31" spans="1:2">
-      <c r="A31" s="2">
+      <c r="A31" s="3">
         <v>45632</v>
       </c>
       <c r="B31">
@@ -612,7 +638,7 @@
       </c>
     </row>
     <row r="32" spans="1:2">
-      <c r="A32" s="2">
+      <c r="A32" s="3">
         <v>45660</v>
       </c>
       <c r="B32">
@@ -620,7 +646,7 @@
       </c>
     </row>
     <row r="33" spans="1:2">
-      <c r="A33" s="2">
+      <c r="A33" s="3">
         <v>45688</v>
       </c>
       <c r="B33">
@@ -628,7 +654,7 @@
       </c>
     </row>
     <row r="34" spans="1:2">
-      <c r="A34" s="2">
+      <c r="A34" s="3">
         <v>45716</v>
       </c>
       <c r="B34">
@@ -636,7 +662,7 @@
       </c>
     </row>
     <row r="35" spans="1:2">
-      <c r="A35" s="2">
+      <c r="A35" s="3">
         <v>45751</v>
       </c>
       <c r="B35">
@@ -644,7 +670,7 @@
       </c>
     </row>
     <row r="36" spans="1:2">
-      <c r="A36" s="2">
+      <c r="A36" s="3">
         <v>45779</v>
       </c>
       <c r="B36">
@@ -652,7 +678,7 @@
       </c>
     </row>
     <row r="37" spans="1:2">
-      <c r="A37" s="2">
+      <c r="A37" s="3">
         <v>45814</v>
       </c>
       <c r="B37">
@@ -660,7 +686,7 @@
       </c>
     </row>
     <row r="38" spans="1:2">
-      <c r="A38" s="2">
+      <c r="A38" s="3">
         <v>45821</v>
       </c>
       <c r="B38">
@@ -668,7 +694,7 @@
       </c>
     </row>
     <row r="39" spans="1:2">
-      <c r="A39" s="2">
+      <c r="A39" s="3">
         <v>45828</v>
       </c>
       <c r="B39">
@@ -676,7 +702,7 @@
       </c>
     </row>
     <row r="40" spans="1:2">
-      <c r="A40" s="2">
+      <c r="A40" s="3">
         <v>45835</v>
       </c>
       <c r="B40">
@@ -684,7 +710,7 @@
       </c>
     </row>
     <row r="41" spans="1:2">
-      <c r="A41" s="2">
+      <c r="A41" s="3">
         <v>45842</v>
       </c>
       <c r="B41">
@@ -692,507 +718,515 @@
       </c>
     </row>
     <row r="42" spans="1:2">
-      <c r="A42" s="2">
+      <c r="A42" s="3">
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712923621003797</v>
+        <v>4.712919631583167</v>
       </c>
     </row>
     <row r="43" spans="1:2">
-      <c r="A43" s="2">
+      <c r="A43" s="3">
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711254967741341</v>
+        <v>4.711273778521764</v>
       </c>
     </row>
     <row r="44" spans="1:2">
-      <c r="A44" s="2">
+      <c r="A44" s="3">
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.719679940738682</v>
+        <v>4.719702649767003</v>
       </c>
     </row>
     <row r="45" spans="1:2">
-      <c r="A45" s="2">
+      <c r="A45" s="3">
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.705889620661495</v>
+        <v>4.705936802034234</v>
       </c>
     </row>
     <row r="46" spans="1:2">
-      <c r="A46" s="2">
+      <c r="A46" s="3">
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.693224482870868</v>
+        <v>4.693272197137578</v>
       </c>
     </row>
     <row r="47" spans="1:2">
-      <c r="A47" s="2">
+      <c r="A47" s="3">
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.677290162901785</v>
+        <v>4.677338292950605</v>
       </c>
     </row>
     <row r="48" spans="1:2">
-      <c r="A48" s="2">
+      <c r="A48" s="3">
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.672296879722987</v>
+        <v>4.672345102101879</v>
       </c>
     </row>
     <row r="49" spans="1:2">
-      <c r="A49" s="2">
+      <c r="A49" s="3">
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.685373963313436</v>
+        <v>4.685422104471833</v>
       </c>
     </row>
     <row r="50" spans="1:2">
-      <c r="A50" s="2">
+      <c r="A50" s="3">
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.701111066285661</v>
+        <v>4.701168431320468</v>
       </c>
     </row>
     <row r="51" spans="1:2">
-      <c r="A51" s="2">
+      <c r="A51" s="3">
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.704750895979952</v>
+        <v>4.704788881232743</v>
       </c>
     </row>
     <row r="52" spans="1:2">
-      <c r="A52" s="2">
+      <c r="A52" s="3">
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.693804516135636</v>
+        <v>4.693843289825237</v>
       </c>
     </row>
     <row r="53" spans="1:2">
-      <c r="A53" s="2">
+      <c r="A53" s="3">
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.663760172988053</v>
+        <v>4.663802258654688</v>
       </c>
     </row>
     <row r="54" spans="1:2">
-      <c r="A54" s="2">
+      <c r="A54" s="3">
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649523327614615</v>
+        <v>4.649527757753823</v>
       </c>
     </row>
     <row r="55" spans="1:2">
-      <c r="A55" s="2">
+      <c r="A55" s="3">
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641041742192674</v>
+        <v>4.641055882390525</v>
       </c>
     </row>
     <row r="56" spans="1:2">
-      <c r="A56" s="2">
+      <c r="A56" s="3">
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.635995079123482</v>
+        <v>4.636004949761356</v>
       </c>
     </row>
     <row r="57" spans="1:2">
-      <c r="A57" s="2">
+      <c r="A57" s="3">
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633453743734549</v>
+        <v>4.633476549286308</v>
       </c>
     </row>
     <row r="58" spans="1:2">
-      <c r="A58" s="2">
+      <c r="A58" s="3">
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637269110019139</v>
+        <v>4.637273293332782</v>
       </c>
     </row>
     <row r="59" spans="1:2">
-      <c r="A59" s="2">
+      <c r="A59" s="3">
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634745932877053</v>
+        <v>4.634732554225784</v>
       </c>
     </row>
     <row r="60" spans="1:2">
-      <c r="A60" s="2">
+      <c r="A60" s="3">
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.628487344579236</v>
+        <v>4.628449127804408</v>
       </c>
     </row>
     <row r="61" spans="1:2">
-      <c r="A61" s="2">
+      <c r="A61" s="3">
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.624811908020865</v>
+        <v>4.624770708552843</v>
       </c>
     </row>
     <row r="62" spans="1:2">
-      <c r="A62" s="2">
+      <c r="A62" s="3">
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.600160163235186</v>
+        <v>4.600119335745388</v>
       </c>
     </row>
     <row r="63" spans="1:2">
-      <c r="A63" s="2">
+      <c r="A63" s="3">
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.581678384656728</v>
+        <v>4.581586560179585</v>
       </c>
     </row>
     <row r="64" spans="1:2">
-      <c r="A64" s="2">
+      <c r="A64" s="3">
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.56423023671818</v>
+        <v>4.564079981411284</v>
       </c>
     </row>
     <row r="65" spans="1:2">
-      <c r="A65" s="2">
+      <c r="A65" s="3">
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.527831457879266</v>
+        <v>4.527612100616176</v>
       </c>
     </row>
     <row r="66" spans="1:2">
-      <c r="A66" s="2">
+      <c r="A66" s="3">
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.527041548831187</v>
+        <v>4.526731837581399</v>
       </c>
     </row>
     <row r="67" spans="1:2">
-      <c r="A67" s="2">
+      <c r="A67" s="3">
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.540574056713291</v>
+        <v>4.540235466570287</v>
       </c>
     </row>
     <row r="68" spans="1:2">
-      <c r="A68" s="2">
+      <c r="A68" s="3">
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.559548895549169</v>
+        <v>4.559207438324719</v>
       </c>
     </row>
     <row r="69" spans="1:2">
-      <c r="A69" s="2">
+      <c r="A69" s="3">
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.592981253815877</v>
+        <v>4.592603371347766</v>
       </c>
     </row>
     <row r="70" spans="1:2">
-      <c r="A70" s="2">
+      <c r="A70" s="3">
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.61388316017017</v>
+        <v>4.613418537829684</v>
       </c>
     </row>
     <row r="71" spans="1:2">
-      <c r="A71" s="2">
+      <c r="A71" s="3">
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.68818610392661</v>
+        <v>4.687651353339377</v>
       </c>
     </row>
     <row r="72" spans="1:2">
-      <c r="A72" s="2">
+      <c r="A72" s="3">
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.724578335585432</v>
+        <v>4.724010705871818</v>
       </c>
     </row>
     <row r="73" spans="1:2">
-      <c r="A73" s="2">
+      <c r="A73" s="3">
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.790209593871247</v>
+        <v>4.789696728461118</v>
       </c>
     </row>
     <row r="74" spans="1:2">
-      <c r="A74" s="2">
+      <c r="A74" s="3">
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.820563132025432</v>
+        <v>4.820260693813042</v>
       </c>
     </row>
     <row r="75" spans="1:2">
-      <c r="A75" s="2">
+      <c r="A75" s="3">
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.818099287940555</v>
+        <v>4.81780815537757</v>
       </c>
     </row>
     <row r="76" spans="1:2">
-      <c r="A76" s="2">
+      <c r="A76" s="3">
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.827220743788097</v>
+        <v>4.826936175632039</v>
       </c>
     </row>
     <row r="77" spans="1:2">
-      <c r="A77" s="2">
+      <c r="A77" s="3">
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.863004082324871</v>
+        <v>4.862980934367239</v>
       </c>
     </row>
     <row r="78" spans="1:2">
-      <c r="A78" s="2">
+      <c r="A78" s="3">
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855420549755292</v>
+        <v>4.855411180794171</v>
       </c>
     </row>
     <row r="79" spans="1:2">
-      <c r="A79" s="2">
+      <c r="A79" s="3">
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.849503478409142</v>
+        <v>4.849645988432313</v>
       </c>
     </row>
     <row r="80" spans="1:2">
-      <c r="A80" s="2">
+      <c r="A80" s="3">
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.827568968383533</v>
+        <v>4.827677983923074</v>
       </c>
     </row>
     <row r="81" spans="1:2">
-      <c r="A81" s="2">
+      <c r="A81" s="3">
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.834657267058294</v>
+        <v>4.834796936811963</v>
       </c>
     </row>
     <row r="82" spans="1:2">
-      <c r="A82" s="2">
+      <c r="A82" s="3">
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.88513530162171</v>
+        <v>4.885377236743606</v>
       </c>
     </row>
     <row r="83" spans="1:2">
-      <c r="A83" s="2">
+      <c r="A83" s="3">
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.913962034229817</v>
+        <v>4.914117028330264</v>
       </c>
     </row>
     <row r="84" spans="1:2">
-      <c r="A84" s="2">
+      <c r="A84" s="3">
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.923156212492233</v>
+        <v>4.923311148307091</v>
       </c>
     </row>
     <row r="85" spans="1:2">
-      <c r="A85" s="2">
+      <c r="A85" s="3">
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.913506565734128</v>
+        <v>4.913646479432967</v>
       </c>
     </row>
     <row r="86" spans="1:2">
-      <c r="A86" s="2">
+      <c r="A86" s="3">
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.895015293359723</v>
+        <v>4.895129106907923</v>
       </c>
     </row>
     <row r="87" spans="1:2">
-      <c r="A87" s="2">
+      <c r="A87" s="3">
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.891553293057239</v>
+        <v>4.891735220599092</v>
       </c>
     </row>
     <row r="88" spans="1:2">
-      <c r="A88" s="2">
+      <c r="A88" s="3">
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.890497483723625</v>
+        <v>4.890742643307174</v>
       </c>
     </row>
     <row r="89" spans="1:2">
-      <c r="A89" s="2">
+      <c r="A89" s="3">
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.88568939612832</v>
+        <v>4.886021856957042</v>
       </c>
     </row>
     <row r="90" spans="1:2">
-      <c r="A90" s="2">
+      <c r="A90" s="3">
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.869901452229282</v>
+        <v>4.870247138153029</v>
       </c>
     </row>
     <row r="91" spans="1:2">
-      <c r="A91" s="2">
+      <c r="A91" s="3">
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.856218279625262</v>
+        <v>4.848128571371246</v>
       </c>
     </row>
     <row r="92" spans="1:2">
-      <c r="A92" s="2">
+      <c r="A92" s="3">
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.842141659251742</v>
+        <v>4.833634199376265</v>
       </c>
     </row>
     <row r="93" spans="1:2">
-      <c r="A93" s="2">
+      <c r="A93" s="3">
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.834684082093801</v>
+        <v>4.8260158129659</v>
       </c>
     </row>
     <row r="94" spans="1:2">
-      <c r="A94" s="2">
+      <c r="A94" s="3">
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.81959787133412</v>
+        <v>4.810096713469547</v>
       </c>
     </row>
     <row r="95" spans="1:2">
-      <c r="A95" s="2">
+      <c r="A95" s="3">
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.811901713918993</v>
+        <v>4.802353897702086</v>
       </c>
     </row>
     <row r="96" spans="1:2">
-      <c r="A96" s="2">
+      <c r="A96" s="3">
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.814350798924933</v>
+        <v>4.803808081362613</v>
       </c>
     </row>
     <row r="97" spans="1:2">
-      <c r="A97" s="2">
+      <c r="A97" s="3">
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.846962251296889</v>
+        <v>4.832439364015295</v>
       </c>
     </row>
     <row r="98" spans="1:2">
-      <c r="A98" s="2">
+      <c r="A98" s="3">
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.84439838298695</v>
+        <v>4.829451834260833</v>
       </c>
     </row>
     <row r="99" spans="1:2">
-      <c r="A99" s="2">
+      <c r="A99" s="3">
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.836303824551635</v>
+        <v>4.821116425913023</v>
       </c>
     </row>
     <row r="100" spans="1:2">
-      <c r="A100" s="2">
+      <c r="A100" s="3">
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.831446397556591</v>
+        <v>4.811845546782495</v>
       </c>
     </row>
     <row r="101" spans="1:2">
-      <c r="A101" s="2">
+      <c r="A101" s="3">
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.804708728161224</v>
+        <v>4.779443632276982</v>
       </c>
     </row>
     <row r="102" spans="1:2">
-      <c r="A102" s="2">
+      <c r="A102" s="3">
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.774659093699023</v>
+        <v>4.748496197771869</v>
       </c>
     </row>
     <row r="103" spans="1:2">
-      <c r="A103" s="2">
+      <c r="A103" s="3">
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.763573685821337</v>
+        <v>4.740094409912256</v>
       </c>
     </row>
     <row r="104" spans="1:2">
-      <c r="A104" s="2">
+      <c r="A104" s="3">
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.724926085822213</v>
+        <v>4.704472646353857</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2">
+      <c r="A105" s="3">
+        <v>46290</v>
+      </c>
+      <c r="B105">
+        <v>4.634657603003631</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-07-12_00-43-20
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.780902456281757</v>
+        <v>4.780720584974439</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.77943280303287</v>
+        <v>4.779096804558217</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.798916590891569</v>
+        <v>4.798274186132311</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.79123338112601</v>
+        <v>4.790643329103778</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.778758165776726</v>
+        <v>4.778412481256151</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.764601625195474</v>
+        <v>4.764352324508238</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.725640888033606</v>
+        <v>4.725287250873802</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.685900761197239</v>
+        <v>4.685218270312918</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.668762504663739</v>
+        <v>4.66727905326813</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.632858724351126</v>
+        <v>4.630781162147461</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.537047856661624</v>
+        <v>4.534229488596599</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.470461025928509</v>
+        <v>4.466869947788049</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.51615726878082</v>
+        <v>4.509075844568263</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-07-13_22-21-09
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712912172845796</v>
+        <v>4.712908681410944</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711308922788138</v>
+        <v>4.71132536264577</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.719745117993728</v>
+        <v>4.71976500212315</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706025005980357</v>
+        <v>4.706066290621247</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.693361397677753</v>
+        <v>4.693403148952573</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.677428270595517</v>
+        <v>4.677470385521219</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.672435255915507</v>
+        <v>4.672477454891506</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.685512116008697</v>
+        <v>4.685554252667615</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.701275758276909</v>
+        <v>4.701326031557327</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.704859960455395</v>
+        <v>4.704893259787783</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.693915838846345</v>
+        <v>4.693949824270279</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.663880993608783</v>
+        <v>4.663917871864814</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649536307979685</v>
+        <v>4.649540430043005</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641082534070489</v>
+        <v>4.641095105971205</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636023412253071</v>
+        <v>4.636032058179322</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633519256434933</v>
+        <v>4.63353927844817</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637281302883382</v>
+        <v>4.637285136362618</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634707577781986</v>
+        <v>4.634695903046492</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.628377567195014</v>
+        <v>4.628344021033556</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.624693610180743</v>
+        <v>4.624657488988234</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.600042955791277</v>
+        <v>4.600007181470096</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.581415285043986</v>
+        <v>4.581335292726299</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.563799908683828</v>
+        <v>4.563669189879715</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.527202890278234</v>
+        <v>4.527011750601559</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.526153821486996</v>
+        <v>4.525883722328651</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.539603036399619</v>
+        <v>4.539307280736523</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.558569194038787</v>
+        <v>4.558270516408001</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.59189638953605</v>
+        <v>4.591565255574914</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.612547619830808</v>
+        <v>4.612138949815491</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.686649159397708</v>
+        <v>4.686178969355272</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.722946951847498</v>
+        <v>4.722447906844106</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.788733269163572</v>
+        <v>4.788280225516639</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.819692690000465</v>
+        <v>4.819425668434547</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.817260801038338</v>
+        <v>4.817003226107664</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.826400407227006</v>
+        <v>4.826147947124893</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862936696409857</v>
+        <v>4.862915557900345</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855392691433492</v>
+        <v>4.85538359907194</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.849913020094846</v>
+        <v>4.850038281108977</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.827881483411838</v>
+        <v>4.82797659640414</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.8350581195125</v>
+        <v>4.835180398297302</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.885830192253717</v>
+        <v>4.886042498486273</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.91440616703414</v>
+        <v>4.914541216492299</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.923600461582738</v>
+        <v>4.923735717700073</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.913908862414893</v>
+        <v>4.914032032197577</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.895342426395698</v>
+        <v>4.895442510052929</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.892077015218662</v>
+        <v>4.892237744934048</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.891204327809811</v>
+        <v>4.891421927859569</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.886647143529373</v>
+        <v>4.886941494367809</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.870896807926135</v>
+        <v>4.871202421885997</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.84868929442613</v>
+        <v>4.848952647672984</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.822605332421769</v>
+        <v>4.822867383656964</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.813614052892564</v>
+        <v>4.813866762294577</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.790798880157428</v>
+        <v>4.784684203900639</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.780720584974439</v>
+        <v>4.774404655681424</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.779096804558217</v>
+        <v>4.772376959306277</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.798274186132311</v>
+        <v>4.78804016265314</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.790643329103778</v>
+        <v>4.779153264910379</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.778412481256151</v>
+        <v>4.765875919201253</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.764352324508238</v>
+        <v>4.750570198926126</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.725287250873802</v>
+        <v>4.711763410236061</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.685218270312918</v>
+        <v>4.67316976474647</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.66727905326813</v>
+        <v>4.652208835447007</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.630781162147461</v>
+        <v>4.617231429181576</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.534229488596599</v>
+        <v>4.534340387392296</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.466869947788049</v>
+        <v>4.487083718702337</v>
       </c>
     </row>
     <row r="107" spans="1:2">

</xml_diff>

<commit_message>
Update forecast data 2026-07-15_21-56-22
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712905335388052</v>
+        <v>4.712902125879445</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711341111117843</v>
+        <v>4.711356210905327</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.719784060920841</v>
+        <v>4.719802344695539</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706105853567463</v>
+        <v>4.706143800242978</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.693443159176696</v>
+        <v>4.693481534954861</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.677510744184898</v>
+        <v>4.677549454126655</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.672517895052795</v>
+        <v>4.672556684038158</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.685594635667342</v>
+        <v>4.685633372175958</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.701374230929527</v>
+        <v>4.701420481983548</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.704925188445923</v>
+        <v>4.704955829289053</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.693982409294724</v>
+        <v>4.694013678666034</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.663953227556508</v>
+        <v>4.663987153002334</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649544452019651</v>
+        <v>4.64954837571407</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.64110721192585</v>
+        <v>4.641118877022904</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636040346207889</v>
+        <v>4.636048298116582</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633558484897835</v>
+        <v>4.633576924516681</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637288860515779</v>
+        <v>4.637292478975239</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634684724739994</v>
+        <v>4.634674011992003</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.628311843100439</v>
+        <v>4.6282809515367</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.624622853465848</v>
+        <v>4.624589613896088</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599972884876459</v>
+        <v>4.599939976500838</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.581258741347987</v>
+        <v>4.581185414282911</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.563544146385769</v>
+        <v>4.563424418220181</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.526828821236427</v>
+        <v>4.526653586980355</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.525625159038269</v>
+        <v>4.52537741201923</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.539024020536774</v>
+        <v>4.538752485265856</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.55798433762993</v>
+        <v>4.557709895102406</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.591247807020997</v>
+        <v>4.590943220228755</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.611746712988412</v>
+        <v>4.611369943724022</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.685727734594465</v>
+        <v>4.685294338642026</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.721968996219275</v>
+        <v>4.721509033029266</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.787844828820253</v>
+        <v>4.787426075325317</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.819169089546858</v>
+        <v>4.818922357191672</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.816755568625736</v>
+        <v>4.816517272168455</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.825905006311874</v>
+        <v>4.825671063522229</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862895041488979</v>
+        <v>4.862875124259611</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855374622519303</v>
+        <v>4.855365769767271</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.850158482316681</v>
+        <v>4.85027392351595</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.828067660004599</v>
+        <v>4.828154926457211</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.835297593487883</v>
+        <v>4.835410014064907</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.886246127181933</v>
+        <v>4.886441598417932</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.914670459144492</v>
+        <v>4.914794258077324</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.923865232010378</v>
+        <v>4.923989358454199</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.914150275896115</v>
+        <v>4.914263879654666</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.895538557332801</v>
+        <v>4.895630804055592</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.89239221698438</v>
+        <v>4.89254078561467</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.891631351776274</v>
+        <v>4.891833045047475</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.887224572307427</v>
+        <v>4.887497005571668</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.871496205365197</v>
+        <v>4.871778827104556</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.849205556748047</v>
+        <v>4.84944862806783</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.823118635601579</v>
+        <v>4.823359739648438</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.814108948651548</v>
+        <v>4.814341253486619</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.784895458505821</v>
+        <v>4.785097804876073</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.76791353218248</v>
+        <v>4.764667177664489</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.765081638906254</v>
+        <v>4.761588492352002</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.778674797559108</v>
+        <v>4.773568902051485</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.768158089506189</v>
+        <v>4.762271584387663</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.753731719295546</v>
+        <v>4.747450090701697</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.736945325553085</v>
+        <v>4.730174258478766</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.697540758913304</v>
+        <v>4.691702811199232</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.659288650623663</v>
+        <v>4.654906936048162</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.637696142728845</v>
+        <v>4.633359327194803</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.59860526144624</v>
+        <v>4.592805289833292</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.517316568435866</v>
+        <v>4.522151372846405</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.472307034141659</v>
+        <v>4.483934599720854</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.477147878040563</v>
+        <v>4.485770267966878</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.416255241791472</v>
+        <v>4.462332812585707</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-07-16_23-03-18
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712902125879445</v>
+        <v>4.712899044698776</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711356210905327</v>
+        <v>4.711370701264952</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.719802344695539</v>
+        <v>4.719819899751073</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706143800242978</v>
+        <v>4.70618022764256</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.693481534954861</v>
+        <v>4.693518374368409</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.677549454126655</v>
+        <v>4.677586614288017</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.672556684038158</v>
+        <v>4.672593920884462</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.685633372175958</v>
+        <v>4.685670560809555</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.701420481983548</v>
+        <v>4.701464900380987</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.704955829289053</v>
+        <v>4.704985258634668</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694013678666034</v>
+        <v>4.694043710432673</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.663987153002334</v>
+        <v>4.664019733210236</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.64954837571407</v>
+        <v>4.649552203126782</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641118877022904</v>
+        <v>4.64113012461028</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636048298116582</v>
+        <v>4.636055933950985</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633576924516681</v>
+        <v>4.633594642238855</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637292478975239</v>
+        <v>4.637295995325175</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634674011992003</v>
+        <v>4.634663736429593</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.6282809515367</v>
+        <v>4.628251270871925</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.624589613896088</v>
+        <v>4.624557687635328</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599939976500838</v>
+        <v>4.599908373904268</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.581185414282911</v>
+        <v>4.581115112660756</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.563424418220181</v>
+        <v>4.563309675085558</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.526653586980355</v>
+        <v>4.526485574654517</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.52537741201923</v>
+        <v>4.525139820008484</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.538752485265856</v>
+        <v>4.538491966093364</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.557709895102406</v>
+        <v>4.557446486580973</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.590943220228755</v>
+        <v>4.590650735767269</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.611369943724022</v>
+        <v>4.61100775012508</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.685294338642026</v>
+        <v>4.684877750465739</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.721509033029266</v>
+        <v>4.721066921250363</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.787426075325317</v>
+        <v>4.787023035390719</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.818922357191672</v>
+        <v>4.818684919382119</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.816517272168455</v>
+        <v>4.816287820733637</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.825671063522229</v>
+        <v>4.825445634290064</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862875124259611</v>
+        <v>4.862855783972241</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855365769767271</v>
+        <v>4.855357047045581</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.85027392351595</v>
+        <v>4.850384881331039</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.828154926457211</v>
+        <v>4.828238627554509</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.835410014064907</v>
+        <v>4.83551794458751</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.886441598417932</v>
+        <v>4.886629391625982</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.914794258077324</v>
+        <v>4.914912946988572</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.923989358454199</v>
+        <v>4.924108422774179</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.914263879654666</v>
+        <v>4.914373108164813</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.895630804055592</v>
+        <v>4.895719468297742</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.89254078561467</v>
+        <v>4.892683779160357</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.891833045047475</v>
+        <v>4.892027421922753</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.887497005571668</v>
+        <v>4.887759377112829</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.871778827104556</v>
+        <v>4.872050906762558</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.84944862806783</v>
+        <v>4.849682422202241</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.823359739648438</v>
+        <v>4.823591296045935</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.814341253486619</v>
+        <v>4.81456426740325</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.785097804876073</v>
+        <v>4.785291789173648</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.764667177664489</v>
+        <v>4.763150835988638</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.761588492352002</v>
+        <v>4.760143391453141</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.773568902051485</v>
+        <v>4.770826631353138</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.762271584387663</v>
+        <v>4.759243309089582</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.747450090701697</v>
+        <v>4.744385658662415</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.730174258478766</v>
+        <v>4.72707447467026</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.691702811199232</v>
+        <v>4.690084697328462</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.654906936048162</v>
+        <v>4.654958940776637</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.633359327194803</v>
+        <v>4.633709945093886</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.592805289833292</v>
+        <v>4.592750893888013</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.522151372846405</v>
+        <v>4.532020637846527</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.483934599720854</v>
+        <v>4.499302804707686</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.485770267966878</v>
+        <v>4.500559539153183</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.462332812585707</v>
+        <v>4.4942764749632</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-07-18_09-20-18
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712899044698776</v>
+        <v>4.712893237722385</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711370701264952</v>
+        <v>4.7113979955085</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.719819899751073</v>
+        <v>4.719852991193687</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.70618022764256</v>
+        <v>4.706248875304293</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.693518374368409</v>
+        <v>4.693587798721554</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.677586614288017</v>
+        <v>4.677656642997829</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.672593920884462</v>
+        <v>4.672664096252285</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.685670560809555</v>
+        <v>4.685740651074918</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.701464900380987</v>
+        <v>4.701548657866955</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.704985258634668</v>
+        <v>4.705040759118416</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694043710432673</v>
+        <v>4.69410034367301</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664019733210236</v>
+        <v>4.664081165565158</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649552203126782</v>
+        <v>4.649559577786971</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.64113012461028</v>
+        <v>4.641151452803082</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636055933950985</v>
+        <v>4.636070329912254</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633594642238855</v>
+        <v>4.633628074869641</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637295995325175</v>
+        <v>4.637302735684574</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634663736429593</v>
+        <v>4.634644394406292</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.628251270871925</v>
+        <v>4.628195268708923</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.624557687635328</v>
+        <v>4.624497475815298</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599908373904268</v>
+        <v>4.599848787623841</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.581115112660756</v>
+        <v>4.580982868585887</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.563309675085558</v>
+        <v>4.563093953576724</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.526485574654517</v>
+        <v>4.526169508598814</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.525139820008484</v>
+        <v>4.524692713698182</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.538491966093364</v>
+        <v>4.538001413806013</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.557446486580973</v>
+        <v>4.556950230137796</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.590650735767269</v>
+        <v>4.590099321357124</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.61100775012508</v>
+        <v>4.610323850566733</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.684877750465739</v>
+        <v>4.684091253583888</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.721066921250363</v>
+        <v>4.720232272436041</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.787023035390719</v>
+        <v>4.786260708932006</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.818684919382119</v>
+        <v>4.818235916794625</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.816287820733637</v>
+        <v>4.815853570023946</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.825445634290064</v>
+        <v>4.825018544139401</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862855783972241</v>
+        <v>4.862818748875913</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855357047045581</v>
+        <v>4.855340009406671</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.850384881331039</v>
+        <v>4.850594350345443</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.828238627554509</v>
+        <v>4.828396170509684</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.83551794458751</v>
+        <v>4.835721365460333</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.886629391625982</v>
+        <v>4.886983681330777</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.914912946988572</v>
+        <v>4.915136199602558</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.924108422774179</v>
+        <v>4.924332543064399</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.914373108164813</v>
+        <v>4.914579402406783</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.895719468297742</v>
+        <v>4.895886842425352</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.892683779160357</v>
+        <v>4.892954238317919</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.892027421922753</v>
+        <v>4.892395742855122</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.887759377112829</v>
+        <v>4.888256063793055</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.872050906762558</v>
+        <v>4.872565698914994</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.849682422202241</v>
+        <v>4.85012421690219</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.823591296045935</v>
+        <v>4.824027940029593</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.81456426740325</v>
+        <v>4.814984559348351</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.785291789173648</v>
+        <v>4.785656643701712</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.763150835988638</v>
+        <v>4.759646623976749</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.760143391453141</v>
+        <v>4.75662039519318</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.770826631353138</v>
+        <v>4.765175177694097</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.759243309089582</v>
+        <v>4.753194387343811</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.744385658662415</v>
+        <v>4.738388670549787</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.72707447467026</v>
+        <v>4.721198382250559</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.690084697328462</v>
+        <v>4.686707903257384</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.654958940776637</v>
+        <v>4.654064398985609</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.633709945093886</v>
+        <v>4.633224033025047</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.592750893888013</v>
+        <v>4.594263463239865</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.532020637846527</v>
+        <v>4.547194745896072</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.499302804707686</v>
+        <v>4.521431212305224</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.500559539153183</v>
+        <v>4.522863698746618</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.4942764749632</v>
+        <v>4.526431746083624</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-07-20_21-22-46
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712893237722385</v>
+        <v>4.712890498522531</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.7113979955085</v>
+        <v>4.711410863554769</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.719852991193687</v>
+        <v>4.719868603460388</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706248875304293</v>
+        <v>4.706281254375715</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.693587798721554</v>
+        <v>4.693620544250357</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.677656642997829</v>
+        <v>4.677689673542413</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.672664096252285</v>
+        <v>4.672697196943236</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.685740651074918</v>
+        <v>4.685773714233485</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.701548657866955</v>
+        <v>4.701588186752878</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705040759118416</v>
+        <v>4.705066955525968</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.69410034367301</v>
+        <v>4.694127073230358</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664081165565158</v>
+        <v>4.664110157163393</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649559577786971</v>
+        <v>4.649563129594317</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641151452803082</v>
+        <v>4.641161572641538</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636070329912254</v>
+        <v>4.636077122894998</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633628074869641</v>
+        <v>4.633643863716007</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637302735684574</v>
+        <v>4.637305966475858</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634644394406292</v>
+        <v>4.634635281606584</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.628195268708923</v>
+        <v>4.628168823056175</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.624497475815298</v>
+        <v>4.624469054568955</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599848787623841</v>
+        <v>4.599820668644121</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.580982868585887</v>
+        <v>4.580920602188796</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.563093953576724</v>
+        <v>4.562992437867369</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.526169508598814</v>
+        <v>4.52602068337421</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.524692713698182</v>
+        <v>4.52448211989531</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.538001413806013</v>
+        <v>4.537770220713425</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.556950230137796</v>
+        <v>4.556716230379438</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.590099321357124</v>
+        <v>4.589839142146158</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.610323850566733</v>
+        <v>4.610000671361026</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.684091253583888</v>
+        <v>4.683719642552467</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.720232272436041</v>
+        <v>4.71983792609015</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.786260708932006</v>
+        <v>4.785899877157724</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.818235916794625</v>
+        <v>4.818023435073425</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.815853570023946</v>
+        <v>4.815647910577852</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.825018544139401</v>
+        <v>4.824816071591108</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862818748875913</v>
+        <v>4.862801013261066</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855340009406671</v>
+        <v>4.855331700403942</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.850594350345443</v>
+        <v>4.85069331746523</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.828396170509684</v>
+        <v>4.828470390773997</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.835721365460333</v>
+        <v>4.835817322717318</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.886983681330777</v>
+        <v>4.887150966302793</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.915136199602558</v>
+        <v>4.91524130815251</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.924332543064399</v>
+        <v>4.924438132557164</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.914579402406783</v>
+        <v>4.914676906763006</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.895886842425352</v>
+        <v>4.895965913419749</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.892954238317919</v>
+        <v>4.893082250544568</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.892395742855122</v>
+        <v>4.892570381694746</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.888256063793055</v>
+        <v>4.888491352094119</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.872565698914994</v>
+        <v>4.872809442552883</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.85012421690219</v>
+        <v>4.85033314523744</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.824027940029593</v>
+        <v>4.82423401383018</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.814984559348351</v>
+        <v>4.81518280567199</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.785656643701712</v>
+        <v>4.785828405817757</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.759646623976749</v>
+        <v>4.757926460488424</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.75662039519318</v>
+        <v>4.754895245492457</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.765175177694097</v>
+        <v>4.7626150986495</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.753194387343811</v>
+        <v>4.750577240366565</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.738388670549787</v>
+        <v>4.735931902184968</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.721198382250559</v>
+        <v>4.718945359649083</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.686707903257384</v>
+        <v>4.685594787567331</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.654064398985609</v>
+        <v>4.653929517861448</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.633224033025047</v>
+        <v>4.63474762742262</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.594263463239865</v>
+        <v>4.597683610919034</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.547194745896072</v>
+        <v>4.555580346615898</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.521431212305224</v>
+        <v>4.53313009024632</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.522863698746618</v>
+        <v>4.53427215062605</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.526431746083624</v>
+        <v>4.539399250457492</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-07-22_20-32-54
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712887860739071</v>
+        <v>4.71288531884271</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711423251000947</v>
+        <v>4.711435184270187</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.71988363934687</v>
+        <v>4.71989813017734</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.70631243301346</v>
+        <v>4.70634247672298</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.693652075830333</v>
+        <v>4.693682459701505</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.677721479547203</v>
+        <v>4.677752127832028</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.672729071082365</v>
+        <v>4.672759785567523</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.685805553810535</v>
+        <v>4.685836236456463</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.701626264006999</v>
+        <v>4.701662968077662</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705092191916362</v>
+        <v>4.705116520080892</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694152822315034</v>
+        <v>4.694177643871569</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664138083480488</v>
+        <v>4.664165002139493</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649566594177499</v>
+        <v>4.649569973906694</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641171353663102</v>
+        <v>4.641180812435554</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.6360836657659</v>
+        <v>4.636089972091352</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633659079082808</v>
+        <v>4.633673751606725</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637309108704193</v>
+        <v>4.637312165514565</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634626512949802</v>
+        <v>4.63461806936904</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.628143339081711</v>
+        <v>4.628118765352534</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.624441674240424</v>
+        <v>4.624415278719162</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599793583834349</v>
+        <v>4.599767477269546</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.580860710726879</v>
+        <v>4.580803061225012</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.562894828124604</v>
+        <v>4.562800904053907</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.525877530916226</v>
+        <v>4.525739734284301</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.524279513560879</v>
+        <v>4.52408445071559</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.537547714815914</v>
+        <v>4.537333417980506</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.556490952276192</v>
+        <v>4.556273920068978</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.589588557611386</v>
+        <v>4.589347050396333</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.609689110985519</v>
+        <v>4.609388556914707</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.683361422640666</v>
+        <v>4.68301588636708</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.719457799750719</v>
+        <v>4.719091141594898</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.785551658298929</v>
+        <v>4.785215406178176</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.817818407953318</v>
+        <v>4.817620452222935</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.815449370349619</v>
+        <v>4.815257588714649</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.82462048448226</v>
+        <v>4.824431441017548</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862783772990444</v>
+        <v>4.862767009545382</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855323533623672</v>
+        <v>4.855315509850443</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.850788716326772</v>
+        <v>4.85088073613069</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.828541805489742</v>
+        <v>4.828610570301682</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.835909727244756</v>
+        <v>4.835998771978781</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.887312156002274</v>
+        <v>4.887467576976432</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.91534240066334</v>
+        <v>4.915439701217307</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.924539731037656</v>
+        <v>4.924637558547843</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.914770916080651</v>
+        <v>4.914861613214932</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.896042126604644</v>
+        <v>4.896115632404913</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.893205784430883</v>
+        <v>4.893325068844932</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.892739097803132</v>
+        <v>4.892902184058113</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.888718531074002</v>
+        <v>4.888938009251281</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.873044713087951</v>
+        <v>4.873271942168349</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.850534658319495</v>
+        <v>4.850729142617418</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.824432519732734</v>
+        <v>4.824623865783233</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.815373705013702</v>
+        <v>4.815557657219234</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.78599359663563</v>
+        <v>4.786152583000264</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.758086192901374</v>
+        <v>4.758240248450195</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.753663165216723</v>
+        <v>4.752691031987946</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.761295420592845</v>
+        <v>4.760269527252253</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.750140098040262</v>
+        <v>4.749911000504015</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.73674147220658</v>
+        <v>4.737638245360291</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.720831320286114</v>
+        <v>4.722687307434812</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.689356796373692</v>
+        <v>4.692849974054674</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.659449621054426</v>
+        <v>4.66446032001519</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.640708722282009</v>
+        <v>4.646104874560559</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.607644779772798</v>
+        <v>4.616438001173928</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.572314503265435</v>
+        <v>4.586503626511978</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.553329675295439</v>
+        <v>4.570131272731785</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.555077241024208</v>
+        <v>4.572039971454267</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.565051297814213</v>
+        <v>4.584745097874954</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.637373797814213</v>
+        <v>4.657067597874955</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-07-22_21-04-02
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.760269527252253</v>
+        <v>4.760258866843434</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.749911000504015</v>
+        <v>4.749866379575897</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.737638245360291</v>
+        <v>4.737512202898452</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.722687307434812</v>
+        <v>4.722527932025841</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.692849974054674</v>
+        <v>4.692692001379474</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.66446032001519</v>
+        <v>4.664262901108789</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.646104874560559</v>
+        <v>4.645920802247574</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.616438001173928</v>
+        <v>4.615014389302952</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.586503626511978</v>
+        <v>4.584317014135104</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.570131272731785</v>
+        <v>4.568093335488837</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.572039971454267</v>
+        <v>4.570946417989271</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.584745097874954</v>
+        <v>4.583670048114737</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.657067597874955</v>
+        <v>4.655992548114737</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-07-22_21-14-40
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.760258866843434</v>
+        <v>4.760266710170427</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.749866379575897</v>
+        <v>4.749919344275795</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.737512202898452</v>
+        <v>4.737668712004035</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.722527932025841</v>
+        <v>4.722739698972183</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.692692001379474</v>
+        <v>4.692929022660781</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.664262901108789</v>
+        <v>4.664454248737862</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.645920802247574</v>
+        <v>4.647179862737185</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.615014389302952</v>
+        <v>4.615961592476562</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.584317014135104</v>
+        <v>4.586952865014342</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.568093335488837</v>
+        <v>4.567851818301429</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.570946417989271</v>
+        <v>4.571527682818459</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.583670048114737</v>
+        <v>4.584185754597859</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.655992548114737</v>
+        <v>4.656508254597858</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-07-23_20-34-45
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.71288531884271</v>
+        <v>4.712882867698884</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711435184270187</v>
+        <v>4.711446687884047</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.71989813017734</v>
+        <v>4.719912105047674</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.70634247672298</v>
+        <v>4.70637144633143</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.693682459701505</v>
+        <v>4.693711757373286</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.677752127832028</v>
+        <v>4.677781680444524</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.672759785567523</v>
+        <v>4.672789402521047</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.685836236456463</v>
+        <v>4.685865824069866</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.701662968077662</v>
+        <v>4.701698371865667</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705116520080892</v>
+        <v>4.705139988153459</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694177643871569</v>
+        <v>4.694201587102131</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664165002139493</v>
+        <v>4.664190966683402</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649569973906694</v>
+        <v>4.649573271151038</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641180812435554</v>
+        <v>4.641189964476254</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636089972091352</v>
+        <v>4.63609605447382</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633673751606725</v>
+        <v>4.633687909783951</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637312165514565</v>
+        <v>4.637315139946786</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.63461806936904</v>
+        <v>4.634609933175885</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.628118765352534</v>
+        <v>4.628095054033042</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.624415278719162</v>
+        <v>4.62438981585303</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599767477269546</v>
+        <v>4.599742296978886</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.580803061225012</v>
+        <v>4.580747530429271</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.562800904053907</v>
+        <v>4.562710461562666</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.525739734284301</v>
+        <v>4.525606999627183</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.52408445071559</v>
+        <v>4.523896519552678</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.537333417980506</v>
+        <v>4.537126886362903</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.556273920068978</v>
+        <v>4.556064691785061</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.589347050396333</v>
+        <v>4.589114139424979</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.609388556914707</v>
+        <v>4.609098438725749</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.68301588636708</v>
+        <v>4.682682374979591</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.719091141594898</v>
+        <v>4.71873725162436</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.785215406178176</v>
+        <v>4.784890517750099</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.817620452222935</v>
+        <v>4.817429210330251</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.815257588714649</v>
+        <v>4.815072228806001</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.824431441017548</v>
+        <v>4.824248621400974</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862767009545382</v>
+        <v>4.862750705146458</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855315509850443</v>
+        <v>4.855307629238407</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.85088073613069</v>
+        <v>4.850969552957782</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.828610570301682</v>
+        <v>4.828676829583033</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.835998771978781</v>
+        <v>4.836084636187438</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.887467576976432</v>
+        <v>4.887617532900066</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.915439701217307</v>
+        <v>4.915533417648584</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.924637558547843</v>
+        <v>4.924731819382892</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.914861613214932</v>
+        <v>4.914949168609684</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.896115632404913</v>
+        <v>4.896186570992368</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.893325068844932</v>
+        <v>4.893440317468561</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.892902184058113</v>
+        <v>4.893059914583263</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.888938009251281</v>
+        <v>4.889150168409252</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.873271942168349</v>
+        <v>4.873491532789805</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.850729142617418</v>
+        <v>4.850916958298177</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.824623865783233</v>
+        <v>4.824808431303663</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.815557657219234</v>
+        <v>4.815735033718402</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.786152583000264</v>
+        <v>4.786305705164521</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.758240248450195</v>
+        <v>4.758388918640607</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.752691031987946</v>
+        <v>4.752035458781704</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.760266710170427</v>
+        <v>4.759624603746708</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.749919344275795</v>
+        <v>4.7500584192235</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.737668712004035</v>
+        <v>4.738977603243756</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.722739698972183</v>
+        <v>4.724997719050112</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.692929022660781</v>
+        <v>4.696698577081625</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.664454248737862</v>
+        <v>4.669547359883472</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.647179862737185</v>
+        <v>4.653574633648796</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.615961592476562</v>
+        <v>4.625134511059239</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.586952865014342</v>
+        <v>4.602153319588631</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.567851818301429</v>
+        <v>4.582704975328674</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.571527682818459</v>
+        <v>4.586969313150279</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.584185754597859</v>
+        <v>4.601279916605479</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.656508254597858</v>
+        <v>4.715488408700498</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-07-24_20-32-43
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712882867698884</v>
+        <v>4.712880502533157</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711446687884047</v>
+        <v>4.7114577846305</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.719912105047674</v>
+        <v>4.71992559102001</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.70637144633143</v>
+        <v>4.706399398397775</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.693711757373286</v>
+        <v>4.693740026039158</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.677781680444524</v>
+        <v>4.677810195078487</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.672789402521047</v>
+        <v>4.672817979708194</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.685865824069866</v>
+        <v>4.685894374213381</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.701698371865667</v>
+        <v>4.701732543205689</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705139988153459</v>
+        <v>4.705162640927611</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694201587102131</v>
+        <v>4.694224697791245</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664190966683402</v>
+        <v>4.664216026929784</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649573271151038</v>
+        <v>4.64957648826417</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641189964476254</v>
+        <v>4.641198824332945</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.63609605447382</v>
+        <v>4.636101924635991</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633687909783951</v>
+        <v>4.633701580153602</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637315139946786</v>
+        <v>4.637318034934326</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634609933175885</v>
+        <v>4.634602087938418</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.628095054033042</v>
+        <v>4.628072160576441</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.62438981585303</v>
+        <v>4.624365237105558</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599742296978886</v>
+        <v>4.59971799460288</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.580747530429271</v>
+        <v>4.580694003936553</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.562710461562666</v>
+        <v>4.562623311302367</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.525606999627183</v>
+        <v>4.525479054125304</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.523896519552678</v>
+        <v>4.523715337586618</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.537126886362903</v>
+        <v>4.536927707401824</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.556064691785061</v>
+        <v>4.555862856307828</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.589114139424979</v>
+        <v>4.588889376798138</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.609098438725749</v>
+        <v>4.608818224560153</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.682682374979591</v>
+        <v>4.682360274351911</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.71873725162436</v>
+        <v>4.718395477297427</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.784890517750099</v>
+        <v>4.784576429584726</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.817429210330251</v>
+        <v>4.817244348284564</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.815072228806001</v>
+        <v>4.814892975606661</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.824248621400974</v>
+        <v>4.824071726116512</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862750705146458</v>
+        <v>4.86273484273766</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855307629238407</v>
+        <v>4.855299891413777</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.850969552957782</v>
+        <v>4.851055330884932</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.828676829583033</v>
+        <v>4.82874071743495</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.836084636187438</v>
+        <v>4.836167486655427</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.887617532900066</v>
+        <v>4.887762306539834</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.915533417648584</v>
+        <v>4.915623742979942</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.924731819382892</v>
+        <v>4.924822703463562</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.914949168609684</v>
+        <v>4.915033741321682</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.896186570992368</v>
+        <v>4.896255073134146</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.893440317468561</v>
+        <v>4.893551730023509</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.893059914583263</v>
+        <v>4.893212546203836</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.889150168409252</v>
+        <v>4.889355365726278</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.873491532789805</v>
+        <v>4.873703861619429</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.850916958298177</v>
+        <v>4.851098441418888</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.824808431303663</v>
+        <v>4.824986569367828</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.815735033718402</v>
+        <v>4.815906179998192</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.786305705164521</v>
+        <v>4.786453279137904</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.758388918640607</v>
+        <v>4.75853247575195</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.752035458781704</v>
+        <v>4.750382894740027</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.759624603746708</v>
+        <v>4.757766230778037</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.7500584192235</v>
+        <v>4.748871292675927</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.738977603243756</v>
+        <v>4.738711819310918</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.724997719050112</v>
+        <v>4.725468869228528</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.696698577081625</v>
+        <v>4.698282254775902</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.669547359883472</v>
+        <v>4.673013524800848</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.653574633648796</v>
+        <v>4.656791529233249</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.625134511059239</v>
+        <v>4.63164866164118</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.602153319588631</v>
+        <v>4.609485370544884</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.582704975328674</v>
+        <v>4.593846633318837</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.586969313150279</v>
+        <v>4.596453487436133</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.601279916605479</v>
+        <v>4.610690451555763</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.715488408700498</v>
+        <v>4.708333342990495</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-07-24_20-35-36
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.757766230778037</v>
+        <v>4.757763765826175</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.748871292675927</v>
+        <v>4.748878485123382</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.738711819310918</v>
+        <v>4.738738026920918</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.725468869228528</v>
+        <v>4.725513816312077</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.698282254775902</v>
+        <v>4.698349504020168</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.673013524800848</v>
+        <v>4.673008162992652</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.656791529233249</v>
+        <v>4.657702856324372</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.63164866164118</v>
+        <v>4.631245844529635</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.609485370544884</v>
+        <v>4.609851485573172</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.593846633318837</v>
+        <v>4.591997799271975</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.596453487436133</v>
+        <v>4.596043312909737</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.610690451555763</v>
+        <v>4.610259966500948</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.708333342990495</v>
+        <v>4.707445923746352</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-07-25_09-21-00
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712880502533157</v>
+        <v>4.712878218900197</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.7114577846305</v>
+        <v>4.711468495714417</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.71992559102001</v>
+        <v>4.719938613297313</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706399398397775</v>
+        <v>4.706426385580516</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.693740026039158</v>
+        <v>4.693767318948504</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.677810195078487</v>
+        <v>4.67783772544897</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.672817979708194</v>
+        <v>4.672845570912368</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.685894374213381</v>
+        <v>4.685921940486619</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.701732543205689</v>
+        <v>4.701765545298469</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705162640927611</v>
+        <v>4.705184520141215</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694224697791245</v>
+        <v>4.694247018597318</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664216026929784</v>
+        <v>4.664240229289093</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.64957648826417</v>
+        <v>4.64957962757275</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641198824332945</v>
+        <v>4.641207405657332</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636101924635991</v>
+        <v>4.636107593496235</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633701580153602</v>
+        <v>4.633714787462631</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637318034934326</v>
+        <v>4.637320853304352</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634602087938418</v>
+        <v>4.634594518371909</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.628072160576441</v>
+        <v>4.628050043447324</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.624365237105558</v>
+        <v>4.624341497248192</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.59971799460288</v>
+        <v>4.599694525085565</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.580694003936553</v>
+        <v>4.580642375415843</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.562623311302367</v>
+        <v>4.562539277364912</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.525479054125304</v>
+        <v>4.525355644148628</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.523715337586618</v>
+        <v>4.523540549098687</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.536927707401824</v>
+        <v>4.536735497122693</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.555862856307828</v>
+        <v>4.555668030744667</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.588889376798138</v>
+        <v>4.58867234500087</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.608818224560153</v>
+        <v>4.608547417934535</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.682360274351911</v>
+        <v>4.682049011285836</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.718395477297427</v>
+        <v>4.718065209593451</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.784576429584726</v>
+        <v>4.784272614686989</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.817244348284564</v>
+        <v>4.81706555375955</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.814892975606661</v>
+        <v>4.81471953422098</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.824071726116512</v>
+        <v>4.823900474365166</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.86273484273766</v>
+        <v>4.862719405967363</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855299891413777</v>
+        <v>4.85529229556216</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.851055330884932</v>
+        <v>4.851138222989204</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.82874071743495</v>
+        <v>4.82880235858179</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.836167486655427</v>
+        <v>4.836247478748165</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.887762306539834</v>
+        <v>4.887902161519925</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.915623742979942</v>
+        <v>4.915710856710577</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.924822703463562</v>
+        <v>4.924910387568636</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.915033741321682</v>
+        <v>4.915115479946335</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.896255073134146</v>
+        <v>4.896321260959314</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.893551730023509</v>
+        <v>4.893659493381961</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.893212546203836</v>
+        <v>4.893360319771435</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.889355365726278</v>
+        <v>4.889553935707834</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.873703861619429</v>
+        <v>4.873909281098458</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.851098441418888</v>
+        <v>4.851273905904188</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.824986569367828</v>
+        <v>4.825158609026223</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.815906179998192</v>
+        <v>4.816071417822718</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.786453279137904</v>
+        <v>4.78659559879244</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.75853247575195</v>
+        <v>4.758671174362827</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.750382894740027</v>
+        <v>4.749104252397999</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.757763765826175</v>
+        <v>4.756317563600136</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.748878485123382</v>
+        <v>4.748054558068775</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.738738026920918</v>
+        <v>4.738740995617157</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.725513816312077</v>
+        <v>4.726052620662148</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.698349504020168</v>
+        <v>4.700170757181908</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.673008162992652</v>
+        <v>4.676101711183619</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.657702856324372</v>
+        <v>4.661126158927494</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.631245844529635</v>
+        <v>4.636141540874346</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.609851485573172</v>
+        <v>4.615341640072916</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.591997799271975</v>
+        <v>4.598234550992457</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.596043312909737</v>
+        <v>4.60127679494878</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.610259966500948</v>
+        <v>4.61403163923668</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.707445923746352</v>
+        <v>4.693845530796164</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-07-28_20-50-29
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712873879932303</v>
+        <v>4.712878218900197</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711488838595651</v>
+        <v>4.711468495714417</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.71996335920851</v>
+        <v>4.719938613297313</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706477658376062</v>
+        <v>4.706426385580516</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.693819172745645</v>
+        <v>4.693767318948504</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.677890030354432</v>
+        <v>4.67783772544897</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.672897992585171</v>
+        <v>4.672845570912368</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.685974317982873</v>
+        <v>4.685921940486619</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.701828273669522</v>
+        <v>4.701765545298469</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705226111070846</v>
+        <v>4.705184520141215</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694289447110599</v>
+        <v>4.694247018597318</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664286230641764</v>
+        <v>4.664240229289093</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649585681895855</v>
+        <v>4.64957962757275</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641223783232535</v>
+        <v>4.641207405657332</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636118367363091</v>
+        <v>4.636107593496235</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.6337399038025</v>
+        <v>4.633714787462631</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637326270975357</v>
+        <v>4.637320853304352</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.63458015027004</v>
+        <v>4.634594518371909</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.628007985612254</v>
+        <v>4.628050043447324</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.624296368195214</v>
+        <v>4.624341497248192</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599649919286602</v>
+        <v>4.599694525085565</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.580544423209435</v>
+        <v>4.580642375415843</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.562379915138801</v>
+        <v>4.562539277364912</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.525121502450814</v>
+        <v>4.525355644148628</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.523208849990008</v>
+        <v>4.523540549098687</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.536370575346857</v>
+        <v>4.536735497122693</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.55529800493181</v>
+        <v>4.555668030744667</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.588259940898809</v>
+        <v>4.58867234500087</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.608032201243928</v>
+        <v>4.608547417934535</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.681456889978612</v>
+        <v>4.682049011285836</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.717436954603984</v>
+        <v>4.718065209593451</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.783693861870402</v>
+        <v>4.784272614686989</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.816725016140897</v>
+        <v>4.81706555375955</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.814388998646903</v>
+        <v>4.81471953422098</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.823573863441331</v>
+        <v>4.823900474365166</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862689747328234</v>
+        <v>4.862719405967363</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855277524753345</v>
+        <v>4.85529229556216</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.851295912381261</v>
+        <v>4.851138222989204</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.828919357513346</v>
+        <v>4.82880235858179</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.836399457823369</v>
+        <v>4.836247478748165</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.888168083670111</v>
+        <v>4.887902161519925</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.915876106572155</v>
+        <v>4.915710856710577</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.925076803800293</v>
+        <v>4.924910387568636</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.915271001957048</v>
+        <v>4.915115479946335</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.896447143083222</v>
+        <v>4.896321260959314</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.893864761702012</v>
+        <v>4.893659493381961</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.893642183420015</v>
+        <v>4.893360319771435</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.88993242869109</v>
+        <v>4.889553935707834</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.874300691897856</v>
+        <v>4.873909281098458</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.851607934554204</v>
+        <v>4.851273905904188</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.825485601032801</v>
+        <v>4.825158609026223</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.816385348329109</v>
+        <v>4.816071417822718</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.786865551106078</v>
+        <v>4.78659559879244</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.758934934085192</v>
+        <v>4.758671174362827</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.748060270331666</v>
+        <v>4.750513434619763</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.753695613693639</v>
+        <v>4.75622893839928</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.746516867541136</v>
+        <v>4.747937150067212</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.738484714775065</v>
+        <v>4.738597365424148</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.727471509107215</v>
+        <v>4.726647104930283</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.703555189879308</v>
+        <v>4.700764581330889</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.681126432600848</v>
+        <v>4.676402229728178</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.666312335646032</v>
+        <v>4.660446750337369</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.643408596861399</v>
+        <v>4.636671533545909</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.623919738275172</v>
+        <v>4.616030413781527</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.606518129648261</v>
+        <v>4.599923601131028</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.607193507875372</v>
+        <v>4.601521532517905</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.616595009512515</v>
+        <v>4.614208897724895</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.672145515419937</v>
+        <v>4.694474863434344</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.619874265419938</v>
+        <v>4.642203613434345</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-07-28_20-55-15
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.747937150067212</v>
+        <v>4.747933364136453</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.738597365424148</v>
+        <v>4.738594729244936</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.726647104930283</v>
+        <v>4.72672803937691</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.700764581330889</v>
+        <v>4.700853776704053</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.676402229728178</v>
+        <v>4.676573568553655</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.660446750337369</v>
+        <v>4.660547512230597</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.636671533545909</v>
+        <v>4.636708383728456</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.616030413781527</v>
+        <v>4.616011870583229</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.599923601131028</v>
+        <v>4.599940927062196</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.601521532517905</v>
+        <v>4.601406961637692</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.614208897724895</v>
+        <v>4.614041768467119</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.694474863434344</v>
+        <v>4.694099953469754</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.642203613434345</v>
+        <v>4.641828703469755</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-07-29_20-35-45
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712878218900197</v>
+        <v>4.712876012655899</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711468495714417</v>
+        <v>4.711478840892678</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.719938613297313</v>
+        <v>4.719951195380259</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706426385580516</v>
+        <v>4.706452456968051</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.693767318948504</v>
+        <v>4.693793685740667</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.67783772544897</v>
+        <v>4.677864321629303</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.672845570912368</v>
+        <v>4.672872226272231</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.685921940486619</v>
+        <v>4.685948572861285</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.701765545298469</v>
+        <v>4.701797437099546</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705184520141215</v>
+        <v>4.705205664732511</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694247018597318</v>
+        <v>4.694268589314833</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664240229289093</v>
+        <v>4.6642636170509</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.64957962757275</v>
+        <v>4.649582691367434</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641207405657332</v>
+        <v>4.641215721272177</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636107593496235</v>
+        <v>4.636113071236441</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633714787462631</v>
+        <v>4.633727554814358</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637320853304352</v>
+        <v>4.637323597778664</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634594518371909</v>
+        <v>4.634587210240718</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.628050043447324</v>
+        <v>4.628028663871838</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.624341497248192</v>
+        <v>4.624318554083416</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599694525085565</v>
+        <v>4.599671846397577</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.580642375415843</v>
+        <v>4.580592545910143</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.562539277364912</v>
+        <v>4.562458196114482</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.525355644148628</v>
+        <v>4.525236533604158</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.523540549098687</v>
+        <v>4.523371822844088</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.536735497122693</v>
+        <v>4.536549897714296</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.555668030744667</v>
+        <v>4.555479858058352</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.58867234500087</v>
+        <v>4.588462654385445</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.608547417934535</v>
+        <v>4.608285554861165</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.682049011285836</v>
+        <v>4.681748050173348</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.718065209593451</v>
+        <v>4.717745879460526</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.784272614686989</v>
+        <v>4.783978579615784</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.81706555375955</v>
+        <v>4.816892534375414</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.81471953422098</v>
+        <v>4.814551628306155</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.823900474365166</v>
+        <v>4.823734602642347</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862719405967363</v>
+        <v>4.862704379167003</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.85529229556216</v>
+        <v>4.855284840503039</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.851138222989204</v>
+        <v>4.851218372252974</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.82880235858179</v>
+        <v>4.82886186917456</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.836247478748165</v>
+        <v>4.836324757369228</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.887902161519925</v>
+        <v>4.888037343912102</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.915710856710577</v>
+        <v>4.915794925972706</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.924910387568636</v>
+        <v>4.924995036443691</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.915115479946335</v>
+        <v>4.915194523455526</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.896321260959314</v>
+        <v>4.896385248652617</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.893659493381961</v>
+        <v>4.893763782573879</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.893360319771435</v>
+        <v>4.893503461370724</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.889553935707834</v>
+        <v>4.889746191941164</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.873909281098458</v>
+        <v>4.874108121347843</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.851273905904188</v>
+        <v>4.851443645332772</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.825158609026223</v>
+        <v>4.825324857309067</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.816071417822718</v>
+        <v>4.816231047229683</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.78659559879244</v>
+        <v>4.786732937754311</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.758671174362827</v>
+        <v>4.758805252737195</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.750513434619763</v>
+        <v>4.750639826128286</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.75622893839928</v>
+        <v>4.754403038774767</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.747933364136453</v>
+        <v>4.746592956469639</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.738594729244936</v>
+        <v>4.737978575337989</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.72672803937691</v>
+        <v>4.727255188780356</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.700853776704053</v>
+        <v>4.702502189726475</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.676573568553655</v>
+        <v>4.679053593036145</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.660547512230597</v>
+        <v>4.663189657365087</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.636708383728456</v>
+        <v>4.640401713975646</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.616011870583229</v>
+        <v>4.620732996835541</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.599940927062196</v>
+        <v>4.604033628916819</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.601406961637692</v>
+        <v>4.60431422866121</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.614041768467119</v>
+        <v>4.615222329228865</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.694099953469754</v>
+        <v>4.681503697787258</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.641828703469755</v>
+        <v>4.630365077770415</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-07-29_20-37-52
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712876012655899</v>
+        <v>4.712871817114962</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711478840892678</v>
+        <v>4.711498506036667</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.719951195380259</v>
+        <v>4.719975125288164</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706452456968051</v>
+        <v>4.706502032615644</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.693793685740667</v>
+        <v>4.693843823255224</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.677864321629303</v>
+        <v>4.677914895294445</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.672872226272231</v>
+        <v>4.672922913580944</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.685948572861285</v>
+        <v>4.685999219442754</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.701797437099546</v>
+        <v>4.701858106490248</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705205664732511</v>
+        <v>4.705245893164991</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694268589314833</v>
+        <v>4.694309626737014</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.6642636170509</v>
+        <v>4.664308107857956</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649582691367434</v>
+        <v>4.649588601357279</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641215721272177</v>
+        <v>4.641231602881721</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636113071236441</v>
+        <v>4.636123490762367</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633727554814358</v>
+        <v>4.633751854632306</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637323597778664</v>
+        <v>4.63732887541098</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634587210240718</v>
+        <v>4.6345733260664</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.628028663871838</v>
+        <v>4.627987974763256</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.624318554083416</v>
+        <v>4.624274902723762</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599671846397577</v>
+        <v>4.599628707052067</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.580592545910143</v>
+        <v>4.580497921286462</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.562458196114482</v>
+        <v>4.562304292305855</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.525236533604158</v>
+        <v>4.525010345362248</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.523371822844088</v>
+        <v>4.523051342257997</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.536549897714296</v>
+        <v>4.536197218204009</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.555479858058352</v>
+        <v>4.555122159840012</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.588462654385445</v>
+        <v>4.588063864027519</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.608285554861165</v>
+        <v>4.607786950519599</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.681748050173348</v>
+        <v>4.68117506150482</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.717745879460526</v>
+        <v>4.717137936578222</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.783978579615784</v>
+        <v>4.783418027516049</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.816892534375414</v>
+        <v>4.816562742038151</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.814551628306155</v>
+        <v>4.814231401858454</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.823734602642347</v>
+        <v>4.82341802407018</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862704379167003</v>
+        <v>4.862675496079124</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855284840503039</v>
+        <v>4.855270346581722</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.851218372252974</v>
+        <v>4.851370968541032</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.82886186917456</v>
+        <v>4.828974924698077</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.836324757369228</v>
+        <v>4.836471706595797</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.888037343912102</v>
+        <v>4.888294595925952</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.915794925972706</v>
+        <v>4.915954543926217</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.924995036443691</v>
+        <v>4.92515583321798</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.915194523455526</v>
+        <v>4.915345037383958</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.896385248652617</v>
+        <v>4.896507044375335</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.893763782573879</v>
+        <v>4.893962584774183</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.893503461370724</v>
+        <v>4.89377668567629</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.889746191941164</v>
+        <v>4.890112922353286</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.874108121347843</v>
+        <v>4.874487283260223</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.851443645332772</v>
+        <v>4.851767031154453</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.825324857309067</v>
+        <v>4.825641108432115</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.816231047229683</v>
+        <v>4.816534582926701</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.786732937754311</v>
+        <v>4.786993676921098</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.758805252737195</v>
+        <v>4.759060427711328</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.750639826128286</v>
+        <v>4.748181603235642</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.754403038774767</v>
+        <v>4.752105543764435</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.746592956469639</v>
+        <v>4.745315478581345</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.737978575337989</v>
+        <v>4.737856310511066</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.727255188780356</v>
+        <v>4.727347381667077</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.702502189726475</v>
+        <v>4.704201824316748</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.679053593036145</v>
+        <v>4.682277296168913</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.663189657365087</v>
+        <v>4.667440638869559</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.640401713975646</v>
+        <v>4.645328780993667</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.620732996835541</v>
+        <v>4.626372056316018</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.604033628916819</v>
+        <v>4.608084328057078</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.60431422866121</v>
+        <v>4.607404614965041</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.615222329228865</v>
+        <v>4.61490713237605</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.681503697787258</v>
+        <v>4.660681118472981</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.630365077770415</v>
+        <v>4.608409868472982</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-07-30_20-32-57
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712871817114962</v>
+        <v>4.712873879932303</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711498506036667</v>
+        <v>4.711488838595651</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.719975125288164</v>
+        <v>4.71996335920851</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706502032615644</v>
+        <v>4.706477658376062</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.693843823255224</v>
+        <v>4.693819172745645</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.677914895294445</v>
+        <v>4.677890030354432</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.672922913580944</v>
+        <v>4.672897992585171</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.685999219442754</v>
+        <v>4.685974317982873</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.701858106490248</v>
+        <v>4.701828273669522</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705245893164991</v>
+        <v>4.705226111070846</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694309626737014</v>
+        <v>4.694289447110599</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664308107857956</v>
+        <v>4.664286230641764</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649588601357279</v>
+        <v>4.649585681895855</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641231602881721</v>
+        <v>4.641223783232535</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636123490762367</v>
+        <v>4.636118367363091</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633751854632306</v>
+        <v>4.6337399038025</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.63732887541098</v>
+        <v>4.637326270975357</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.6345733260664</v>
+        <v>4.63458015027004</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627987974763256</v>
+        <v>4.628007985612254</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.624274902723762</v>
+        <v>4.624296368195214</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599628707052067</v>
+        <v>4.599649919286602</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.580497921286462</v>
+        <v>4.580544423209435</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.562304292305855</v>
+        <v>4.562379915138801</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.525010345362248</v>
+        <v>4.525121502450814</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.523051342257997</v>
+        <v>4.523208849990008</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.536197218204009</v>
+        <v>4.536370575346857</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.555122159840012</v>
+        <v>4.55529800493181</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.588063864027519</v>
+        <v>4.588259940898809</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.607786950519599</v>
+        <v>4.608032201243928</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.68117506150482</v>
+        <v>4.681456889978612</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.717137936578222</v>
+        <v>4.717436954603984</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.783418027516049</v>
+        <v>4.783693861870402</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.816562742038151</v>
+        <v>4.816725016140897</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.814231401858454</v>
+        <v>4.814388998646903</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.82341802407018</v>
+        <v>4.823573863441331</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862675496079124</v>
+        <v>4.862689747328234</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855270346581722</v>
+        <v>4.855277524753345</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.851370968541032</v>
+        <v>4.851295912381261</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.828974924698077</v>
+        <v>4.828919357513346</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.836471706595797</v>
+        <v>4.836399457823369</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.888294595925952</v>
+        <v>4.888168083670111</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.915954543926217</v>
+        <v>4.915876106572155</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.92515583321798</v>
+        <v>4.925076803800293</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.915345037383958</v>
+        <v>4.915271001957048</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.896507044375335</v>
+        <v>4.896447143083222</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.893962584774183</v>
+        <v>4.893864761702012</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.89377668567629</v>
+        <v>4.893642183420015</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.890112922353286</v>
+        <v>4.88993242869109</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.874487283260223</v>
+        <v>4.874300691897856</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.851767031154453</v>
+        <v>4.851607934554204</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.825641108432115</v>
+        <v>4.825485601032801</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.816534582926701</v>
+        <v>4.816385348329109</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.786993676921098</v>
+        <v>4.786865551106078</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.759060427711328</v>
+        <v>4.758934934085192</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.748181603235642</v>
+        <v>4.750762258975438</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.752105543764435</v>
+        <v>4.751652949061699</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.745315478581345</v>
+        <v>4.744123754332573</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.737856310511066</v>
+        <v>4.736115696202784</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.727347381667077</v>
+        <v>4.726176500241142</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.704201824316748</v>
+        <v>4.702267068744298</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.682277296168913</v>
+        <v>4.679394396541389</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.667440638869559</v>
+        <v>4.663575122044363</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.645328780993667</v>
+        <v>4.641442517520861</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.626372056316018</v>
+        <v>4.622075364296297</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.608084328057078</v>
+        <v>4.604377129336613</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.607404614965041</v>
+        <v>4.603183570815087</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.61490713237605</v>
+        <v>4.611850323952472</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.660681118472981</v>
+        <v>4.664622598797662</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.608409868472982</v>
+        <v>4.608527643965873</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-08-01_09-22-44
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712873879932303</v>
+        <v>4.712869820822521</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711488838595651</v>
+        <v>4.711507859310824</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.71996335920851</v>
+        <v>4.719986512806905</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706477658376062</v>
+        <v>4.706525619735528</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.693819172745645</v>
+        <v>4.693867677767903</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.677890030354432</v>
+        <v>4.677938957301652</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.672897992585171</v>
+        <v>4.67294703016887</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.685974317982873</v>
+        <v>4.686023318024004</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.701828273669522</v>
+        <v>4.70188698375071</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705226111070846</v>
+        <v>4.705265042851488</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694289447110599</v>
+        <v>4.694329160724887</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664286230641764</v>
+        <v>4.66432928407586</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649585681895855</v>
+        <v>4.64959145189862</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641223783232535</v>
+        <v>4.641239190902513</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636118367363091</v>
+        <v>4.636128449749937</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.6337399038025</v>
+        <v>4.633763426230251</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637326270975357</v>
+        <v>4.637331413503139</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.63458015027004</v>
+        <v>4.634566726045901</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.628007985612254</v>
+        <v>4.627968599567516</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.624296368195214</v>
+        <v>4.624254123161657</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599649919286602</v>
+        <v>4.599608175341391</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.580544423209435</v>
+        <v>4.580452959788063</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.562379915138801</v>
+        <v>4.56223119491392</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.525121502450814</v>
+        <v>4.52490287052077</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.523208849990008</v>
+        <v>4.522899030247529</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.536370575346857</v>
+        <v>4.536029534704713</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.55529800493181</v>
+        <v>4.554952031306052</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.588259940898809</v>
+        <v>4.587874104936371</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.608032201243928</v>
+        <v>4.607549421518016</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.681456889978612</v>
+        <v>4.68090212491516</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.717436954603984</v>
+        <v>4.716848358149185</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.783693861870402</v>
+        <v>4.783150669023462</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.816725016140897</v>
+        <v>4.816405470735526</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.814388998646903</v>
+        <v>4.814078609204709</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.823573863441331</v>
+        <v>4.823266865570835</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862689747328234</v>
+        <v>4.862661611659824</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855277524753345</v>
+        <v>4.855263304054856</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.851295912381261</v>
+        <v>4.85144365803102</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.828919357513346</v>
+        <v>4.829028665215736</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.836399457823369</v>
+        <v>4.83654162205697</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.888168083670111</v>
+        <v>4.888417082163214</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.915876106572155</v>
+        <v>4.916030373910361</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.925076803800293</v>
+        <v>4.925232258959792</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.915271001957048</v>
+        <v>4.915416744121206</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.896447143083222</v>
+        <v>4.896565046426828</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.893864761702012</v>
+        <v>4.894057396461353</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.893642183420015</v>
+        <v>4.893907156154</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.88993242869109</v>
+        <v>4.890287932779508</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.874300691897856</v>
+        <v>4.874668168359173</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.851607934554204</v>
+        <v>4.851921176786336</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.825485601032801</v>
+        <v>4.825791630636801</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.816385348329109</v>
+        <v>4.816678995991471</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.786865551106078</v>
+        <v>4.78711753764903</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.758934934085192</v>
+        <v>4.759181930061327</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.750762258975438</v>
+        <v>4.748299314758032</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.751652949061699</v>
+        <v>4.751694854686076</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.744123754332573</v>
+        <v>4.745555198369468</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.736115696202784</v>
+        <v>4.738843966428937</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.726176500241142</v>
+        <v>4.729415598700902</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.702267068744298</v>
+        <v>4.707643776577807</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.679394396541389</v>
+        <v>4.686921006933111</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.663575122044363</v>
+        <v>4.672921951991436</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.641442517520861</v>
+        <v>4.652219511131811</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.622075364296297</v>
+        <v>4.635094706022998</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.604377129336613</v>
+        <v>4.618123562230819</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.603183570815087</v>
+        <v>4.617630714834592</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.611850323952472</v>
+        <v>4.625508913577971</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.664622598797662</v>
+        <v>4.671601312665572</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.608527643965873</v>
+        <v>4.643091536989962</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-08-03_21-11-05
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712869820822521</v>
+        <v>4.712867887888216</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711507859310824</v>
+        <v>4.711516913484314</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.719986512806905</v>
+        <v>4.71999753973825</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706525619735528</v>
+        <v>4.706548457241251</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.693867677767903</v>
+        <v>4.693890774210512</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.677938957301652</v>
+        <v>4.677962254634158</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.67294703016887</v>
+        <v>4.672970380661521</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686023318024004</v>
+        <v>4.686046651923874</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.70188698375071</v>
+        <v>4.701914950605983</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705265042851488</v>
+        <v>4.705283589965304</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694329160724887</v>
+        <v>4.694348079558097</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.66432928407586</v>
+        <v>4.664349792442509</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.64959145189862</v>
+        <v>4.649594235611573</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641239190902513</v>
+        <v>4.641246557364059</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636128449749937</v>
+        <v>4.636133252116022</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633763426230251</v>
+        <v>4.633774636343475</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637331413503139</v>
+        <v>4.63733388757333</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634566726045901</v>
+        <v>4.634560339369336</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627968599567516</v>
+        <v>4.627949830248463</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.624254123161657</v>
+        <v>4.624233997169318</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599608175341391</v>
+        <v>4.599588291965418</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.580452959788063</v>
+        <v>4.580409463575861</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.56223119491392</v>
+        <v>4.562160498924329</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.52490287052077</v>
+        <v>4.52479889852763</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.522899030247529</v>
+        <v>4.522751661920491</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.536029534704713</v>
+        <v>4.53586725189415</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.554952031306052</v>
+        <v>4.554787346321281</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.587874104936371</v>
+        <v>4.587690364779887</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.607549421518016</v>
+        <v>4.607319256517915</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.68090212491516</v>
+        <v>4.680637667480855</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.716848358149185</v>
+        <v>4.716567780898628</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.783150669023462</v>
+        <v>4.782891403300569</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.816405470735526</v>
+        <v>4.816252975415085</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.814078609204709</v>
+        <v>4.813930405519906</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.823266865570835</v>
+        <v>4.823120181730422</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862661611659824</v>
+        <v>4.862648080898103</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855263304054856</v>
+        <v>4.855256395077048</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.85144365803102</v>
+        <v>4.851514090889548</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.829028665215736</v>
+        <v>4.829080667471169</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.83654162205697</v>
+        <v>4.8366093151011</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.888417082163214</v>
+        <v>4.88853573128088</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.916030373910361</v>
+        <v>4.916103723623912</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.925232258959792</v>
+        <v>4.925306206710811</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.915416744121206</v>
+        <v>4.915486229576024</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.896565046426828</v>
+        <v>4.896621237381213</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.894057396461353</v>
+        <v>4.894149332789015</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.893907156154</v>
+        <v>4.894033771966064</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.890287932779508</v>
+        <v>4.890457704487634</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.874668168359173</v>
+        <v>4.874843603835883</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.851921176786336</v>
+        <v>4.852070598379175</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.825791630636801</v>
+        <v>4.825937403010329</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.816678995991471</v>
+        <v>4.816818816984716</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.78711753764903</v>
+        <v>4.787237341368896</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.759181930061327</v>
+        <v>4.759299625677675</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.748299314758032</v>
+        <v>4.748413560475131</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.751694854686076</v>
+        <v>4.751310513067219</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.745555198369468</v>
+        <v>4.745763242247619</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.738843966428937</v>
+        <v>4.739741522996269</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.729415598700902</v>
+        <v>4.731298528757993</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.707643776577807</v>
+        <v>4.71079624597955</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.686921006933111</v>
+        <v>4.691204052889341</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.672921951991436</v>
+        <v>4.677887680571043</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.652219511131811</v>
+        <v>4.658444111894196</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.635094706022998</v>
+        <v>4.64287924433197</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.618123562230819</v>
+        <v>4.627035383196576</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.617630714834592</v>
+        <v>4.62665795194516</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.625508913577971</v>
+        <v>4.634736044587116</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.671601312665572</v>
+        <v>4.680337026722484</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.643091536989962</v>
+        <v>4.670518213086879</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-08-04_20-35-47
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712867887888216</v>
+        <v>4.712866015343125</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711516913484314</v>
+        <v>4.711525682675338</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.71999753973825</v>
+        <v>4.720008222936054</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706548457241251</v>
+        <v>4.706570580293787</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.693890774210512</v>
+        <v>4.693913148139066</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.677962254634158</v>
+        <v>4.677984823158474</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.672970380661521</v>
+        <v>4.672993000977454</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686046651923874</v>
+        <v>4.686069256955439</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.701914950605983</v>
+        <v>4.701942049412115</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705283589965304</v>
+        <v>4.705301562494599</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694348079558097</v>
+        <v>4.694366411832019</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664349792442509</v>
+        <v>4.664369664048394</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649594235611573</v>
+        <v>4.649596954530671</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641246557364059</v>
+        <v>4.641253711764886</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636133252116022</v>
+        <v>4.636137905166266</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633774636343475</v>
+        <v>4.63378550163012</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.63733388757333</v>
+        <v>4.637336299850019</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634560339369336</v>
+        <v>4.634554155883445</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627949830248463</v>
+        <v>4.627931638858437</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.624233997169318</v>
+        <v>4.624214494407495</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599588291965418</v>
+        <v>4.599569026730975</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.580409463575861</v>
+        <v>4.58036736231073</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.562160498924329</v>
+        <v>4.562092088267763</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.52479889852763</v>
+        <v>4.524698261416848</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.522751661920491</v>
+        <v>4.522609001228933</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.53586725189415</v>
+        <v>4.535710113985182</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.554787346321281</v>
+        <v>4.554627848911858</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.587690364779887</v>
+        <v>4.587512363168321</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.607319256517915</v>
+        <v>4.607096119477982</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.680637667480855</v>
+        <v>4.680381301532541</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.716567780898628</v>
+        <v>4.716295793044857</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.782891403300569</v>
+        <v>4.782639869896713</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.816252975415085</v>
+        <v>4.816105042703161</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.813930405519906</v>
+        <v>4.813786588223483</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.823120181730422</v>
+        <v>4.822977778175814</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862648080898103</v>
+        <v>4.862634891184993</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855256395077048</v>
+        <v>4.855249617424001</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.851514090889548</v>
+        <v>4.851582370446934</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.829080667471169</v>
+        <v>4.829131014267672</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.8366093151011</v>
+        <v>4.836674889725463</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.88853573128088</v>
+        <v>4.8886507205593</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.916103723623912</v>
+        <v>4.91617471208353</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.925306206710811</v>
+        <v>4.925377794248007</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.915486229576024</v>
+        <v>4.915553594697814</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.896621237381213</v>
+        <v>4.89667570005777</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.894149332789015</v>
+        <v>4.894238521768552</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.894033771966064</v>
+        <v>4.89415670009447</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.890457704487634</v>
+        <v>4.890622467767908</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.874843603835883</v>
+        <v>4.87501383123911</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.852070598379175</v>
+        <v>4.852215509240193</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.825937403010329</v>
+        <v>4.826078646364962</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.816818816984716</v>
+        <v>4.816954261065348</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.787237341368896</v>
+        <v>4.787353282924164</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.759299625677675</v>
+        <v>4.759413688072785</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.751107541126864</v>
+        <v>4.748524487438184</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.751036559287916</v>
+        <v>4.751472956257077</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.743812873370253</v>
+        <v>4.745059261185702</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.737713790447097</v>
+        <v>4.739496367306812</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.729668343955138</v>
+        <v>4.731504629230277</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.70934860376962</v>
+        <v>4.712690159428689</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.688721671585933</v>
+        <v>4.694012700710838</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.673976837864206</v>
+        <v>4.681337726027865</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.654478546625905</v>
+        <v>4.663156722528498</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.637871013273847</v>
+        <v>4.649124130537682</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.620343338750931</v>
+        <v>4.634701224183329</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.616530500860587</v>
+        <v>4.635063792748839</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.622711269997369</v>
+        <v>4.643930168962694</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.662851902663623</v>
+        <v>4.690008494171652</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.634164917517662</v>
+        <v>4.693752206433306</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.636814244349647</v>
+        <v>4.746023456433305</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-08-05_20-33-15
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.748524487438184</v>
+        <v>4.751215826175638</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.751472956257077</v>
+        <v>4.751207413842916</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.745059261185702</v>
+        <v>4.744414209554312</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.739496367306812</v>
+        <v>4.738950862961294</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.731504629230277</v>
+        <v>4.731464438740936</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.712690159428689</v>
+        <v>4.712760971179501</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.694012700710838</v>
+        <v>4.692727875735451</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.681337726027865</v>
+        <v>4.678422263314411</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.663156722528498</v>
+        <v>4.659717549944556</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.649124130537682</v>
+        <v>4.6440906638262</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.634701224183329</v>
+        <v>4.627291874553226</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.635063792748839</v>
+        <v>4.622620048519578</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.643930168962694</v>
+        <v>4.6284495930726</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.690008494171652</v>
+        <v>4.666999838090203</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.693752206433306</v>
+        <v>4.645035940761469</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.746023456433305</v>
+        <v>4.668402622166458</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-08-05_20-36-26
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712866015343125</v>
+        <v>4.712864200400956</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711525682675338</v>
+        <v>4.711534180127502</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720008222936054</v>
+        <v>4.720018578220326</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706570580293787</v>
+        <v>4.706592021889866</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.693913148139066</v>
+        <v>4.69393483292109</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.677984823158474</v>
+        <v>4.67800669653346</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.672993000977454</v>
+        <v>4.673014924825258</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686069256955439</v>
+        <v>4.686091166730698</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.701942049412115</v>
+        <v>4.701968319939565</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705301562494599</v>
+        <v>4.705318986721398</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694366411832019</v>
+        <v>4.694384184397479</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664369664048394</v>
+        <v>4.664388928084452</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649596954530671</v>
+        <v>4.649599610632086</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641253711764886</v>
+        <v>4.641260663072385</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636137905166266</v>
+        <v>4.636142415758837</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.63378550163012</v>
+        <v>4.633796037741498</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637336299850019</v>
+        <v>4.637338652471806</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634554155883445</v>
+        <v>4.634548166067622</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627931638858437</v>
+        <v>4.627913999140556</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.624214494407495</v>
+        <v>4.624195586385056</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599569026730975</v>
+        <v>4.599550351288725</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.58036736231073</v>
+        <v>4.580326590076345</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.562092088267763</v>
+        <v>4.562025854215981</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.524698261416848</v>
+        <v>4.524600801761277</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.522609001228933</v>
+        <v>4.522470826870562</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.535710113985182</v>
+        <v>4.535557881034304</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.554627848911858</v>
+        <v>4.554473298836204</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.587512363168321</v>
+        <v>4.587339836772051</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.607096119477982</v>
+        <v>4.606879694425007</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.680381301532541</v>
+        <v>4.680132662593904</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.716295793044857</v>
+        <v>4.716032007457517</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.782639869896713</v>
+        <v>4.782395729362111</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.816105042703161</v>
+        <v>4.815961471693582</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.813786588223483</v>
+        <v>4.813646966418904</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.822977778175814</v>
+        <v>4.822839471543498</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862634891184993</v>
+        <v>4.86262203045078</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855249617424001</v>
+        <v>4.855242968771631</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.851582370446934</v>
+        <v>4.851648593828299</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.829131014267672</v>
+        <v>4.829179783242807</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.836674889725463</v>
+        <v>4.836738443556834</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.8886507205593</v>
+        <v>4.888762216538677</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.91617471208353</v>
+        <v>4.91624345085231</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.925377794248007</v>
+        <v>4.925447132048654</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.915553594697814</v>
+        <v>4.915618934452631</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.89667570005777</v>
+        <v>4.896728512344025</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.894238521768552</v>
+        <v>4.894325083974538</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.89415670009447</v>
+        <v>4.894276098097219</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.890622467767908</v>
+        <v>4.890782439695531</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.87501383123911</v>
+        <v>4.875179078113375</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.852215509240193</v>
+        <v>4.852356110058788</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.826078646364962</v>
+        <v>4.826215568066502</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.816954261065348</v>
+        <v>4.817085530184782</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.787353282924164</v>
+        <v>4.787465544952523</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.759413688072785</v>
+        <v>4.759524280527801</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.751215826175638</v>
+        <v>4.748632234728814</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.751207413842916</v>
+        <v>4.751631246427197</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.744414209554312</v>
+        <v>4.745574162590534</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.738950862961294</v>
+        <v>4.740598423744132</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.731464438740936</v>
+        <v>4.733259844639816</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.712760971179501</v>
+        <v>4.716078868202238</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.692727875735451</v>
+        <v>4.698420451277189</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.678422263314411</v>
+        <v>4.686487234963083</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.659717549944556</v>
+        <v>4.669637950222205</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.6440906638262</v>
+        <v>4.657290021776928</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.627291874553226</v>
+        <v>4.644348141286654</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.622620048519578</v>
+        <v>4.645627325447425</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.6284495930726</v>
+        <v>4.655453075546752</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.666999838090203</v>
+        <v>4.702815119993426</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.645035940761469</v>
+        <v>4.718264889514428</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.668402622166458</v>
+        <v>4.770536139514427</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-08-06_20-33-11
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.748632234728814</v>
+        <v>4.751320949547302</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.751631246427197</v>
+        <v>4.751373810307898</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.745574162590534</v>
+        <v>4.745411200504873</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.740598423744132</v>
+        <v>4.740633022783004</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.733259844639816</v>
+        <v>4.733813495452916</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.716078868202238</v>
+        <v>4.716596337675188</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.698420451277189</v>
+        <v>4.697339653086992</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.686487234963083</v>
+        <v>4.683480959400096</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.669637950222205</v>
+        <v>4.665636676013134</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.657290021776928</v>
+        <v>4.651095441221752</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.644348141286654</v>
+        <v>4.635135583293053</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.645627325447425</v>
+        <v>4.62996347123537</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.655453075546752</v>
+        <v>4.635718619131501</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.702815119993426</v>
+        <v>4.673605074413755</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.718264889514428</v>
+        <v>4.657811987223591</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.770536139514427</v>
+        <v>4.691106425543316</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-08-06_20-36-50
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712864200400956</v>
+        <v>4.712862440444212</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711534180127502</v>
+        <v>4.711542418276479</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720018578220326</v>
+        <v>4.720028620455285</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706592021889866</v>
+        <v>4.706612813025898</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.69393483292109</v>
+        <v>4.693955859901386</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.67800669653346</v>
+        <v>4.678027906377536</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673014924825258</v>
+        <v>4.673036183870882</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686091166730698</v>
+        <v>4.686112412827034</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.701968319939565</v>
+        <v>4.701993799567395</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705318986721398</v>
+        <v>4.705335887349587</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694384184397479</v>
+        <v>4.69440142249174</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664388928084452</v>
+        <v>4.664407611984911</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649599610632086</v>
+        <v>4.64960220583305</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641260663072385</v>
+        <v>4.641267419759099</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636142415758837</v>
+        <v>4.636146790338179</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633796037741498</v>
+        <v>4.63380625939693</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637338652471806</v>
+        <v>4.637340947490681</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634548166067622</v>
+        <v>4.634542360985506</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627913999140556</v>
+        <v>4.627896886402928</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.624195586385056</v>
+        <v>4.624177246320458</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599550351288725</v>
+        <v>4.599532238994698</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.580326590076345</v>
+        <v>4.580287085037537</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.562025854215981</v>
+        <v>4.56196169481194</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.524600801761277</v>
+        <v>4.524506371861037</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.522470826870562</v>
+        <v>4.522336931158366</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.535557881034304</v>
+        <v>4.535410327737839</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.554473298836204</v>
+        <v>4.554323470399674</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.587339836772051</v>
+        <v>4.587172538050048</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.606879694425007</v>
+        <v>4.606669683983215</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.680132662593904</v>
+        <v>4.679891407679042</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.716032007457517</v>
+        <v>4.715776059846661</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.782395729362111</v>
+        <v>4.782158661747232</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.815961471693582</v>
+        <v>4.815822073054423</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.813646966418904</v>
+        <v>4.813511360068336</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.822839471543498</v>
+        <v>4.822705088717619</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.86262203045078</v>
+        <v>4.862609487141476</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855242968771631</v>
+        <v>4.855236446720663</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.851648593828299</v>
+        <v>4.85171285241185</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.829179783242807</v>
+        <v>4.829227047264236</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.836738443556834</v>
+        <v>4.836800068330565</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.888762216538677</v>
+        <v>4.888870375819135</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.91624345085231</v>
+        <v>4.916310044611315</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.925447132048654</v>
+        <v>4.925514323843795</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.915618934452631</v>
+        <v>4.915682338256774</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.896728512344025</v>
+        <v>4.896779747554323</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.894325083974538</v>
+        <v>4.894409133073223</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.894276098097219</v>
+        <v>4.894392114757535</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.890782439695531</v>
+        <v>4.890937825058653</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.875179078113375</v>
+        <v>4.87533955899479</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.852356110058788</v>
+        <v>4.852492589823475</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.826215568066502</v>
+        <v>4.82634836304011</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.817085530184782</v>
+        <v>4.817212814082968</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.787465544952523</v>
+        <v>4.787574298821532</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.759524280527801</v>
+        <v>4.759631556824175</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.751320949547302</v>
+        <v>4.748736933973565</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.751373810307898</v>
+        <v>4.751785534105119</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.745411200504873</v>
+        <v>4.746482350457239</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.740633022783004</v>
+        <v>4.742159200580813</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.733813495452916</v>
+        <v>4.735556962423712</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.716596337675188</v>
+        <v>4.719963184485895</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.697339653086992</v>
+        <v>4.703400726008264</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.683480959400096</v>
+        <v>4.692301705071877</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.665636676013134</v>
+        <v>4.676844973878919</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.651095441221752</v>
+        <v>4.666260559942814</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.635135583293053</v>
+        <v>4.654868784045101</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.62996347123537</v>
+        <v>4.657410107631515</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.635718619131501</v>
+        <v>4.668381835213083</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.673605074413755</v>
+        <v>4.717477037556458</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.657811987223591</v>
+        <v>4.742766944012038</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.691106425543316</v>
+        <v>4.831295753286478</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-08-07_20-33-04
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.748736933973565</v>
+        <v>4.751423044926354</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.751785534105119</v>
+        <v>4.751535914816518</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.746482350457239</v>
+        <v>4.745449240809208</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.742159200580813</v>
+        <v>4.741122252619931</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.735556962423712</v>
+        <v>4.73467696202985</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.719963184485895</v>
+        <v>4.718753288556779</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.703400726008264</v>
+        <v>4.700144577380675</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.692301705071877</v>
+        <v>4.686650038169422</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.676844973878919</v>
+        <v>4.669489444255235</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.666260559942814</v>
+        <v>4.655681392212383</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.654868784045101</v>
+        <v>4.640326713435906</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.657410107631515</v>
+        <v>4.634510831245238</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.668381835213083</v>
+        <v>4.639899575677101</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.717477037556458</v>
+        <v>4.676006640172082</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.742766944012038</v>
+        <v>4.663258343364158</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.831295753286478</v>
+        <v>4.692818710813657</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-08-08_13-25-43
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712862440444212</v>
+        <v>4.712859075786589</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711542418276479</v>
+        <v>4.711558162726627</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720028620455285</v>
+        <v>4.720047820875387</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706612813025898</v>
+        <v>4.706652558784249</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.693955859901386</v>
+        <v>4.693996056614607</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678027906377536</v>
+        <v>4.678068452644531</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673036183870882</v>
+        <v>4.67307682490686</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686112412827034</v>
+        <v>4.686153031015647</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.701993799567395</v>
+        <v>4.702042524729798</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705335887349587</v>
+        <v>4.705368209424684</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.69440142249174</v>
+        <v>4.694434388853634</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664407611984911</v>
+        <v>4.664443341101799</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.64960220583305</v>
+        <v>4.649607220907673</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641267419759099</v>
+        <v>4.641280380883718</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636146790338179</v>
+        <v>4.636155155348053</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.63380625939693</v>
+        <v>4.633825813961011</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637340947490681</v>
+        <v>4.637345372514269</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634542360985506</v>
+        <v>4.634531271937869</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627896886402928</v>
+        <v>4.627864150247204</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.624177246320458</v>
+        <v>4.624142170740007</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599532238994698</v>
+        <v>4.599497605056221</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.580287085037537</v>
+        <v>4.580211647776609</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.56196169481194</v>
+        <v>4.561839222915093</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.524506371861037</v>
+        <v>4.524326054802028</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.522336931158366</v>
+        <v>4.522081206922842</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.535410327737839</v>
+        <v>4.535128425613033</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.554323470399674</v>
+        <v>4.554037142013395</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.587172538050048</v>
+        <v>4.586852705547775</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.606669683983215</v>
+        <v>4.606267802469506</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.679891407679042</v>
+        <v>4.679429776229636</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.715776059846661</v>
+        <v>4.715286325812823</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.782158661747232</v>
+        <v>4.781704554847551</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.815822073054423</v>
+        <v>4.815555088591417</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.813511360068336</v>
+        <v>4.813251523392552</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.822705088717619</v>
+        <v>4.822447449115302</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862609487141476</v>
+        <v>4.862585309023499</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855236446720663</v>
+        <v>4.855223772572316</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.85171285241185</v>
+        <v>4.851835814437785</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.829227047264236</v>
+        <v>4.8293173301954</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.836800068330565</v>
+        <v>4.836917870770819</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.888870375819135</v>
+        <v>4.889077265298411</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.916310044611315</v>
+        <v>4.916437184487742</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.925514323843795</v>
+        <v>4.925642653591126</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.915682338256774</v>
+        <v>4.915803670276471</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.896779747554323</v>
+        <v>4.896877759079157</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.894409133073223</v>
+        <v>4.894570114938617</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.894392114757535</v>
+        <v>4.894614558843424</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.890937825058653</v>
+        <v>4.891235598848076</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.87533955899479</v>
+        <v>4.875647021280654</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.852492589823475</v>
+        <v>4.852753888599933</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.82634836304011</v>
+        <v>4.826602295723683</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.817212814082968</v>
+        <v>4.817456129483047</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.787574298821532</v>
+        <v>4.787781916233468</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.759631556824175</v>
+        <v>4.759836732537485</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.751423044926354</v>
+        <v>4.748937680383005</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.751535914816518</v>
+        <v>4.752082670646482</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.745449240809208</v>
+        <v>4.747418666433061</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.741122252619931</v>
+        <v>4.744108497865794</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.73467696202985</v>
+        <v>4.738470422205173</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.718753288556779</v>
+        <v>4.724968231340428</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.700144577380675</v>
+        <v>4.709971191474958</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.686650038169422</v>
+        <v>4.699999562902379</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.669489444255235</v>
+        <v>4.686435291480639</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.655681392212383</v>
+        <v>4.678038748638626</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.640326713435906</v>
+        <v>4.668661359503762</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.634510831245238</v>
+        <v>4.671843833388097</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.639899575677101</v>
+        <v>4.683201945924843</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.676006640172082</v>
+        <v>4.730174719333442</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.663258343364158</v>
+        <v>4.757099969827961</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.692818710813657</v>
+        <v>4.818424930120894</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-08-10_20-33-01
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712859075786589</v>
+        <v>4.71286073301161</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711558162726627</v>
+        <v>4.7115504088107</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720047820875387</v>
+        <v>4.720038363620429</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706652558784249</v>
+        <v>4.70663298284723</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.693996056614607</v>
+        <v>4.693976258552953</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678068452644531</v>
+        <v>4.678048482420934</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.67307682490686</v>
+        <v>4.673056807889981</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686153031015647</v>
+        <v>4.686133024938815</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702042524729798</v>
+        <v>4.702018523460239</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705368209424684</v>
+        <v>4.70535228762156</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694434388853634</v>
+        <v>4.694418149857863</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664443341101799</v>
+        <v>4.66442574155742</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649607220907673</v>
+        <v>4.649604741991754</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641280380883718</v>
+        <v>4.641273989836094</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636155155348053</v>
+        <v>4.636151034965748</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633825813961011</v>
+        <v>4.633816180452016</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637345372514269</v>
+        <v>4.637343186875307</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634531271937869</v>
+        <v>4.634536732240944</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627864150247204</v>
+        <v>4.62788027740389</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.624142170740007</v>
+        <v>4.624159449015482</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599497605056221</v>
+        <v>4.599514664784111</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.580211647776609</v>
+        <v>4.580248789129788</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.561839222915093</v>
+        <v>4.561899514352042</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.524326054802028</v>
+        <v>4.524414833005627</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.522081206922842</v>
+        <v>4.52220711899235</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.535128425613033</v>
+        <v>4.535267242335898</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.554037142013395</v>
+        <v>4.554178151374363</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.586852705547775</v>
+        <v>4.587010234089839</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.606267802469506</v>
+        <v>4.606465808030568</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.679429776229636</v>
+        <v>4.679657213737111</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.715286325812823</v>
+        <v>4.715527607108577</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.781704554847551</v>
+        <v>4.781928365228405</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.815555088591417</v>
+        <v>4.815686668210081</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.813251523392552</v>
+        <v>4.813379599235827</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.822447449115302</v>
+        <v>4.822574466129838</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862585309023499</v>
+        <v>4.862597250195908</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855223772572316</v>
+        <v>4.855230048817554</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.851835814437785</v>
+        <v>4.851775232247214</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.8293173301954</v>
+        <v>4.829272874789779</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.836917870770819</v>
+        <v>4.836859850327178</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.889077265298411</v>
+        <v>4.888975345790437</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.916437184487742</v>
+        <v>4.916374591679553</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.925642653591126</v>
+        <v>4.925579467122379</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.915803670276471</v>
+        <v>4.915743890373506</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.896877759079157</v>
+        <v>4.896829474757872</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.894570114938617</v>
+        <v>4.894490776306943</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.894614558843424</v>
+        <v>4.894504890680713</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.891235598848076</v>
+        <v>4.891088817209817</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.875647021280654</v>
+        <v>4.875495476323485</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.852753888599933</v>
+        <v>4.852625126660225</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.826602295723683</v>
+        <v>4.826477214687386</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.817456129483047</v>
+        <v>4.817336291195816</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.787781916233468</v>
+        <v>4.78767970547995</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.759836732537485</v>
+        <v>4.759735661914376</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.748937680383005</v>
+        <v>4.751522238730244</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.752082670646482</v>
+        <v>4.751693885734014</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.747418666433061</v>
+        <v>4.746483147561973</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.744108497865794</v>
+        <v>4.742803654113176</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.738470422205173</v>
+        <v>4.736950360269963</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.724968231340428</v>
+        <v>4.722046041739827</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.709971191474958</v>
+        <v>4.704275265649402</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.699999562902379</v>
+        <v>4.691351616443439</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.686435291480639</v>
+        <v>4.675082964399962</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.678038748638626</v>
+        <v>4.662324503506781</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.668661359503762</v>
+        <v>4.647821512806264</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.671843833388097</v>
+        <v>4.641907839110415</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.683201945924843</v>
+        <v>4.647417623267318</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.730174719333442</v>
+        <v>4.683319553503778</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.757099969827961</v>
+        <v>4.674928212692953</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.818424930120894</v>
+        <v>4.708233639695985</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-08-10_20-35-26
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.71286073301161</v>
+        <v>4.71285746658684</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.7115504088107</v>
+        <v>4.711565690379212</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720038363620429</v>
+        <v>4.720057004619123</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.70663298284723</v>
+        <v>4.70667156667664</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.693976258552953</v>
+        <v>4.694015280216637</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678048482420934</v>
+        <v>4.6780878434066</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673056807889981</v>
+        <v>4.673096261321311</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686133024938815</v>
+        <v>4.686172457388607</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702018523460239</v>
+        <v>4.70206583458241</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.70535228762156</v>
+        <v>4.705383673388586</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694418149857863</v>
+        <v>4.694450160551107</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.66442574155742</v>
+        <v>4.664460433518528</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649604741991754</v>
+        <v>4.649609644322182</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641273989836094</v>
+        <v>4.641286600079924</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636151034965748</v>
+        <v>4.636159156862262</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633816180452016</v>
+        <v>4.633835172233861</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637343186875307</v>
+        <v>4.637347506219321</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634536732240944</v>
+        <v>4.634525972643685</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.62788027740389</v>
+        <v>4.627848484286198</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.624159449015482</v>
+        <v>4.624125389126667</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599514664784111</v>
+        <v>4.599481037569078</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.580248789129788</v>
+        <v>4.580175609631921</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.561899514352042</v>
+        <v>4.561780735933091</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.524414833005627</v>
+        <v>4.524239914562038</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.52220711899235</v>
+        <v>4.521959022295985</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.535267242335898</v>
+        <v>4.534993689985829</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.554178151374363</v>
+        <v>4.5539002541502</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.587010234089839</v>
+        <v>4.586699745679653</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.606465808030568</v>
+        <v>4.606075418100952</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.679657213737111</v>
+        <v>4.679208807827525</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.715527607108577</v>
+        <v>4.715051910816641</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.781928365228405</v>
+        <v>4.781486961355119</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.815686668210081</v>
+        <v>4.81542717494749</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.813379599235827</v>
+        <v>4.813126980778245</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.822574466129838</v>
+        <v>4.822323891319574</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862597250195908</v>
+        <v>4.862573653482811</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855230048817554</v>
+        <v>4.855217615473622</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.851775232247214</v>
+        <v>4.851894675490656</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.829272874789779</v>
+        <v>4.829360474074398</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.836859850327178</v>
+        <v>4.836974206193359</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.888975345790437</v>
+        <v>4.88917626525444</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.916374591679553</v>
+        <v>4.916497910010555</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.925579467122379</v>
+        <v>4.925703969594553</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.915743890373506</v>
+        <v>4.915861752983016</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.896829474757872</v>
+        <v>4.896924661973425</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.894490776306943</v>
+        <v>4.894647244660094</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.894504890680713</v>
+        <v>4.894721245099745</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.891088817209817</v>
+        <v>4.891378342738221</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.875495476323485</v>
+        <v>4.87579437455733</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.852625126660225</v>
+        <v>4.852879034281871</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.826477214687386</v>
+        <v>4.826723768943628</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.817336291195816</v>
+        <v>4.817572487184481</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.78767970547995</v>
+        <v>4.787881073452486</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.759735661914376</v>
+        <v>4.759934897784763</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.751522238730244</v>
+        <v>4.749033957646995</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.751693885734014</v>
+        <v>4.752225788119594</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.746483147561973</v>
+        <v>4.748302481286419</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.742803654113176</v>
+        <v>4.745512181831399</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.736950360269963</v>
+        <v>4.74040873733727</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.722046041739827</v>
+        <v>4.727788193832593</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.704275265649402</v>
+        <v>4.7133363700499</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.691351616443439</v>
+        <v>4.703697440280288</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.675082964399962</v>
+        <v>4.690757458217949</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.662324503506781</v>
+        <v>4.683081839925046</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.647821512806264</v>
+        <v>4.674375178535959</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.641907839110415</v>
+        <v>4.677276800622169</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.647417623267318</v>
+        <v>4.688288293034976</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.683319553503778</v>
+        <v>4.733085384483036</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.674928212692953</v>
+        <v>4.758031203987971</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.708233639695985</v>
+        <v>4.808096237666262</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-08-12_20-33-19
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712855903354704</v>
+        <v>4.71285746658684</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711573001527986</v>
+        <v>4.711565690379212</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720065926544111</v>
+        <v>4.720057004619123</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706690030887003</v>
+        <v>4.70667156667664</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694033953995688</v>
+        <v>4.694015280216637</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678106679558706</v>
+        <v>4.6780878434066</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.67311514202461</v>
+        <v>4.673096261321311</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686191328885699</v>
+        <v>4.686172457388607</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702088482454078</v>
+        <v>4.70206583458241</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705398698974183</v>
+        <v>4.705383673388586</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694465484827679</v>
+        <v>4.694450160551107</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664477040408019</v>
+        <v>4.664460433518528</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649612013919445</v>
+        <v>4.649609644322182</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641292654226435</v>
+        <v>4.641286600079924</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636163044579632</v>
+        <v>4.636159156862262</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633844266888452</v>
+        <v>4.633835172233861</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637349589728541</v>
+        <v>4.637347506219321</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.63452082735583</v>
+        <v>4.634525972643685</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627833260035968</v>
+        <v>4.627848484286198</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.624109083074478</v>
+        <v>4.624125389126667</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.59946494134324</v>
+        <v>4.599481037569078</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.5801406263449</v>
+        <v>4.580175609631921</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.561723973799618</v>
+        <v>4.561780735933091</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.524156296742856</v>
+        <v>4.524239914562038</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.521840402473184</v>
+        <v>4.521959022295985</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.534862858668728</v>
+        <v>4.534993689985829</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.5537673103744</v>
+        <v>4.5539002541502</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.586551159452915</v>
+        <v>4.586699745679653</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.605888419591624</v>
+        <v>4.606075418100952</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.678994037216254</v>
+        <v>4.679208807827525</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.714824073994485</v>
+        <v>4.715051910816641</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.781275330146626</v>
+        <v>4.781486961355119</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.815302776713057</v>
+        <v>4.81542717494749</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.81300582781367</v>
+        <v>4.813126980778245</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.82220365415197</v>
+        <v>4.822323891319574</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.86256227386087</v>
+        <v>4.862573653482811</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855211575001626</v>
+        <v>4.855217615473622</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.851951887637293</v>
+        <v>4.851894675490656</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.829402363510717</v>
+        <v>4.829360474074398</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.837028928767579</v>
+        <v>4.836974206193359</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.889272469193548</v>
+        <v>4.88917626525444</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.916556850161502</v>
+        <v>4.916497910010555</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.925763496499107</v>
+        <v>4.925703969594553</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.915918209360245</v>
+        <v>4.915861752983016</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.896970241479591</v>
+        <v>4.896924661973425</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.894722255967744</v>
+        <v>4.894647244660094</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.89482506864784</v>
+        <v>4.894721245099745</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.891517212372903</v>
+        <v>4.891378342738221</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.87593770706129</v>
+        <v>4.87579437455733</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.853000713599274</v>
+        <v>4.852879034281871</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.826841787921884</v>
+        <v>4.826723768943628</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.817685513511865</v>
+        <v>4.817572487184481</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.787977311218771</v>
+        <v>4.787881073452486</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.760030279619814</v>
+        <v>4.759934897784763</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.74912764785495</v>
+        <v>4.751712393760768</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.752365440949818</v>
+        <v>4.751998023898523</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.748379464200715</v>
+        <v>4.74667214115712</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.746076516559754</v>
+        <v>4.744460016227569</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.741276309189209</v>
+        <v>4.73932096505856</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.729068318018635</v>
+        <v>4.725390515330996</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.715408931732989</v>
+        <v>4.709726117050837</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.706290975493142</v>
+        <v>4.698167418903656</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.693095299474997</v>
+        <v>4.682015084119501</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.685647967654939</v>
+        <v>4.670413175328749</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.677195343534132</v>
+        <v>4.6569976156656</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.679777806388994</v>
+        <v>4.651505988159358</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.689483981334678</v>
+        <v>4.655666348902199</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.731124355511843</v>
+        <v>4.6891980324386</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.751893778373498</v>
+        <v>4.684525950198852</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.789428017409994</v>
+        <v>4.713207969563305</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.737156767409995</v>
+        <v>4.718259184199558</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-08-12_20-35-37
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.71285746658684</v>
+        <v>4.712854384148416</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711565690379212</v>
+        <v>4.711580105379255</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720057004619123</v>
+        <v>4.720074597685915</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.70667156667664</v>
+        <v>4.70670797440489</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694015280216637</v>
+        <v>4.694052101199956</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.6780878434066</v>
+        <v>4.678124984551821</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673096261321311</v>
+        <v>4.67313349050572</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686172457388607</v>
+        <v>4.686209668937561</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.70206583458241</v>
+        <v>4.702110496134186</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705383673388586</v>
+        <v>4.705413304555261</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694450160551107</v>
+        <v>4.69448038044954</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664460433518528</v>
+        <v>4.664493182161545</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649609644322182</v>
+        <v>4.649614331327493</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641286600079924</v>
+        <v>4.641298549772891</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636159156862262</v>
+        <v>4.636166823286956</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633835172233861</v>
+        <v>4.633853108898519</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637347506219321</v>
+        <v>4.637351624709443</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634525972643685</v>
+        <v>4.634515829471178</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627848484286198</v>
+        <v>4.627818459092896</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.624125389126667</v>
+        <v>4.624093232660497</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599481037569078</v>
+        <v>4.599449296573527</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.580175609631921</v>
+        <v>4.580106652345037</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.561780735933091</v>
+        <v>4.561668861512033</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.524239914562038</v>
+        <v>4.524075092435588</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.521959022295985</v>
+        <v>4.521725194117121</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.534993689985829</v>
+        <v>4.534735764910435</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.5539002541502</v>
+        <v>4.553638143276833</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.586699745679653</v>
+        <v>4.586406762732529</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.606075418100952</v>
+        <v>4.605706584525801</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.679208807827525</v>
+        <v>4.678785207998901</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.715051910816641</v>
+        <v>4.714602543071656</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.781486961355119</v>
+        <v>4.781069420284056</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.81542717494749</v>
+        <v>4.815181751426712</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.813126980778245</v>
+        <v>4.812887928559447</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.822323891319574</v>
+        <v>4.822086606281117</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862573653482811</v>
+        <v>4.862551160853318</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855217615473622</v>
+        <v>4.855205648638783</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.851894675490656</v>
+        <v>4.852007519127758</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.829360474074398</v>
+        <v>4.829443052328933</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.836974206193359</v>
+        <v>4.837082106612412</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.88917626525444</v>
+        <v>4.889365993786115</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.916497910010555</v>
+        <v>4.916614082154158</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.925703969594553</v>
+        <v>4.925821311044922</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.915861752983016</v>
+        <v>4.91597310640635</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.896924661973425</v>
+        <v>4.897014552452664</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.894647244660094</v>
+        <v>4.894795234508227</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.894721245099745</v>
+        <v>4.894926142460742</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.891378342738221</v>
+        <v>4.891652362582835</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.87579437455733</v>
+        <v>4.876077180567793</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.852879034281871</v>
+        <v>4.853119068292514</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.826723768943628</v>
+        <v>4.826956497655476</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.817572487184481</v>
+        <v>4.817795349282546</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.787881073452486</v>
+        <v>4.788070755917024</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.759934897784763</v>
+        <v>4.760122993357458</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.751712393760768</v>
+        <v>4.749218851858179</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.751998023898523</v>
+        <v>4.752501749110236</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.74667214115712</v>
+        <v>4.748455023298625</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.744460016227569</v>
+        <v>4.746835388119507</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.73932096505856</v>
+        <v>4.74234812382649</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.725390515330996</v>
+        <v>4.730555641608123</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.709726117050837</v>
+        <v>4.717770498399565</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.698167418903656</v>
+        <v>4.708523212663061</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.682015084119501</v>
+        <v>4.695662648374732</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.670413175328749</v>
+        <v>4.688467512137426</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.6569976156656</v>
+        <v>4.680283356004441</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.651505988159358</v>
+        <v>4.682610695741992</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.655666348902199</v>
+        <v>4.691198168296835</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.6891980324386</v>
+        <v>4.730208201821</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.684525950198852</v>
+        <v>4.747989899594454</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.713207969563305</v>
+        <v>4.777241385464771</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.718259184199558</v>
+        <v>4.724970135464772</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-08-13_20-32-52
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712854384148416</v>
+        <v>4.712855903354704</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711580105379255</v>
+        <v>4.711573001527986</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720074597685915</v>
+        <v>4.720065926544111</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.70670797440489</v>
+        <v>4.706690030887003</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694052101199956</v>
+        <v>4.694033953995688</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678124984551821</v>
+        <v>4.678106679558706</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.67313349050572</v>
+        <v>4.67311514202461</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686209668937561</v>
+        <v>4.686191328885699</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702110496134186</v>
+        <v>4.702088482454078</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705413304555261</v>
+        <v>4.705398698974183</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.69448038044954</v>
+        <v>4.694465484827679</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664493182161545</v>
+        <v>4.664477040408019</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649614331327493</v>
+        <v>4.649612013919445</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641298549772891</v>
+        <v>4.641292654226435</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636166823286956</v>
+        <v>4.636163044579632</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633853108898519</v>
+        <v>4.633844266888452</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637351624709443</v>
+        <v>4.637349589728541</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634515829471178</v>
+        <v>4.63452082735583</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627818459092896</v>
+        <v>4.627833260035968</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.624093232660497</v>
+        <v>4.624109083074478</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599449296573527</v>
+        <v>4.59946494134324</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.580106652345037</v>
+        <v>4.5801406263449</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.561668861512033</v>
+        <v>4.561723973799618</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.524075092435588</v>
+        <v>4.524156296742856</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.521725194117121</v>
+        <v>4.521840402473184</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.534735764910435</v>
+        <v>4.534862858668728</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.553638143276833</v>
+        <v>4.5537673103744</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.586406762732529</v>
+        <v>4.586551159452915</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.605706584525801</v>
+        <v>4.605888419591624</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.678785207998901</v>
+        <v>4.678994037216254</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.714602543071656</v>
+        <v>4.714824073994485</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.781069420284056</v>
+        <v>4.781275330146626</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.815181751426712</v>
+        <v>4.815302776713057</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.812887928559447</v>
+        <v>4.81300582781367</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.822086606281117</v>
+        <v>4.82220365415197</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862551160853318</v>
+        <v>4.86256227386087</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855205648638783</v>
+        <v>4.855211575001626</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.852007519127758</v>
+        <v>4.851951887637293</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.829443052328933</v>
+        <v>4.829402363510717</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.837082106612412</v>
+        <v>4.837028928767579</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.889365993786115</v>
+        <v>4.889272469193548</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.916614082154158</v>
+        <v>4.916556850161502</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.925821311044922</v>
+        <v>4.925763496499107</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.91597310640635</v>
+        <v>4.915918209360245</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.897014552452664</v>
+        <v>4.896970241479591</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.894795234508227</v>
+        <v>4.894722255967744</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.894926142460742</v>
+        <v>4.89482506864784</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.891652362582835</v>
+        <v>4.891517212372903</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.876077180567793</v>
+        <v>4.87593770706129</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.853119068292514</v>
+        <v>4.853000713599274</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.826956497655476</v>
+        <v>4.826841787921884</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.817795349282546</v>
+        <v>4.817685513511865</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.788070755917024</v>
+        <v>4.787977311218771</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.760122993357458</v>
+        <v>4.760030279619814</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.749218851858179</v>
+        <v>4.751803575585807</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.752501749110236</v>
+        <v>4.752144472678436</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.748455023298625</v>
+        <v>4.746763734278757</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.746835388119507</v>
+        <v>4.745311997161117</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.74234812382649</v>
+        <v>4.740518425990204</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.730555641608123</v>
+        <v>4.7270182835653</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.717770498399565</v>
+        <v>4.712341204316703</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.708523212663061</v>
+        <v>4.701370976001961</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.695662648374732</v>
+        <v>4.685284461925105</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.688467512137426</v>
+        <v>4.674197615192202</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.680283356004441</v>
+        <v>4.661269624248312</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.682610695741992</v>
+        <v>4.655966191044334</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.691198168296835</v>
+        <v>4.659566959941598</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.730208201821</v>
+        <v>4.6920656004009</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.747989899594454</v>
+        <v>4.688783475708606</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.777241385464771</v>
+        <v>4.715644200129018</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.724970135464772</v>
+        <v>4.720333606695085</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-08-13_20-34-53
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712855903354704</v>
+        <v>4.712852907134048</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711573001527986</v>
+        <v>4.711587010624736</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720065926544111</v>
+        <v>4.720083028468686</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706690030887003</v>
+        <v>4.706725418942133</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694033953995688</v>
+        <v>4.694069743785596</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678106679558706</v>
+        <v>4.678142780533582</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.67311514202461</v>
+        <v>4.673151328948626</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686191328885699</v>
+        <v>4.686227499674366</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702088482454078</v>
+        <v>4.70213190187898</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705398698974183</v>
+        <v>4.705427507493312</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694465484827679</v>
+        <v>4.694494865148227</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664477040408019</v>
+        <v>4.664508878044651</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649612013919445</v>
+        <v>4.649616598119465</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641292654226435</v>
+        <v>4.641304292839184</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636163044579632</v>
+        <v>4.636170497506238</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633844266888452</v>
+        <v>4.633861708637639</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637349589728541</v>
+        <v>4.637353612761972</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.63452082735583</v>
+        <v>4.634510972758013</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627833260035968</v>
+        <v>4.627804064060729</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.624109083074478</v>
+        <v>4.624077819058792</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.59946494134324</v>
+        <v>4.599434084548101</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.5801406263449</v>
+        <v>4.580073644645431</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.561723973799618</v>
+        <v>4.561615328344136</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.524156296742856</v>
+        <v>4.523996198896978</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.521840402473184</v>
+        <v>4.52161325253785</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.534862858668728</v>
+        <v>4.534612251294011</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.5537673103744</v>
+        <v>4.553512594757063</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.586551159452915</v>
+        <v>4.586266381533545</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.605888419591624</v>
+        <v>4.605529702533609</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.678994037216254</v>
+        <v>4.678582077687856</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.714824073994485</v>
+        <v>4.714387060552296</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.781275330146626</v>
+        <v>4.780869003594383</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.815302776713057</v>
+        <v>4.815063964194965</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.81300582781367</v>
+        <v>4.812773154217027</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.82220365415197</v>
+        <v>4.821972623169046</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.86256227386087</v>
+        <v>4.862540305545373</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855211575001626</v>
+        <v>4.855199833878952</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.851951887637293</v>
+        <v>4.852061634501004</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.829402363510717</v>
+        <v>4.829482591323206</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.837028928767579</v>
+        <v>4.837133804072965</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.889272469193548</v>
+        <v>4.889456949307627</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.916556850161502</v>
+        <v>4.916669678833014</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.925763496499107</v>
+        <v>4.92587748566831</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.915918209360245</v>
+        <v>4.916026507509533</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.896970241479591</v>
+        <v>4.89705764677759</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.894722255967744</v>
+        <v>4.89486626139721</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.89482506864784</v>
+        <v>4.895024573684404</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.891517212372903</v>
+        <v>4.891783940099717</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.87593770706129</v>
+        <v>4.876212948319242</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.853000713599274</v>
+        <v>4.853234232494762</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.826841787921884</v>
+        <v>4.827068035153258</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.817685513511865</v>
+        <v>4.817902127500606</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.787977311218771</v>
+        <v>4.788161526776742</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.760030279619814</v>
+        <v>4.760213148105043</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.751803575585807</v>
+        <v>4.749307665445988</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.752144472678436</v>
+        <v>4.75263482735349</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.746763734278757</v>
+        <v>4.748529188932888</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.745311997161117</v>
+        <v>4.747537988564877</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.740518425990204</v>
+        <v>4.743336825069974</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.7270182835653</v>
+        <v>4.731902404291593</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.712341204316703</v>
+        <v>4.719958944140902</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.701370976001961</v>
+        <v>4.710545256384923</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.685284461925105</v>
+        <v>4.697980601987314</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.674197615192202</v>
+        <v>4.690992021889011</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.661269624248312</v>
+        <v>4.683040316435489</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.655966191044334</v>
+        <v>4.685119268345537</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.659566959941598</v>
+        <v>4.692657325154996</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.6920656004009</v>
+        <v>4.729262722138447</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.688783475708606</v>
+        <v>4.744516699375068</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.715644200129018</v>
+        <v>4.767522063913536</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.720333606695085</v>
+        <v>4.679853855699101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-08-14_20-34-27
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712852907134048</v>
+        <v>4.712851470578128</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711587010624736</v>
+        <v>4.711593725477015</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720083028468686</v>
+        <v>4.720091228746907</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706725418942133</v>
+        <v>4.706742385020389</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694069743785596</v>
+        <v>4.694086902505232</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678142780533582</v>
+        <v>4.678160088437575</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673151328948626</v>
+        <v>4.673168678321706</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686227499674366</v>
+        <v>4.686244842014795</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.70213190187898</v>
+        <v>4.702152724515812</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705427507493312</v>
+        <v>4.705441324206276</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694494865148227</v>
+        <v>4.694508955690935</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664508878044651</v>
+        <v>4.664524146273761</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649616598119465</v>
+        <v>4.64961881581495</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641304292839184</v>
+        <v>4.64130988923613</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636170497506238</v>
+        <v>4.636174071512754</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633861708637639</v>
+        <v>4.633870075919665</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637353612761972</v>
+        <v>4.637355555421442</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634510972758013</v>
+        <v>4.634506251330331</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627804064060729</v>
+        <v>4.627790058482666</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.624077819058792</v>
+        <v>4.624062824465991</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599434084548101</v>
+        <v>4.599419287574101</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.580073644645431</v>
+        <v>4.580041562662499</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.561615328344136</v>
+        <v>4.561563307546296</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.523996198896978</v>
+        <v>4.523919519120168</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.52161325253785</v>
+        <v>4.521504441093176</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.534612251294011</v>
+        <v>4.534492169094606</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.553512594757063</v>
+        <v>4.553390515387446</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.586266381533545</v>
+        <v>4.586129851334114</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.605529702533609</v>
+        <v>4.605357574488753</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.678582077687856</v>
+        <v>4.678384416776968</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.714387060552296</v>
+        <v>4.714177382732943</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.780869003594383</v>
+        <v>4.780673863838269</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.815063964194965</v>
+        <v>4.814949287198139</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.812773154217027</v>
+        <v>4.812661382668097</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.821972623169046</v>
+        <v>4.821861586640436</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862540305545373</v>
+        <v>4.862529699393626</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855199833878952</v>
+        <v>4.855194128235032</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.852061634501004</v>
+        <v>4.852114294833448</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.829482591323206</v>
+        <v>4.829521028467236</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.837133804072965</v>
+        <v>4.837184081977693</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.889456949307627</v>
+        <v>4.889545440070393</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.916669678833014</v>
+        <v>4.9167237089769</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.92587748566831</v>
+        <v>4.925932088797786</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.916026507509533</v>
+        <v>4.916078472686516</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.89705764677759</v>
+        <v>4.89709957356622</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.89486626139721</v>
+        <v>4.894935413513424</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.895024573684404</v>
+        <v>4.895120464005851</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.891783940099717</v>
+        <v>4.891912084076088</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.876212948319242</v>
+        <v>4.876345155578422</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.853234232494762</v>
+        <v>4.853346333234477</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.827068035153258</v>
+        <v>4.827176529977522</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.817902127500606</v>
+        <v>4.818005973890452</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.788161526776742</v>
+        <v>4.788249736369137</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.760213148105043</v>
+        <v>4.760300847169517</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.749307665445988</v>
+        <v>4.749394179651492</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.75263482735349</v>
+        <v>4.752764785473518</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.748529188932888</v>
+        <v>4.748601991242907</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.747537988564877</v>
+        <v>4.74796433989557</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.743336825069974</v>
+        <v>4.743989859224684</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.731902404291593</v>
+        <v>4.732803457247835</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.719958944140902</v>
+        <v>4.721336610528667</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.710545256384923</v>
+        <v>4.711843985737396</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.697980601987314</v>
+        <v>4.699553168355569</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.690992021889011</v>
+        <v>4.692704856764033</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.683040316435489</v>
+        <v>4.68493332772487</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.685119268345537</v>
+        <v>4.686739245974933</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.692657325154996</v>
+        <v>4.693204565887342</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.729262722138447</v>
+        <v>4.727426248251566</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.744516699375068</v>
+        <v>4.740180964990985</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.767522063913536</v>
+        <v>4.757850755801613</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.679853855699101</v>
+        <v>4.675866176588413</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-08-15_11-59-47
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712851470578128</v>
+        <v>4.712850072840855</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711593725477015</v>
+        <v>4.711600257702102</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720091228746907</v>
+        <v>4.72009920784377</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706742385020389</v>
+        <v>4.706758892051553</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694086902505232</v>
+        <v>4.694103596989277</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678160088437575</v>
+        <v>4.678176928065366</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673168678321706</v>
+        <v>4.673185558459836</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686244842014795</v>
+        <v>4.686261715747787</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702152724515812</v>
+        <v>4.702172987538977</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705441324206276</v>
+        <v>4.705454770231763</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694508955690935</v>
+        <v>4.694522667945176</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664524146273761</v>
+        <v>4.664539004086603</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.64961881581495</v>
+        <v>4.64962098588142</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.64130988923613</v>
+        <v>4.641315344484607</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636174071512754</v>
+        <v>4.636177549351649</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633870075919665</v>
+        <v>4.633878220035932</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637355555421442</v>
+        <v>4.637357454161338</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634506251330331</v>
+        <v>4.634501659624231</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627790058482666</v>
+        <v>4.627776426778835</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.624062824465991</v>
+        <v>4.62404823203282</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599419287574101</v>
+        <v>4.599404888909291</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.580041562662499</v>
+        <v>4.580010368050593</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.561563307546296</v>
+        <v>4.561512736070435</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.523919519120168</v>
+        <v>4.523844961440735</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.521504441093176</v>
+        <v>4.521398630638112</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.534492169094606</v>
+        <v>4.534375377689332</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.553390515387446</v>
+        <v>4.553271763828453</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.586129851334114</v>
+        <v>4.585997016443295</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.605357574488753</v>
+        <v>4.605190011769334</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.678384416776968</v>
+        <v>4.678192007886779</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.714177382732943</v>
+        <v>4.713973278793846</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.780673863838269</v>
+        <v>4.780483795942621</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.814949287198139</v>
+        <v>4.81483759923433</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.812661382668097</v>
+        <v>4.81255249804899</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.821861586640436</v>
+        <v>4.821753384483987</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862529699393626</v>
+        <v>4.862519334208626</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855194128235032</v>
+        <v>4.855188529245329</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.852114294833448</v>
+        <v>4.85216555796787</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.829521028467236</v>
+        <v>4.829558409107026</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.837184081977693</v>
+        <v>4.837232997874872</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.889545440070393</v>
+        <v>4.889631564820823</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.9167237089769</v>
+        <v>4.916776237577539</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.925932088797786</v>
+        <v>4.925985185126109</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.916078472686516</v>
+        <v>4.916129058802522</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.89709957356622</v>
+        <v>4.897140379338916</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.894935413513424</v>
+        <v>4.895002763770238</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.895120464005851</v>
+        <v>4.895213909993988</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.891912084076088</v>
+        <v>4.892036926565884</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.876345155578422</v>
+        <v>4.876473940139365</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.853346333234477</v>
+        <v>4.853455490898698</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.827176529977522</v>
+        <v>4.827282104742206</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.818005973890452</v>
+        <v>4.818107007387359</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.788249736369137</v>
+        <v>4.788335491063402</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.760300847169517</v>
+        <v>4.760386188433301</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.749394179651492</v>
+        <v>4.749478481036193</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.752764785473518</v>
+        <v>4.75289172855345</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.748601991242907</v>
+        <v>4.748673460081834</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.74796433989557</v>
+        <v>4.749113126765234</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.743989859224684</v>
+        <v>4.745458388260237</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.732803457247835</v>
+        <v>4.734748438368303</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.721336610528667</v>
+        <v>4.723931574724329</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.711843985737396</v>
+        <v>4.714542238442958</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.699553168355569</v>
+        <v>4.70267981762345</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.692704856764033</v>
+        <v>4.696078359622001</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.68493332772487</v>
+        <v>4.688380422761883</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.686739245974933</v>
+        <v>4.689734445450494</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.693204565887342</v>
+        <v>4.694974313600611</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.727426248251566</v>
+        <v>4.727006783167683</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.740180964990985</v>
+        <v>4.737987751107324</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.757850755801613</v>
+        <v>4.752375845206604</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.675866176588413</v>
+        <v>4.679695834640982</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-08-17_20-34-17
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712850072840855</v>
+        <v>4.712848712369858</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711600257702102</v>
+        <v>4.711606614649382</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.72009920784377</v>
+        <v>4.720106974586502</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706758892051553</v>
+        <v>4.706774958411754</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694103596989277</v>
+        <v>4.694119845820756</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678176928065366</v>
+        <v>4.678193318161983</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673185558459836</v>
+        <v>4.67320198813994</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686261715747787</v>
+        <v>4.686278139607769</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702172987538977</v>
+        <v>4.702192713197964</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705454770231763</v>
+        <v>4.705467860285254</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694522667945176</v>
+        <v>4.694536016938301</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664539004086603</v>
+        <v>4.664553467807045</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.64962098588142</v>
+        <v>4.649623109735726</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641315344484607</v>
+        <v>4.641320663833311</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636177549351649</v>
+        <v>4.636180934853234</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633878220035932</v>
+        <v>4.633886149789561</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637357454161338</v>
+        <v>4.637359310396051</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634501659624231</v>
+        <v>4.634497192376229</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627776426778835</v>
+        <v>4.62776315418871</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.62404823203282</v>
+        <v>4.624034025801064</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599404888909291</v>
+        <v>4.599390872699122</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.580010368050593</v>
+        <v>4.579980024550037</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.561512736070435</v>
+        <v>4.561463554317464</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.523844961440735</v>
+        <v>4.523772439174714</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.521398630638112</v>
+        <v>4.521295699018835</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.534375377689332</v>
+        <v>4.534261744014464</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.553271763828453</v>
+        <v>4.553156206290518</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.585997016443295</v>
+        <v>4.585867729418695</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.605190011769334</v>
+        <v>4.60502683557606</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.678192007886779</v>
+        <v>4.678004644976212</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.713973278793846</v>
+        <v>4.713774529960975</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.780483795942621</v>
+        <v>4.780298605291433</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.81483759923433</v>
+        <v>4.814728785298064</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.81255249804899</v>
+        <v>4.812446390357074</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.821753384483987</v>
+        <v>4.821647910083186</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862519334208626</v>
+        <v>4.862509202138289</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855188529245329</v>
+        <v>4.855183034478822</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.85216555796787</v>
+        <v>4.852215478724398</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.829558409107026</v>
+        <v>4.829594776138078</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.837232997874872</v>
+        <v>4.837280606250286</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.889631564820823</v>
+        <v>4.889715417105377</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.916776237577539</v>
+        <v>4.916827326095623</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.925985185126109</v>
+        <v>4.926036835860572</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.916129058802522</v>
+        <v>4.916178319774335</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.897140379338916</v>
+        <v>4.89718010819216</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.895002763770238</v>
+        <v>4.895068381366745</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.895213909993988</v>
+        <v>4.895305003415402</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.892036926565884</v>
+        <v>4.892158592969072</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.876473940139365</v>
+        <v>4.876599432799646</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.853455490898698</v>
+        <v>4.8535618196606</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.827282104742206</v>
+        <v>4.827384875571717</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.818107007387359</v>
+        <v>4.818205340588907</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.788335491063402</v>
+        <v>4.788418891446134</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.760386188433301</v>
+        <v>4.760469264701658</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.749478481036193</v>
+        <v>4.749560651954941</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.75289172855345</v>
+        <v>4.753015757200346</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.748673460081834</v>
+        <v>4.748743624955519</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.749113126765234</v>
+        <v>4.750186796411636</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.745458388260237</v>
+        <v>4.746824492527086</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.734748438368303</v>
+        <v>4.736517227688378</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.723931574724329</v>
+        <v>4.726316474349285</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.714542238442958</v>
+        <v>4.717013261487937</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.70267981762345</v>
+        <v>4.705549771458724</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.696078359622001</v>
+        <v>4.699161619790859</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.688380422761883</v>
+        <v>4.691521856621325</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.689734445450494</v>
+        <v>4.692444751310342</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.694974313600611</v>
+        <v>4.696525831654833</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.727006783167683</v>
+        <v>4.726526106099071</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.737987751107324</v>
+        <v>4.735935364510794</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.752375845206604</v>
+        <v>4.747630757433394</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.679695834640982</v>
+        <v>4.681829427098798</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-08-18_20-33-36
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712852907134048</v>
+        <v>4.71284738769445</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711587010624736</v>
+        <v>4.711612803279171</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720083028468686</v>
+        <v>4.720114537338898</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706725418942133</v>
+        <v>4.706790601509503</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694069743785596</v>
+        <v>4.69413566660422</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678142780533582</v>
+        <v>4.678209276485431</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673151328948626</v>
+        <v>4.673217985150582</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686227499674366</v>
+        <v>4.686294131343949</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.70213190187898</v>
+        <v>4.702211922578774</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705427507493312</v>
+        <v>4.705480608313755</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694494865148227</v>
+        <v>4.694549016912365</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664508878044651</v>
+        <v>4.664567552904854</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649616598119465</v>
+        <v>4.649625188745627</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641304292839184</v>
+        <v>4.64132585227522</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636170497506238</v>
+        <v>4.636184231647041</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633861708637639</v>
+        <v>4.633893873527061</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637353612761972</v>
+        <v>4.637361125483475</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634510972758013</v>
+        <v>4.634492844603279</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627804064060729</v>
+        <v>4.627750226717991</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.624077819058792</v>
+        <v>4.624020190645455</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599434084548101</v>
+        <v>4.599377223918714</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.580073644645431</v>
+        <v>4.579950497847379</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.561615328344136</v>
+        <v>4.561415705905082</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.523996198896978</v>
+        <v>4.523701870285565</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.52161325253785</v>
+        <v>4.521195530606983</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.534612251294011</v>
+        <v>4.534151142065578</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.553512594757063</v>
+        <v>4.553043716038138</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.586266381533545</v>
+        <v>4.585741850529415</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.605529702533609</v>
+        <v>4.604867876302727</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.678582077687856</v>
+        <v>4.677822132614808</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.714387060552296</v>
+        <v>4.71358092873242</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.780869003594383</v>
+        <v>4.780118107069795</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.815063964194965</v>
+        <v>4.814622736190631</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.812773154217027</v>
+        <v>4.812342955086349</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.821972623169046</v>
+        <v>4.821545062073984</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862540305545373</v>
+        <v>4.862499295652059</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855199833878952</v>
+        <v>4.855177641539498</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.852061634501004</v>
+        <v>4.852264109095198</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.829482591323206</v>
+        <v>4.829630170168459</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.837133804072965</v>
+        <v>4.837326958727842</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.889456949307627</v>
+        <v>4.889797085608054</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.916669678833014</v>
+        <v>4.916877032696465</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.92587748566831</v>
+        <v>4.926087098953507</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.916026507509533</v>
+        <v>4.916226306757959</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.89705764677759</v>
+        <v>4.897218801953414</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.89486626139721</v>
+        <v>4.895132332020092</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.895024573684404</v>
+        <v>4.895393831527231</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.891783940099717</v>
+        <v>4.892277202443478</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.876212948319242</v>
+        <v>4.876721757797381</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.853234232494762</v>
+        <v>4.853665427874518</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.827068035153258</v>
+        <v>4.827484952523916</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.817902127500606</v>
+        <v>4.818301080170961</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.788161526776742</v>
+        <v>4.788500032707303</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.760213148105043</v>
+        <v>4.760550164024023</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.751978656985716</v>
+        <v>4.749640770802789</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.752426786166637</v>
+        <v>4.753136967767404</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.746941367116193</v>
+        <v>4.748812514971819</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.745892027698307</v>
+        <v>4.750190415350391</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.743394670093702</v>
+        <v>4.74846749857153</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.731168680557309</v>
+        <v>4.738832844934851</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.717826806055154</v>
+        <v>4.728992825661026</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.707777479758342</v>
+        <v>4.720288375699575</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.693260505025545</v>
+        <v>4.709519647727154</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.683099989272336</v>
+        <v>4.702966384009123</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.671283661682669</v>
+        <v>4.695430464800573</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.666571717298302</v>
+        <v>4.696024627109013</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.66997460401684</v>
+        <v>4.699726805134448</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.701283335358643</v>
+        <v>4.727492167916944</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.701234642272976</v>
+        <v>4.735866920534346</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.727516050204862</v>
+        <v>4.74568461864464</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.738894310280537</v>
+        <v>4.695015099371291</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.791165560280537</v>
+        <v>4.747286349371291</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-08-19_20-33-08
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.71284738769445</v>
+        <v>4.712851470578128</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711612803279171</v>
+        <v>4.711593725477015</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720114537338898</v>
+        <v>4.720091228746907</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706790601509503</v>
+        <v>4.706742385020389</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.69413566660422</v>
+        <v>4.694086902505232</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678209276485431</v>
+        <v>4.678160088437575</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673217985150582</v>
+        <v>4.673168678321706</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686294131343949</v>
+        <v>4.686244842014795</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702211922578774</v>
+        <v>4.702152724515812</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705480608313755</v>
+        <v>4.705441324206276</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694549016912365</v>
+        <v>4.694508955690935</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664567552904854</v>
+        <v>4.664524146273761</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649625188745627</v>
+        <v>4.64961881581495</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.64132585227522</v>
+        <v>4.64130988923613</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636184231647041</v>
+        <v>4.636174071512754</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633893873527061</v>
+        <v>4.633870075919665</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637361125483475</v>
+        <v>4.637355555421442</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634492844603279</v>
+        <v>4.634506251330331</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627750226717991</v>
+        <v>4.627790058482666</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.624020190645455</v>
+        <v>4.624062824465991</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599377223918714</v>
+        <v>4.599419287574101</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.579950497847379</v>
+        <v>4.580041562662499</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.561415705905082</v>
+        <v>4.561563307546296</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.523701870285565</v>
+        <v>4.523919519120168</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.521195530606983</v>
+        <v>4.521504441093176</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.534151142065578</v>
+        <v>4.534492169094606</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.553043716038138</v>
+        <v>4.553390515387446</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.585741850529415</v>
+        <v>4.586129851334114</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.604867876302727</v>
+        <v>4.605357574488753</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.677822132614808</v>
+        <v>4.678384416776968</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.71358092873242</v>
+        <v>4.714177382732943</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.780118107069795</v>
+        <v>4.780673863838269</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.814622736190631</v>
+        <v>4.814949287198139</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.812342955086349</v>
+        <v>4.812661382668097</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.821545062073984</v>
+        <v>4.821861586640436</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862499295652059</v>
+        <v>4.862529699393626</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855177641539498</v>
+        <v>4.855194128235032</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.852264109095198</v>
+        <v>4.852114294833448</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.829630170168459</v>
+        <v>4.829521028467236</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.837326958727842</v>
+        <v>4.837184081977693</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.889797085608054</v>
+        <v>4.889545440070393</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.916877032696465</v>
+        <v>4.9167237089769</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.926087098953507</v>
+        <v>4.925932088797786</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.916226306757959</v>
+        <v>4.916078472686516</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.897218801953414</v>
+        <v>4.89709957356622</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.895132332020092</v>
+        <v>4.894935413513424</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.895393831527231</v>
+        <v>4.895120464005851</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.892277202443478</v>
+        <v>4.891912084076088</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.876721757797381</v>
+        <v>4.876345155578422</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.853665427874518</v>
+        <v>4.853346333234477</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.827484952523916</v>
+        <v>4.827176529977522</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.818301080170961</v>
+        <v>4.818005973890452</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.788500032707303</v>
+        <v>4.788249736369137</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.760550164024023</v>
+        <v>4.760300847169517</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.749640770802789</v>
+        <v>4.752062744734657</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.753136967767404</v>
+        <v>4.752562895957204</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.748812514971819</v>
+        <v>4.747027504645599</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.750190415350391</v>
+        <v>4.745919257548858</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.74846749857153</v>
+        <v>4.744928792332303</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.738832844934851</v>
+        <v>4.733509878653373</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.728992825661026</v>
+        <v>4.720670440586998</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.720288375699575</v>
+        <v>4.711387613364067</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.709519647727154</v>
+        <v>4.698030737772678</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.702966384009123</v>
+        <v>4.688042701126724</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.695430464800573</v>
+        <v>4.676830937534136</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.696024627109013</v>
+        <v>4.672502716274133</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.699726805134448</v>
+        <v>4.676242146803352</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.727492167916944</v>
+        <v>4.707261384746026</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.735866920534346</v>
+        <v>4.708924599413353</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.74568461864464</v>
+        <v>4.735658824633502</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.695015099371291</v>
+        <v>4.750486431923036</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.747286349371291</v>
+        <v>4.802757681923035</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-08-19_20-37-07
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712851470578128</v>
+        <v>4.712846097420315</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711593725477015</v>
+        <v>4.711618830188129</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720091228746907</v>
+        <v>4.720121904031337</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706742385020389</v>
+        <v>4.706805837848545</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694086902505232</v>
+        <v>4.694151076029293</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678160088437575</v>
+        <v>4.678224819870794</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673168678321706</v>
+        <v>4.67323356635613</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686244842014795</v>
+        <v>4.68630970778423</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702152724515812</v>
+        <v>4.702230635678957</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705441324206276</v>
+        <v>4.705493027545288</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694508955690935</v>
+        <v>4.694561681374751</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664524146273761</v>
+        <v>4.664581274050811</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.64961881581495</v>
+        <v>4.649627224231333</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.64130988923613</v>
+        <v>4.641330914562894</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636174071512754</v>
+        <v>4.636187443174827</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633870075919665</v>
+        <v>4.63390139916755</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637355555421442</v>
+        <v>4.637362900727519</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634506251330331</v>
+        <v>4.634488611584377</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627790058482666</v>
+        <v>4.627737631089568</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.624062824465991</v>
+        <v>4.624006712220047</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599419287574101</v>
+        <v>4.59936392831934</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.580041562662499</v>
+        <v>4.57992175544671</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.561563307546296</v>
+        <v>4.561369137454071</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.523919519120168</v>
+        <v>4.523633177077492</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.521504441093176</v>
+        <v>4.521098015870626</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.534492169094606</v>
+        <v>4.534043452436739</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.553390515387446</v>
+        <v>4.552934172932449</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.586129851334114</v>
+        <v>4.585619247260254</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.605357574488753</v>
+        <v>4.604712972954394</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.678384416776968</v>
+        <v>4.677644285310148</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.714177382732943</v>
+        <v>4.713392278163496</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.780673863838269</v>
+        <v>4.779942125656504</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.814949287198139</v>
+        <v>4.814519348159346</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.812661382668097</v>
+        <v>4.812242092889782</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.821861586640436</v>
+        <v>4.821444744027136</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862529699393626</v>
+        <v>4.862489607525831</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855194128235032</v>
+        <v>4.855172348069871</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.852114294833448</v>
+        <v>4.852311498424342</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.829521028467236</v>
+        <v>4.829664629669033</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.837184081977693</v>
+        <v>4.837372104254654</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.889545440070393</v>
+        <v>4.889876654461964</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.9167237089769</v>
+        <v>4.916925412467084</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.925932088797786</v>
+        <v>4.926136029314856</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.916078472686516</v>
+        <v>4.916273068322199</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.89709957356622</v>
+        <v>4.897256500324331</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.894935413513424</v>
+        <v>4.895194678180704</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.895120464005851</v>
+        <v>4.895480477349015</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.891912084076088</v>
+        <v>4.892392868286545</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.876345155578422</v>
+        <v>4.876841033215998</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.853346333234477</v>
+        <v>4.853766418441269</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.827176529977522</v>
+        <v>4.827582439980519</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.818005973890452</v>
+        <v>4.818394327271329</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.788249736369137</v>
+        <v>4.788579004995858</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.760300847169517</v>
+        <v>4.760628969991527</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.752062744734657</v>
+        <v>4.74971891224512</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.752562895957204</v>
+        <v>4.75325545256425</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.747027504645599</v>
+        <v>4.748880158798864</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.745919257548858</v>
+        <v>4.750194427527852</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.744928792332303</v>
+        <v>4.749664322809723</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.733509878653373</v>
+        <v>4.74056909368574</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.720670440586998</v>
+        <v>4.730937027714708</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.711387613364067</v>
+        <v>4.722564104238951</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.698030737772678</v>
+        <v>4.712036404659479</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.688042701126724</v>
+        <v>4.705623623893354</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.676830937534136</v>
+        <v>4.698077739691806</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.672502716274133</v>
+        <v>4.698240984945802</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.676242146803352</v>
+        <v>4.701423453518421</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.707261384746026</v>
+        <v>4.726666653004997</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.708924599413353</v>
+        <v>4.733518309151404</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.735658824633502</v>
+        <v>4.741001003302543</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.750486431923036</v>
+        <v>4.702120544544628</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.802757681923035</v>
+        <v>4.75130387934888</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-08-20_20-33-27
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712846097420315</v>
+        <v>4.712850072840855</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711618830188129</v>
+        <v>4.711600257702102</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720121904031337</v>
+        <v>4.72009920784377</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706805837848545</v>
+        <v>4.706758892051553</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694151076029293</v>
+        <v>4.694103596989277</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678224819870794</v>
+        <v>4.678176928065366</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.67323356635613</v>
+        <v>4.673185558459836</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.68630970778423</v>
+        <v>4.686261715747787</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702230635678957</v>
+        <v>4.702172987538977</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705493027545288</v>
+        <v>4.705454770231763</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694561681374751</v>
+        <v>4.694522667945176</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664581274050811</v>
+        <v>4.664539004086603</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649627224231333</v>
+        <v>4.64962098588142</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641330914562894</v>
+        <v>4.641315344484607</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636187443174827</v>
+        <v>4.636177549351649</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.63390139916755</v>
+        <v>4.633878220035932</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637362900727519</v>
+        <v>4.637357454161338</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634488611584377</v>
+        <v>4.634501659624231</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627737631089568</v>
+        <v>4.627776426778835</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.624006712220047</v>
+        <v>4.62404823203282</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.59936392831934</v>
+        <v>4.599404888909291</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.57992175544671</v>
+        <v>4.580010368050593</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.561369137454071</v>
+        <v>4.561512736070435</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.523633177077492</v>
+        <v>4.523844961440735</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.521098015870626</v>
+        <v>4.521398630638112</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.534043452436739</v>
+        <v>4.534375377689332</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.552934172932449</v>
+        <v>4.553271763828453</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.585619247260254</v>
+        <v>4.585997016443295</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.604712972954394</v>
+        <v>4.605190011769334</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.677644285310148</v>
+        <v>4.678192007886779</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.713392278163496</v>
+        <v>4.713973278793846</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.779942125656504</v>
+        <v>4.780483795942621</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.814519348159346</v>
+        <v>4.81483759923433</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.812242092889782</v>
+        <v>4.81255249804899</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.821444744027136</v>
+        <v>4.821753384483987</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862489607525831</v>
+        <v>4.862519334208626</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855172348069871</v>
+        <v>4.855188529245329</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.852311498424342</v>
+        <v>4.85216555796787</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.829664629669033</v>
+        <v>4.829558409107026</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.837372104254654</v>
+        <v>4.837232997874872</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.889876654461964</v>
+        <v>4.889631564820823</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.916925412467084</v>
+        <v>4.916776237577539</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.926136029314856</v>
+        <v>4.925985185126109</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.916273068322199</v>
+        <v>4.916129058802522</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.897256500324331</v>
+        <v>4.897140379338916</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.895194678180704</v>
+        <v>4.895002763770238</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.895480477349015</v>
+        <v>4.895213909993988</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.892392868286545</v>
+        <v>4.892036926565884</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.876841033215998</v>
+        <v>4.876473940139365</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.853766418441269</v>
+        <v>4.853455490898698</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.827582439980519</v>
+        <v>4.827282104742206</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.818394327271329</v>
+        <v>4.818107007387359</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.788579004995858</v>
+        <v>4.788335491063402</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.760628969991527</v>
+        <v>4.760386188433301</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.74971891224512</v>
+        <v>4.752144648104572</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.75325545256425</v>
+        <v>4.752695795473572</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.748880158798864</v>
+        <v>4.747111919343624</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.750194427527852</v>
+        <v>4.745946318992313</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.749664322809723</v>
+        <v>4.746968211529135</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.74056909368574</v>
+        <v>4.736413654311963</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.730937027714708</v>
+        <v>4.724252960417298</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.722564104238951</v>
+        <v>4.715885370662664</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.712036404659479</v>
+        <v>4.703225719802663</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.705623623893354</v>
+        <v>4.693831743993091</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.698077739691806</v>
+        <v>4.683291100953552</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.698240984945802</v>
+        <v>4.679435227439867</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.701423453518421</v>
+        <v>4.683624816905992</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.726666653004997</v>
+        <v>4.71475169548934</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.733518309151404</v>
+        <v>4.718296981663894</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.741001003302543</v>
+        <v>4.74613316679909</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.702120544544628</v>
+        <v>4.765163164641804</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.75130387934888</v>
+        <v>4.819719079057368</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-08-20_20-36-46
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712850072840855</v>
+        <v>4.712844840224624</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711600257702102</v>
+        <v>4.711624701632696</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.72009920784377</v>
+        <v>4.720129082188484</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706758892051553</v>
+        <v>4.706820683085859</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694103596989277</v>
+        <v>4.694166089929327</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678176928065366</v>
+        <v>4.678239964289413</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673185558459836</v>
+        <v>4.673248747755991</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686261715747787</v>
+        <v>4.686324884894194</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702172987538977</v>
+        <v>4.702248871476916</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705454770231763</v>
+        <v>4.705505130534636</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694522667945176</v>
+        <v>4.694574023144921</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664539004086603</v>
+        <v>4.664594645167623</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.64962098588142</v>
+        <v>4.649629217467064</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641315344484607</v>
+        <v>4.641335855222693</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636177549351649</v>
+        <v>4.636190572702553</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633878220035932</v>
+        <v>4.633908734229723</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637357454161338</v>
+        <v>4.637364637380522</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634501659624231</v>
+        <v>4.634484488843593</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627776426778835</v>
+        <v>4.627725354698198</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.62404823203282</v>
+        <v>4.62399357690869</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599404888909291</v>
+        <v>4.599350972378991</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.580010368050593</v>
+        <v>4.57989376655106</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.561512736070435</v>
+        <v>4.561323798391345</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.523844961440735</v>
+        <v>4.523566285912659</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.521398630638112</v>
+        <v>4.521003050978553</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.534375377689332</v>
+        <v>4.533938561895234</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.553271763828453</v>
+        <v>4.552827463008827</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.585997016443295</v>
+        <v>4.585499793853546</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.605190011769334</v>
+        <v>4.604561972609049</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.678192007886779</v>
+        <v>4.677470926885665</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.713973278793846</v>
+        <v>4.713208391205432</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.780483795942621</v>
+        <v>4.779770494061145</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.81483759923433</v>
+        <v>4.814418522563294</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.81255249804899</v>
+        <v>4.812143709266119</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.821753384483987</v>
+        <v>4.821346864153186</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862519334208626</v>
+        <v>4.862480130827599</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855188529245329</v>
+        <v>4.855167151753793</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.85216555796787</v>
+        <v>4.852357693574106</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.829558409107026</v>
+        <v>4.829698191112037</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.837232997874872</v>
+        <v>4.837416089271967</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.889631564820823</v>
+        <v>4.889954203537254</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.916776237577539</v>
+        <v>4.916972517616423</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.925985185126109</v>
+        <v>4.926183679008323</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.916129058802522</v>
+        <v>4.916318650609378</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.897140379338916</v>
+        <v>4.897293241013316</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.895002763770238</v>
+        <v>4.895255479231791</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.895213909993988</v>
+        <v>4.895565019915264</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.892036926565884</v>
+        <v>4.892505698289563</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.876473940139365</v>
+        <v>4.876957371359505</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.853455490898698</v>
+        <v>4.853864889146354</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.827282104742206</v>
+        <v>4.827677437007777</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.818107007387359</v>
+        <v>4.818485177844041</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.788335491063402</v>
+        <v>4.788655893747689</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.760386188433301</v>
+        <v>4.760705762012693</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.752144648104572</v>
+        <v>4.749795147432301</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.752695795473572</v>
+        <v>4.753371300055935</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.747111919343624</v>
+        <v>4.748946584631105</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.745946318992313</v>
+        <v>4.750198801973537</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.746968211529135</v>
+        <v>4.751349863142135</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.736413654311963</v>
+        <v>4.742903062057859</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.724252960417298</v>
+        <v>4.733709728677135</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.715885370662664</v>
+        <v>4.725846346605833</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.703225719802663</v>
+        <v>4.715451920381577</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.693831743993091</v>
+        <v>4.709323577474668</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.683291100953552</v>
+        <v>4.701913577529641</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.679435227439867</v>
+        <v>4.701838693884852</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.683624816905992</v>
+        <v>4.704743353893174</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.71475169548934</v>
+        <v>4.728228805999112</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.718296981663894</v>
+        <v>4.734494109735509</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.74613316679909</v>
+        <v>4.740934336199333</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.765163164641804</v>
+        <v>4.711767134972384</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.819719079057368</v>
+        <v>4.759808954483865</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-08-21_21-18-32
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712844840224624</v>
+        <v>4.712843614851505</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711624701632696</v>
+        <v>4.711630423550748</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720129082188484</v>
+        <v>4.720136078954903</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706820683085859</v>
+        <v>4.706835152085264</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694166089929327</v>
+        <v>4.694180723335615</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678239964289413</v>
+        <v>4.678254724903558</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673248747755991</v>
+        <v>4.67326354453935</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686324884894194</v>
+        <v>4.686339677831633</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702248871476916</v>
+        <v>4.702266647995987</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705505130534636</v>
+        <v>4.705516929205602</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694574023144921</v>
+        <v>4.694586054397642</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664594645167623</v>
+        <v>4.664607679476996</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649629217467064</v>
+        <v>4.649631169682602</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641335855222693</v>
+        <v>4.641340678568007</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636190572702553</v>
+        <v>4.636193623331474</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633908734229723</v>
+        <v>4.633915885856843</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637364637380522</v>
+        <v>4.63736633664554</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634484488843593</v>
+        <v>4.634480472134383</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627725354698198</v>
+        <v>4.627713385568569</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.62399357690869</v>
+        <v>4.623980771779213</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599350972378991</v>
+        <v>4.599338343256662</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.57989376655106</v>
+        <v>4.57986650195293</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.561323798391345</v>
+        <v>4.561279640768287</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.523566285912659</v>
+        <v>4.523501126950199</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.521003050978553</v>
+        <v>4.520910537434944</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.533938561895234</v>
+        <v>4.533836362988693</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.552827463008827</v>
+        <v>4.552723478086444</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.585499793853546</v>
+        <v>4.585383370885342</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.604561972609049</v>
+        <v>4.604414729919091</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.677470926885665</v>
+        <v>4.677301889904502</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.713208391205432</v>
+        <v>4.713029090093043</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.779770494061145</v>
+        <v>4.779603053401912</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.814418522563294</v>
+        <v>4.814320165563305</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.812143709266119</v>
+        <v>4.812047714269141</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.821346864153186</v>
+        <v>4.821251335028221</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862480130827599</v>
+        <v>4.862470858903805</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855167151753793</v>
+        <v>4.855162050318697</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.852357693574106</v>
+        <v>4.852402739078928</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.829698191112037</v>
+        <v>4.829730889099014</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.837416089271967</v>
+        <v>4.837458957873187</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.889954203537254</v>
+        <v>4.890029808707493</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.916972517616423</v>
+        <v>4.917018397660206</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.926183679008323</v>
+        <v>4.926230097432656</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.916318650609378</v>
+        <v>4.916363097484283</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.897293241013316</v>
+        <v>4.897329059858356</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.895255479231791</v>
+        <v>4.89531479167452</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.895565019915264</v>
+        <v>4.895647534510284</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.892505698289563</v>
+        <v>4.89261579506663</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.876957371359505</v>
+        <v>4.877070879100707</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.853864889146354</v>
+        <v>4.853960932973328</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.827677437007777</v>
+        <v>4.827770037690033</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.818485177844041</v>
+        <v>4.818573722986791</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.788655893747689</v>
+        <v>4.788730779988402</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.760705762012693</v>
+        <v>4.760780615569157</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.749795147432301</v>
+        <v>4.749869544200058</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.753371300055935</v>
+        <v>4.753484595051215</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.748946584631105</v>
+        <v>4.749011820162109</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.750198801973537</v>
+        <v>4.750203509934606</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.751349863142135</v>
+        <v>4.752442095672347</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.742903062057859</v>
+        <v>4.744486127215519</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.733709728677135</v>
+        <v>4.735475681573572</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.725846346605833</v>
+        <v>4.727884781536575</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.715451920381577</v>
+        <v>4.717678397753788</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.709323577474668</v>
+        <v>4.711646966439731</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.701913577529641</v>
+        <v>4.704211300757581</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.701838693884852</v>
+        <v>4.703744303578752</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.704743353893174</v>
+        <v>4.706177747511294</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.728228805999112</v>
+        <v>4.727489312404872</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.734494109735509</v>
+        <v>4.732529492153688</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.740934336199333</v>
+        <v>4.737236149596411</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.711767134972384</v>
+        <v>4.716832103069737</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.759808954483865</v>
+        <v>4.757744369873497</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-08-22_12-46-21
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712843614851505</v>
+        <v>4.712842420107867</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711630423550748</v>
+        <v>4.711636001581605</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720136078954903</v>
+        <v>4.72014290111876</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706835152085264</v>
+        <v>4.706849258967008</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694180723335615</v>
+        <v>4.694194990527515</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678254724903558</v>
+        <v>4.67826911611701</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.67326354453935</v>
+        <v>4.673277971135797</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686339677831633</v>
+        <v>4.686354100996978</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702266647995987</v>
+        <v>4.702283982363745</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705516929205602</v>
+        <v>4.705528434890165</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694586054397642</v>
+        <v>4.694597786703011</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664607679476996</v>
+        <v>4.664620389543186</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649631169682602</v>
+        <v>4.649633082064813</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641340678568007</v>
+        <v>4.641345388711564</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636193623331474</v>
+        <v>4.636196598008389</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633915885856843</v>
+        <v>4.633922860839853</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.63736633664554</v>
+        <v>4.637367999678559</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634480472134383</v>
+        <v>4.634476557425128</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627713385568569</v>
+        <v>4.627701712316469</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.623980771779213</v>
+        <v>4.623968284541045</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599338343256662</v>
+        <v>4.59932602875006</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.57986650195293</v>
+        <v>4.579839933933183</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.561279640768287</v>
+        <v>4.561236619093001</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.523501126950199</v>
+        <v>4.523437633905067</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.520910537434944</v>
+        <v>4.520820381741716</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.533836362988693</v>
+        <v>4.533736753681771</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.552723478086444</v>
+        <v>4.552622115406988</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.585383370885342</v>
+        <v>4.585269864872978</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.604414729919091</v>
+        <v>4.604271106649184</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.677301889904502</v>
+        <v>4.677137015135493</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.713029090093043</v>
+        <v>4.712854205777175</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.779603053401912</v>
+        <v>4.779439652420752</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.814320165563305</v>
+        <v>4.814224187834157</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.812047714269141</v>
+        <v>4.811954022237529</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.821251335028221</v>
+        <v>4.821158073338756</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862470858903805</v>
+        <v>4.862461785366352</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855162050318697</v>
+        <v>4.855157041537283</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.852402739078928</v>
+        <v>4.852446677288039</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.829730889099014</v>
+        <v>4.829762756479057</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.837458957873187</v>
+        <v>4.837500751950109</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.890029808707493</v>
+        <v>4.89010354209632</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.917018397660206</v>
+        <v>4.917063099591754</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.926230097432656</v>
+        <v>4.926275331489264</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.916363097484283</v>
+        <v>4.916406450672321</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.897329059858356</v>
+        <v>4.897363990940917</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.89531479167452</v>
+        <v>4.89537266929996</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.895647534510284</v>
+        <v>4.895728092886706</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.89261579506663</v>
+        <v>4.892723256360433</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.877070879100707</v>
+        <v>4.877181658204638</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.853960932973328</v>
+        <v>4.854054638394473</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.827770037690033</v>
+        <v>4.82786033143853</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.818573722986791</v>
+        <v>4.818660049243936</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.788730779988402</v>
+        <v>4.788803740613162</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.760780615569157</v>
+        <v>4.760853602453043</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.749869544200058</v>
+        <v>4.749942167256583</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.753484595051215</v>
+        <v>4.753595418880706</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.749011820162109</v>
+        <v>4.74907589256321</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.750203509934606</v>
+        <v>4.750208524706331</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.752442095672347</v>
+        <v>4.754784075523244</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.744486127215519</v>
+        <v>4.747708979065561</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.735475681573572</v>
+        <v>4.739270184620971</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.727884781536575</v>
+        <v>4.732549737596853</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.717678397753788</v>
+        <v>4.722751017468158</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.711646966439731</v>
+        <v>4.717424882613404</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.704211300757581</v>
+        <v>4.710597066615271</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.703744303578752</v>
+        <v>4.710499824940905</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.706177747511294</v>
+        <v>4.713447220702193</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.727489312404872</v>
+        <v>4.735344575982831</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.732529492153688</v>
+        <v>4.742104250410291</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.737236149596411</v>
+        <v>4.748435788448724</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.716832103069737</v>
+        <v>4.73467708360156</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.757744369873497</v>
+        <v>4.784731591623908</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-08-24_20-44-19
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712842420107867</v>
+        <v>4.71284125485952</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711636001581605</v>
+        <v>4.711641441084574</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.72014290111876</v>
+        <v>4.720149555133757</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706849258967008</v>
+        <v>4.706863017153669</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694194990527515</v>
+        <v>4.694208905078894</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.67826911611701</v>
+        <v>4.678283151621889</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673277971135797</v>
+        <v>4.673292041262225</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686354100996978</v>
+        <v>4.686368168080012</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702283982363745</v>
+        <v>4.702300890866939</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705528434890165</v>
+        <v>4.705539658364719</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694597786703011</v>
+        <v>4.694609231063516</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664620389543186</v>
+        <v>4.664632787313359</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649633082064813</v>
+        <v>4.649634955759175</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641345388711564</v>
+        <v>4.641349989576914</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636196598008389</v>
+        <v>4.636199499535147</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633922860839853</v>
+        <v>4.633929665638824</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637367999678559</v>
+        <v>4.63736962759058</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634476557425128</v>
+        <v>4.634472740885702</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627701712316469</v>
+        <v>4.62769032411279</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.623968284541045</v>
+        <v>4.623956103505898</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.59932602875006</v>
+        <v>4.599314017256396</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.579839933933183</v>
+        <v>4.57981403616755</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.561236619093001</v>
+        <v>4.561194690175228</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.523437633905067</v>
+        <v>4.523375743825016</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.520820381741716</v>
+        <v>4.520732495086142</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.533736753681771</v>
+        <v>4.53363963701983</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.552622115406988</v>
+        <v>4.55252327730008</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.585269864872978</v>
+        <v>4.585159167911386</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.604271106649184</v>
+        <v>4.604130971247493</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.677137015135493</v>
+        <v>4.676976151057747</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.712854205777175</v>
+        <v>4.712683577398217</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.779439652420752</v>
+        <v>4.779280147032795</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.814224187834157</v>
+        <v>4.814130504297164</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.811954022237529</v>
+        <v>4.811862551543636</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.821158073338756</v>
+        <v>4.821066999644182</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862461785366352</v>
+        <v>4.862452904080273</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855157041537283</v>
+        <v>4.8551521232288</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.852446677288039</v>
+        <v>4.852489548497751</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.829762756479057</v>
+        <v>4.829793824458221</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.837500751950109</v>
+        <v>4.837541511328388</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.89010354209632</v>
+        <v>4.890175472306089</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.917063099591754</v>
+        <v>4.917106668040034</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.926275331489264</v>
+        <v>4.926319425737425</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.916406450672321</v>
+        <v>4.916448749887798</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.897363990940917</v>
+        <v>4.897398066691693</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.89537266929996</v>
+        <v>4.895429163348947</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.895728092886706</v>
+        <v>4.895806763469008</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.892723256360433</v>
+        <v>4.892828175326684</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.877181658204638</v>
+        <v>4.877289805629209</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.854054638394473</v>
+        <v>4.854146089640638</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.82786033143853</v>
+        <v>4.827948403277546</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.818660049243936</v>
+        <v>4.818744238887083</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.788803740613162</v>
+        <v>4.788874848645554</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.760853602453043</v>
+        <v>4.760924790987508</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.749942167256583</v>
+        <v>4.750013078357403</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.753595418880706</v>
+        <v>4.75370384956544</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.74907589256321</v>
+        <v>4.749138828467181</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.750208524706331</v>
+        <v>4.750213821476697</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.754784075523244</v>
+        <v>4.756989575339025</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.747708979065561</v>
+        <v>4.750759580187355</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.739270184620971</v>
+        <v>4.742843658777504</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.732549737596853</v>
+        <v>4.736673421626147</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.722751017468158</v>
+        <v>4.72749681402027</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.717424882613404</v>
+        <v>4.722806848505634</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.710597066615271</v>
+        <v>4.716531677929979</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.710499824940905</v>
+        <v>4.716761771466116</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.713447220702193</v>
+        <v>4.720158643395044</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.735344575982831</v>
+        <v>4.742487914886367</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.742104250410291</v>
+        <v>4.750633793419824</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.748435788448724</v>
+        <v>4.758184134166021</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.73467708360156</v>
+        <v>4.749259297643462</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.784731591623908</v>
+        <v>4.802205483583688</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-08-25_20-36-08
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712846097420315</v>
+        <v>4.712840118027586</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711618830188129</v>
+        <v>4.7116467471561</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720121904031337</v>
+        <v>4.720156047139484</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706805837848545</v>
+        <v>4.706876439412719</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694151076029293</v>
+        <v>4.694222479901139</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678224819870794</v>
+        <v>4.678296844442063</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.67323356635613</v>
+        <v>4.673305767966267</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.68630970778423</v>
+        <v>4.686381892103158</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702230635678957</v>
+        <v>4.702317389002456</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705493027545288</v>
+        <v>4.705550609883721</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694561681374751</v>
+        <v>4.694620397948412</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664581274050811</v>
+        <v>4.664644884155003</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649627224231333</v>
+        <v>4.649636791871246</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641330914562894</v>
+        <v>4.641354484909127</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636187443174827</v>
+        <v>4.636202330577439</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.63390139916755</v>
+        <v>4.633936306402844</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637362900727519</v>
+        <v>4.637371221449646</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634488611584377</v>
+        <v>4.634469018875077</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627737631089568</v>
+        <v>4.627679210650122</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.624006712220047</v>
+        <v>4.623944217551363</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.59936392831934</v>
+        <v>4.599302297736058</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.57992175544671</v>
+        <v>4.579788783640073</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.561369137454071</v>
+        <v>4.561153812982853</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.523633177077492</v>
+        <v>4.523315396884108</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.521098015870626</v>
+        <v>4.520646793051565</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.534043452436739</v>
+        <v>4.533544920817305</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.552934172932449</v>
+        <v>4.552426870873058</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.585619247260254</v>
+        <v>4.585051177335681</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.604712972954394</v>
+        <v>4.603994198447451</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.677644285310148</v>
+        <v>4.676819153400597</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.713392278163496</v>
+        <v>4.712517051797214</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.779942125656504</v>
+        <v>4.779124399907273</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.814519348159346</v>
+        <v>4.814039033871496</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.812242092889782</v>
+        <v>4.811773224359676</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.821444744027136</v>
+        <v>4.820978038155424</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862489607525831</v>
+        <v>4.862444209151996</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855172348069871</v>
+        <v>4.855147293259928</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.852311498424342</v>
+        <v>4.852531391074251</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.829664629669033</v>
+        <v>4.829824122700839</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.837372104254654</v>
+        <v>4.837581273893131</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.889876654461964</v>
+        <v>4.890245664629983</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.916925412467084</v>
+        <v>4.917149145415987</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.926136029314856</v>
+        <v>4.926362422538087</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.916273068322199</v>
+        <v>4.916490032953103</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.897256500324331</v>
+        <v>4.897431317988815</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.895194678180704</v>
+        <v>4.895484322660807</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.895480477349015</v>
+        <v>4.895883611543209</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.892392868286545</v>
+        <v>4.892930640798982</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.876841033215998</v>
+        <v>4.877395413804946</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.853766418441269</v>
+        <v>4.854235366951965</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.827582439980519</v>
+        <v>4.828034334109812</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.818394327271329</v>
+        <v>4.818826370175229</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.788579004995858</v>
+        <v>4.788944173477306</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.760628969991527</v>
+        <v>4.760994246231805</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.752378059141657</v>
+        <v>4.750082336468907</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.75307630305622</v>
+        <v>4.753809961976353</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.747355277524941</v>
+        <v>4.749200653956312</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.746026366701452</v>
+        <v>4.750219377183867</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.750993790179465</v>
+        <v>4.756919995697224</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.744559479843293</v>
+        <v>4.752598741846091</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.734327919124137</v>
+        <v>4.745234366807482</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.727868342503395</v>
+        <v>4.739470643804835</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.717317857775836</v>
+        <v>4.731419766687702</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.709831841644883</v>
+        <v>4.726891616531984</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.70056093403986</v>
+        <v>4.720950155801331</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.69776471045172</v>
+        <v>4.72128481725125</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.702932172265969</v>
+        <v>4.724868655097527</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.73383139178754</v>
+        <v>4.747159778890004</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.741167729209785</v>
+        <v>4.756045487434851</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.769710433100911</v>
+        <v>4.764089901446605</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.79232239453774</v>
+        <v>4.757574281800079</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.832422865821497</v>
+        <v>4.807077486323173</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.841675861389463</v>
+        <v>4.821982328339169</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-08-26_20-33-30
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712840118027586</v>
+        <v>4.712844840224624</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.7116467471561</v>
+        <v>4.711624701632696</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720156047139484</v>
+        <v>4.720129082188484</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706876439412719</v>
+        <v>4.706820683085859</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694222479901139</v>
+        <v>4.694166089929327</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678296844442063</v>
+        <v>4.678239964289413</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673305767966267</v>
+        <v>4.673248747755991</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686381892103158</v>
+        <v>4.686324884894194</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702317389002456</v>
+        <v>4.702248871476916</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705550609883721</v>
+        <v>4.705505130534636</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694620397948412</v>
+        <v>4.694574023144921</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664644884155003</v>
+        <v>4.664594645167623</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649636791871246</v>
+        <v>4.649629217467064</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641354484909127</v>
+        <v>4.641335855222693</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636202330577439</v>
+        <v>4.636190572702553</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633936306402844</v>
+        <v>4.633908734229723</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637371221449646</v>
+        <v>4.637364637380522</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634469018875077</v>
+        <v>4.634484488843593</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627679210650122</v>
+        <v>4.627725354698198</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.623944217551363</v>
+        <v>4.62399357690869</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599302297736058</v>
+        <v>4.599350972378991</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.579788783640073</v>
+        <v>4.57989376655106</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.561153812982853</v>
+        <v>4.561323798391345</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.523315396884108</v>
+        <v>4.523566285912659</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.520646793051565</v>
+        <v>4.521003050978553</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.533544920817305</v>
+        <v>4.533938561895234</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.552426870873058</v>
+        <v>4.552827463008827</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.585051177335681</v>
+        <v>4.585499793853546</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.603994198447451</v>
+        <v>4.604561972609049</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.676819153400597</v>
+        <v>4.677470926885665</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.712517051797214</v>
+        <v>4.713208391205432</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.779124399907273</v>
+        <v>4.779770494061145</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.814039033871496</v>
+        <v>4.814418522563294</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.811773224359676</v>
+        <v>4.812143709266119</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.820978038155424</v>
+        <v>4.821346864153186</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862444209151996</v>
+        <v>4.862480130827599</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855147293259928</v>
+        <v>4.855167151753793</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.852531391074251</v>
+        <v>4.852357693574106</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.829824122700839</v>
+        <v>4.829698191112037</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.837581273893131</v>
+        <v>4.837416089271967</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.890245664629983</v>
+        <v>4.889954203537254</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.917149145415987</v>
+        <v>4.916972517616423</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.926362422538087</v>
+        <v>4.926183679008323</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.916490032953103</v>
+        <v>4.916318650609378</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.897431317988815</v>
+        <v>4.897293241013316</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.895484322660807</v>
+        <v>4.895255479231791</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.895883611543209</v>
+        <v>4.895565019915264</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.892930640798982</v>
+        <v>4.892505698289563</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.877395413804946</v>
+        <v>4.876957371359505</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.854235366951965</v>
+        <v>4.853864889146354</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.828034334109812</v>
+        <v>4.827677437007777</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.818826370175229</v>
+        <v>4.818485177844041</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.788944173477306</v>
+        <v>4.788655893747689</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.760994246231805</v>
+        <v>4.760705762012693</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.750082336468907</v>
+        <v>4.752452012857145</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.753809961976353</v>
+        <v>4.753197409313406</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.749200653956312</v>
+        <v>4.747433245731481</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.750219377183867</v>
+        <v>4.746052635836393</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.756919995697224</v>
+        <v>4.750943111641114</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.752598741846091</v>
+        <v>4.74699059874663</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.745234366807482</v>
+        <v>4.737507502458533</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.739470643804835</v>
+        <v>4.731447010075863</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.731419766687702</v>
+        <v>4.722077287043064</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.726891616531984</v>
+        <v>4.715256129818776</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.720950155801331</v>
+        <v>4.705878219200089</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.72128481725125</v>
+        <v>4.703336162974395</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.724868655097527</v>
+        <v>4.70874310658956</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.747159778890004</v>
+        <v>4.739548344740749</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.756045487434851</v>
+        <v>4.747704316893927</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.764089901446605</v>
+        <v>4.776055717704232</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.757574281800079</v>
+        <v>4.798690904505682</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.807077486323173</v>
+        <v>4.83524719305438</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.821982328339169</v>
+        <v>4.84586168706995</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-08-26_21-36-29
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712844840224624</v>
+        <v>4.712839008585165</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711624701632696</v>
+        <v>4.711651924645695</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720129082188484</v>
+        <v>4.720162382980289</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706820683085859</v>
+        <v>4.706889537895989</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694166089929327</v>
+        <v>4.694235727283088</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678239964289413</v>
+        <v>4.678310206973411</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673248747755991</v>
+        <v>4.673319163666625</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686324884894194</v>
+        <v>4.686395285461647</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702248871476916</v>
+        <v>4.702333491524597</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705505130534636</v>
+        <v>4.705561299210882</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694574023144921</v>
+        <v>4.694631297325635</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664594645167623</v>
+        <v>4.664656690890653</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649629217467064</v>
+        <v>4.649638591468125</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641335855222693</v>
+        <v>4.64135887828478</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636190572702553</v>
+        <v>4.636205093672983</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633908734229723</v>
+        <v>4.633942788988497</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637364637380522</v>
+        <v>4.637372782282744</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634484488843593</v>
+        <v>4.634465387929804</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627725354698198</v>
+        <v>4.627668362111737</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.62399357690869</v>
+        <v>4.623932616087075</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599350972378991</v>
+        <v>4.599290859678867</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.57989376655106</v>
+        <v>4.57976415256293</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.561323798391345</v>
+        <v>4.561113948509009</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.523566285912659</v>
+        <v>4.523256536191377</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.521003050978553</v>
+        <v>4.520563195349251</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.533938561895234</v>
+        <v>4.533452517368703</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.552827463008827</v>
+        <v>4.552332807723158</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.585499793853546</v>
+        <v>4.584945795407897</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.604561972609049</v>
+        <v>4.603860668897649</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.677470926885665</v>
+        <v>4.676665884716041</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.713208391205432</v>
+        <v>4.71235448306151</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.779770494061145</v>
+        <v>4.778972280077395</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.814418522563294</v>
+        <v>4.813949699242722</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.812143709266119</v>
+        <v>4.811685966439917</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.821346864153186</v>
+        <v>4.820891116528518</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862480130827599</v>
+        <v>4.862435694918218</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855167151753793</v>
+        <v>4.855142549545346</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.852357693574106</v>
+        <v>4.852572241567708</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.829698191112037</v>
+        <v>4.829853679423442</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.837416089271967</v>
+        <v>4.837620075705461</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.889954203537254</v>
+        <v>4.890314181249007</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.916972517616423</v>
+        <v>4.917190572048175</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.926183679008323</v>
+        <v>4.926404362187248</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.916318650609378</v>
+        <v>4.916530335909576</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.897293241013316</v>
+        <v>4.897463774249188</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.895255479231791</v>
+        <v>4.895538193811827</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.895565019915264</v>
+        <v>4.895958699433806</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.892505698289563</v>
+        <v>4.893030737535568</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.876957371359505</v>
+        <v>4.877498570895452</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.853864889146354</v>
+        <v>4.854322546811083</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.827677437007777</v>
+        <v>4.828118200962895</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.818485177844041</v>
+        <v>4.818906517596144</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.788655893747689</v>
+        <v>4.789011781090468</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.760705762012693</v>
+        <v>4.761062030172109</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.752452012857145</v>
+        <v>4.750149997921318</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.753197409313406</v>
+        <v>4.753913827985225</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.747433245731481</v>
+        <v>4.749261394554219</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.746052635836393</v>
+        <v>4.750225170385359</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.750943111641114</v>
+        <v>4.756852372358496</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.74699059874663</v>
+        <v>4.754505718529667</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.737507502458533</v>
+        <v>4.747692671598472</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.731447010075863</v>
+        <v>4.742306699654907</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.722077287043064</v>
+        <v>4.735317760453425</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.715256129818776</v>
+        <v>4.730835816979694</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.705878219200089</v>
+        <v>4.725277837319332</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.703336162974395</v>
+        <v>4.725767185800688</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.70874310658956</v>
+        <v>4.729572025984346</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.739548344740749</v>
+        <v>4.751865503654647</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.747704316893927</v>
+        <v>4.761476243479237</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.776055717704232</v>
+        <v>4.770005115677276</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.798690904505682</v>
+        <v>4.765578503464358</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.83524719305438</v>
+        <v>4.812286470695111</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.84586168706995</v>
+        <v>4.828066229561163</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-08-27_20-36-56
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712839008585165</v>
+        <v>4.712837925554252</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711651924645695</v>
+        <v>4.711656978170707</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720162382980289</v>
+        <v>4.720168568222816</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706889537895989</v>
+        <v>4.706902324176331</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694235727283088</v>
+        <v>4.694248658928087</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678310206973411</v>
+        <v>4.678323251021219</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673319163666625</v>
+        <v>4.6733322401905</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686395285461647</v>
+        <v>4.686408359960816</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702333491524597</v>
+        <v>4.702349212489024</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705561299210882</v>
+        <v>4.70557173564819</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694631297325635</v>
+        <v>4.69464193869144</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664656690890653</v>
+        <v>4.664668217830161</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649638591468125</v>
+        <v>4.64964035557986</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.64135887828478</v>
+        <v>4.641363173121285</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636205093672983</v>
+        <v>4.636207791239104</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633942788988497</v>
+        <v>4.633949118977043</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637372782282744</v>
+        <v>4.637374311077632</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634465387929804</v>
+        <v>4.634461844753339</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627668362111737</v>
+        <v>4.627657769142756</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.623932616087075</v>
+        <v>4.623921289023277</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599290859678867</v>
+        <v>4.599279693072744</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.57976415256293</v>
+        <v>4.579740120302055</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.561113948509009</v>
+        <v>4.561075059648839</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.523256536191377</v>
+        <v>4.523199107613339</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.520563195349251</v>
+        <v>4.520481625569585</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.533452517368703</v>
+        <v>4.533362343180288</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.552332807723158</v>
+        <v>4.552241003670185</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.584945795407897</v>
+        <v>4.584842929025836</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.603860668897649</v>
+        <v>4.603730268817494</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.676665884716041</v>
+        <v>4.676516213981003</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.71235448306151</v>
+        <v>4.712195732102124</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.778972280077395</v>
+        <v>4.778823662576885</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.813949699242722</v>
+        <v>4.813862426647203</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.811685966439917</v>
+        <v>4.811600706917647</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.820891116528518</v>
+        <v>4.820806165671971</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862435694918218</v>
+        <v>4.862427355935315</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855142549545346</v>
+        <v>4.855137890048017</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.852572241567708</v>
+        <v>4.852612134818366</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.829853679423442</v>
+        <v>4.829882521481912</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.837620075705461</v>
+        <v>4.837657951110797</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.890314181249007</v>
+        <v>4.890381081415071</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.917190572048175</v>
+        <v>4.917230986308615</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.926404362187248</v>
+        <v>4.926445283039783</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.916530335909576</v>
+        <v>4.916569693120683</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.897463774249188</v>
+        <v>4.89749546351349</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.895538193811827</v>
+        <v>4.895590821244317</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.895958699433806</v>
+        <v>4.896032086668955</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.893030737535568</v>
+        <v>4.893128546449478</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.877498570895452</v>
+        <v>4.87759936104017</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.854322546811083</v>
+        <v>4.854407702160156</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.828118200962895</v>
+        <v>4.828200077218164</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.818906517596144</v>
+        <v>4.818984752090557</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.789011781090468</v>
+        <v>4.78907773426354</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.761062030172109</v>
+        <v>4.761128201899235</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.750149997921318</v>
+        <v>4.750216116551925</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.753913827985225</v>
+        <v>4.75401551660752</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.749261394554219</v>
+        <v>4.749321075220911</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.750225170385359</v>
+        <v>4.750231181137862</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.756852372358496</v>
+        <v>4.756786628682773</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.754505718529667</v>
+        <v>4.756597821861727</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.747692671598472</v>
+        <v>4.750371401675504</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.742306699654907</v>
+        <v>4.745330934039554</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.735317760453425</v>
+        <v>4.739288058118711</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.730835816979694</v>
+        <v>4.734993644016042</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.725277837319332</v>
+        <v>4.729829058890063</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.725767185800688</v>
+        <v>4.730502523676157</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.729572025984346</v>
+        <v>4.734558834998694</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.751865503654647</v>
+        <v>4.756921902164825</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.761476243479237</v>
+        <v>4.767303217529619</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.770005115677276</v>
+        <v>4.776375056454711</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.765578503464358</v>
+        <v>4.773963933676676</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.812286470695111</v>
+        <v>4.818810933181796</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.828066229561163</v>
+        <v>4.837604916816018</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-08-28_20-36-39
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712837925554252</v>
+        <v>4.712836868002851</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711656978170707</v>
+        <v>4.711661912130046</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720168568222816</v>
+        <v>4.720174608172298</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706902324176331</v>
+        <v>4.706914809281683</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694248658928087</v>
+        <v>4.694261285988447</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678323251021219</v>
+        <v>4.678335987834923</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.6733322401905</v>
+        <v>4.673345008808382</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686408359960816</v>
+        <v>4.686421126850782</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702349212489024</v>
+        <v>4.702364565293601</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.70557173564819</v>
+        <v>4.705581928062859</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.69464193869144</v>
+        <v>4.694652331097973</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664668217830161</v>
+        <v>4.664679474800681</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.64964035557986</v>
+        <v>4.64964208520083</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641363173121285</v>
+        <v>4.641367372685607</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636207791239104</v>
+        <v>4.636210425579799</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633949118977043</v>
+        <v>4.633955301690386</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637374311077632</v>
+        <v>4.637375808784586</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634461844753339</v>
+        <v>4.634458386206116</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627657769142756</v>
+        <v>4.627647422823318</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.623921289023277</v>
+        <v>4.623910226741618</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599279693072744</v>
+        <v>4.599268788374569</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.579740120302055</v>
+        <v>4.579716665308106</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.561075059648839</v>
+        <v>4.561037111085167</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.523199107613339</v>
+        <v>4.523143059609215</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.520481625569585</v>
+        <v>4.520402010951029</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.533362343180288</v>
+        <v>4.533274318720811</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.552241003670185</v>
+        <v>4.552151378508009</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.584842929025836</v>
+        <v>4.584742489452285</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.603730268817494</v>
+        <v>4.60360288967658</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.676516213981003</v>
+        <v>4.676370016227054</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.712195732102124</v>
+        <v>4.712040666260291</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.778823662576885</v>
+        <v>4.778678428101065</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.813862426647203</v>
+        <v>4.813777145671093</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.811600706917647</v>
+        <v>4.811517378115723</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.820806165671971</v>
+        <v>4.820723119566832</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862427355935315</v>
+        <v>4.8624191869693</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855137890048017</v>
+        <v>4.855133312779248</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.852612134818366</v>
+        <v>4.852651104055305</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.829882521481912</v>
+        <v>4.829910674452412</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.837657951110797</v>
+        <v>4.83769493283952</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.890381081415071</v>
+        <v>4.890446421621318</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.917230986308615</v>
+        <v>4.917270424729629</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.926445283039783</v>
+        <v>4.926485221624493</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.916569693120683</v>
+        <v>4.916608137368152</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.89749546351349</v>
+        <v>4.897526412525326</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.895590821244317</v>
+        <v>4.895642247386959</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.896032086668955</v>
+        <v>4.896103830134773</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.893128546449478</v>
+        <v>4.893224144823312</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.87759936104017</v>
+        <v>4.877697864580785</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.854407702160156</v>
+        <v>4.854490902603081</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.828200077218164</v>
+        <v>4.828280032823713</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.818984752090557</v>
+        <v>4.819061141260564</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.78907773426354</v>
+        <v>4.789142092762887</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.761128201899235</v>
+        <v>4.761192817774277</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.750216116551925</v>
+        <v>4.750280743839257</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.75401551660752</v>
+        <v>4.754115094137584</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.749321075220911</v>
+        <v>4.749379720350619</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.750231181137862</v>
+        <v>4.750237390886774</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.756786628682773</v>
+        <v>4.756722691809647</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.756597821861727</v>
+        <v>4.759129498132911</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.750371401675504</v>
+        <v>4.753577066487587</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.745330934039554</v>
+        <v>4.748942719749329</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.739288058118711</v>
+        <v>4.743672105403475</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.734993644016042</v>
+        <v>4.739820584636075</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.729829058890063</v>
+        <v>4.735114007814286</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.730502523676157</v>
+        <v>4.73605460828283</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.734558834998694</v>
+        <v>4.740455448834731</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.756921902164825</v>
+        <v>4.763074798516851</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.767303217529619</v>
+        <v>4.774498676531957</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.776375056454711</v>
+        <v>4.784371483848702</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.773963933676676</v>
+        <v>4.78435368607878</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.818810933181796</v>
+        <v>4.828940820214944</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.837604916816018</v>
+        <v>4.854613391354675</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-08-29_09-21-07
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712836868002851</v>
+        <v>4.712835835042304</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711661912130046</v>
+        <v>4.711666730716956</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720174608172298</v>
+        <v>4.720180507887726</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706914809281683</v>
+        <v>4.706927003726762</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694261285988447</v>
+        <v>4.694273619097488</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678335987834923</v>
+        <v>4.678348428140446</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673345008808382</v>
+        <v>4.673357480266426</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686421126850782</v>
+        <v>4.686433596858696</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702364565293601</v>
+        <v>4.702379562716422</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705581928062859</v>
+        <v>4.705591884912444</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694652331097973</v>
+        <v>4.694662483178923</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664679474800681</v>
+        <v>4.664690471174596</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.64964208520083</v>
+        <v>4.649643781291072</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641367372685607</v>
+        <v>4.641371480102414</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636210425579799</v>
+        <v>4.636212998892295</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633955301690386</v>
+        <v>4.633961342205969</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637375808784586</v>
+        <v>4.63737727631805</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634458386206116</v>
+        <v>4.63445500929633</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627647422823318</v>
+        <v>4.627637314643607</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.623910226741618</v>
+        <v>4.623899420067927</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599268788374569</v>
+        <v>4.599258136483055</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.579716665308106</v>
+        <v>4.579693767052322</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.561037111085167</v>
+        <v>4.561000069182272</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.523143059609215</v>
+        <v>4.523088343077802</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.520402010951029</v>
+        <v>4.520324282165362</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.533274318720811</v>
+        <v>4.533188368189679</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.552151378508009</v>
+        <v>4.552063855773376</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.584742489452285</v>
+        <v>4.584644392062913</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.60360288967658</v>
+        <v>4.60347842789594</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.676370016227054</v>
+        <v>4.676227172195381</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.712040666260291</v>
+        <v>4.711889158940868</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.778678428101065</v>
+        <v>4.77853646269062</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.813777145671093</v>
+        <v>4.813693789062794</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.811517378115723</v>
+        <v>4.811435915369705</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.820723119566832</v>
+        <v>4.820641915098518</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.8624191869693</v>
+        <v>4.862411182986276</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855133312779248</v>
+        <v>4.855128815798548</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.852651104055305</v>
+        <v>4.852689180988436</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.829910674452412</v>
+        <v>4.829938162706625</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.83769493283952</v>
+        <v>4.837731052100636</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.890446421621318</v>
+        <v>4.890510255760715</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.917270424729629</v>
+        <v>4.917308922112444</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.926485221624493</v>
+        <v>4.926524212751102</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.916608137368152</v>
+        <v>4.916645699941575</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.897526412525326</v>
+        <v>4.897556646805008</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.895642247386959</v>
+        <v>4.895692512767138</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.896103830134773</v>
+        <v>4.896173984219581</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.893224144823312</v>
+        <v>4.89331760650983</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.877697864580785</v>
+        <v>4.877794158272552</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.854490902603081</v>
+        <v>4.85457221459401</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.828280032823713</v>
+        <v>4.828358134492571</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.819061141260564</v>
+        <v>4.819135749563502</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.789142092762887</v>
+        <v>4.789204913520622</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.761192817774277</v>
+        <v>4.76125593158311</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.750280743839257</v>
+        <v>4.75034392902882</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.754115094137584</v>
+        <v>4.754212624276668</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.749379720350619</v>
+        <v>4.749437353772034</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.750237390886774</v>
+        <v>4.750243782364583</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.756722691809647</v>
+        <v>4.756660492436497</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.759129498132911</v>
+        <v>4.76100742692861</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.753577066487587</v>
+        <v>4.755983231014248</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.748942719749329</v>
+        <v>4.751608098819657</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.743672105403475</v>
+        <v>4.747191763424359</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.739820584636075</v>
+        <v>4.743408998223371</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.735114007814286</v>
+        <v>4.738990337536901</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.73605460828283</v>
+        <v>4.740034262900068</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.740455448834731</v>
+        <v>4.744575498996959</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.763074798516851</v>
+        <v>4.767067435456217</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.774498676531957</v>
+        <v>4.778749129520552</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.784371483848702</v>
+        <v>4.788639269777972</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.78435368607878</v>
+        <v>4.789231587718302</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.828940820214944</v>
+        <v>4.830446949153044</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.854613391354675</v>
+        <v>4.849814359820475</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-08-31_20-38-19
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712835835042304</v>
+        <v>4.712834825824801</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711666730716956</v>
+        <v>4.711671437930885</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720180507887726</v>
+        <v>4.72018627219596</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706927003726762</v>
+        <v>4.706938917542571</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694273619097488</v>
+        <v>4.694285668399374</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678348428140446</v>
+        <v>4.678360582170288</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673357480266426</v>
+        <v>4.673369664816581</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686433596858696</v>
+        <v>4.686445780218771</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702379562716422</v>
+        <v>4.702394216951226</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705591884912444</v>
+        <v>4.705601614268216</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694662483178923</v>
+        <v>4.694672403173422</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664690471174596</v>
+        <v>4.664701215895507</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649643781291072</v>
+        <v>4.649645444777589</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641371480102414</v>
+        <v>4.641375498361716</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636212998892295</v>
+        <v>4.636215513273164</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633961342205969</v>
+        <v>4.633967245370634</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.63737727631805</v>
+        <v>4.63737871455822</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.63445500929633</v>
+        <v>4.634451711171359</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627637314643607</v>
+        <v>4.627627436480571</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.623899420067927</v>
+        <v>4.623888860246888</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599258136483055</v>
+        <v>4.599247728713496</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.579693767052322</v>
+        <v>4.579671405966883</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.561000069182272</v>
+        <v>4.560963901887172</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.523088343077802</v>
+        <v>4.523034911215071</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.520324282165362</v>
+        <v>4.520248373117889</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.533188368189679</v>
+        <v>4.533104419301198</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.552063855773376</v>
+        <v>4.551978362530614</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.584644392062913</v>
+        <v>4.584548556111411</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.60347842789594</v>
+        <v>4.603356784569397</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.676227172195381</v>
+        <v>4.676087568015044</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.711889158940868</v>
+        <v>4.711741089270481</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.77853646269062</v>
+        <v>4.778397657436251</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.813693789062794</v>
+        <v>4.813612292557844</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.811435915369705</v>
+        <v>4.811356256862577</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.820641915098518</v>
+        <v>4.820562491899524</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862411182986276</v>
+        <v>4.862403339143379</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855128815798548</v>
+        <v>4.855124397213316</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.852689180988436</v>
+        <v>4.852726395894274</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.829938162706625</v>
+        <v>4.829965009481745</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.837731052100636</v>
+        <v>4.837766338669024</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.890510255760715</v>
+        <v>4.890572635273829</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.917308922112444</v>
+        <v>4.917346511628207</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.926524212751102</v>
+        <v>4.926562289609841</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.916645699941575</v>
+        <v>4.916682410722043</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.897556646805008</v>
+        <v>4.897586190718396</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.895692512767138</v>
+        <v>4.895741656115872</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.896173984219581</v>
+        <v>4.896242600948872</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.89331760650983</v>
+        <v>4.893409002119448</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.877794158272552</v>
+        <v>4.877888315481715</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.85457221459401</v>
+        <v>4.85465170161326</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.828358134492571</v>
+        <v>4.828434445887344</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.819135749563502</v>
+        <v>4.819208638492531</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.789204913520622</v>
+        <v>4.789266250800076</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.76125593158311</v>
+        <v>4.761317594680588</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.75034392902882</v>
+        <v>4.750405719251049</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.754212624276668</v>
+        <v>4.754308168254125</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.749437353772034</v>
+        <v>4.749493998750534</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.750243782364583</v>
+        <v>4.750250339497345</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.756660492436497</v>
+        <v>4.756599964611548</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.76100742692861</v>
+        <v>4.762787300863545</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.755983231014248</v>
+        <v>4.758253640187151</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.751608098819657</v>
+        <v>4.754104917172948</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.747191763424359</v>
+        <v>4.750223664559626</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.743408998223371</v>
+        <v>4.746772851259509</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.738990337536901</v>
+        <v>4.742615139920922</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.740034262900068</v>
+        <v>4.743744000505136</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.744575498996959</v>
+        <v>4.748400231167346</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.767067435456217</v>
+        <v>4.770728329371779</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.778749129520552</v>
+        <v>4.782571101618919</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.788639269777972</v>
+        <v>4.792402995737838</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.789231587718302</v>
+        <v>4.793366839446707</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.830446949153044</v>
+        <v>4.831400412838743</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.849814359820475</v>
+        <v>4.845972603668369</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-09-02_20-35-57
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712833839541064</v>
+        <v>4.712832875418177</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.71167603758856</v>
+        <v>4.711680533334295</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720191905704901</v>
+        <v>4.720197412815757</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706950560303888</v>
+        <v>4.706961941154908</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694297443576914</v>
+        <v>4.694308953877498</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678372459691571</v>
+        <v>4.678384070032195</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.67338157224467</v>
+        <v>4.673393211896583</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686457686700273</v>
+        <v>4.686469325633621</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702408539640409</v>
+        <v>4.702422541905824</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705611123836966</v>
+        <v>4.705620420981339</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694682098948327</v>
+        <v>4.694691578019</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664711717502483</v>
+        <v>4.664721984152661</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649647076555586</v>
+        <v>4.649648677489688</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641379430326007</v>
+        <v>4.641383278736963</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636217970724027</v>
+        <v>4.636220373156863</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633973015813567</v>
+        <v>4.633978657958356</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.63738012435255</v>
+        <v>4.637381506517183</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.63444848910977</v>
+        <v>4.634445340513878</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627617780576211</v>
+        <v>4.627608339517312</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.623878538918405</v>
+        <v>4.623868448095561</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599237556774217</v>
+        <v>4.599227612744592</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.579649563389379</v>
+        <v>4.579628221511104</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.560928578637743</v>
+        <v>4.560894070277161</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.522982719381583</v>
+        <v>4.522931724978985</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.520174220761429</v>
+        <v>4.520101764922954</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.533022403083566</v>
+        <v>4.532942253691506</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.551894829171015</v>
+        <v>4.551813189225717</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.584454904510482</v>
+        <v>4.584363363627475</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.603237865203496</v>
+        <v>4.603121579474588</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.675951094902706</v>
+        <v>4.675817648882166</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.711596341778501</v>
+        <v>4.71145480609908</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.778261908202653</v>
+        <v>4.778129115370366</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.813532594715284</v>
+        <v>4.813454636764644</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.811278343470198</v>
+        <v>4.811202118616677</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.820484792202194</v>
+        <v>4.820408760700804</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862395650780165</v>
+        <v>4.862388113410439</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855120055178386</v>
+        <v>4.855115787895467</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.852762777695957</v>
+        <v>4.852798354037979</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.829991236945649</v>
+        <v>4.830016866257644</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.837800820966748</v>
+        <v>4.837834526138904</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.890633609286652</v>
+        <v>4.890693224739239</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.917383224912041</v>
+        <v>4.917419092150668</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.926599483864217</v>
+        <v>4.926635825737487</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.916718298260215</v>
+        <v>4.916753389849286</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.897615067541145</v>
+        <v>4.897643299518731</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.895789714465892</v>
+        <v>4.895836723243383</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.896309730111637</v>
+        <v>4.896375419378741</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.893498399195611</v>
+        <v>4.893585862378944</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.877980406370055</v>
+        <v>4.878070498067533</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.854729424331574</v>
+        <v>4.854805440763643</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.828509027792383</v>
+        <v>4.828581938274418</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.819279866744884</v>
+        <v>4.819349490378821</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.789326156349857</v>
+        <v>4.789384679547377</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.761377856125272</v>
+        <v>4.761436762805332</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.750466159631957</v>
+        <v>4.750525293397056</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.75440178494221</v>
+        <v>4.754493530964822</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.749549677992165</v>
+        <v>4.749604413649063</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.750257047318527</v>
+        <v>4.750263891889619</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.75654104554078</v>
+        <v>4.756483675407609</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.762638961584386</v>
+        <v>4.762493918915899</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.759928768438259</v>
+        <v>4.761134712514429</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.75606767396167</v>
+        <v>4.757458686877721</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.752433147172376</v>
+        <v>4.754078712877288</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.749958325898364</v>
+        <v>4.752014452962229</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.745981152867685</v>
+        <v>4.74828822102817</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.747166536247583</v>
+        <v>4.749565662687342</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.751937549146144</v>
+        <v>4.754442604290783</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.774152414625174</v>
+        <v>4.776448083028205</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.786291555504267</v>
+        <v>4.788696320507602</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.796515220915427</v>
+        <v>4.799068914609546</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.79816513102995</v>
+        <v>4.800950454554766</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.833896062071885</v>
+        <v>4.833981789039971</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.846306363380102</v>
+        <v>4.843184936494402</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1306,7 +1306,7 @@
         <v>46360</v>
       </c>
       <c r="B115">
-        <v>4.835568908529755</v>
+        <v>4.822895842879978</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-09-03_20-36-29
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712832875418177</v>
+        <v>4.712831932717568</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711680533334295</v>
+        <v>4.711684928649627</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720197412815757</v>
+        <v>4.720202797734502</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706961941154908</v>
+        <v>4.706973068833176</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694308953877498</v>
+        <v>4.694320208137283</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678384070032195</v>
+        <v>4.678395422105249</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673393211896583</v>
+        <v>4.673404592702717</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686469325633621</v>
+        <v>4.686480705934749</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702422541905824</v>
+        <v>4.702436234377547</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705620420981339</v>
+        <v>4.705629512738832</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694691578019</v>
+        <v>4.694700847568724</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664721984152661</v>
+        <v>4.664732023642367</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649648677489688</v>
+        <v>4.649650248415107</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641383278736963</v>
+        <v>4.64138704622173</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636220373156863</v>
+        <v>4.636222722398977</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633978657958356</v>
+        <v>4.633984176034289</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637381506517183</v>
+        <v>4.637382861838313</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634445340513878</v>
+        <v>4.634442262902794</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627608339517312</v>
+        <v>4.627599106216516</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.623868448095561</v>
+        <v>4.623858580144033</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599227612744592</v>
+        <v>4.599217889054554</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.579628221511104</v>
+        <v>4.579607363328838</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.560894070277161</v>
+        <v>4.560860348974179</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.522931724978985</v>
+        <v>4.522881887334862</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.520101764922954</v>
+        <v>4.520030948141931</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.532942253691506</v>
+        <v>4.532863908231414</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.551813189225717</v>
+        <v>4.551733379191035</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.584363363627475</v>
+        <v>4.584273863093529</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.603121579474588</v>
+        <v>4.603007841001745</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.675817648882166</v>
+        <v>4.675687130522238</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.71145480609908</v>
+        <v>4.711316376692665</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.778129115370366</v>
+        <v>4.777999183594142</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.813454636764644</v>
+        <v>4.813378362462739</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.811202118616677</v>
+        <v>4.811127528138952</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.820408760700804</v>
+        <v>4.820334344422328</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862388113410439</v>
+        <v>4.862380722714486</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855115787895467</v>
+        <v>4.85511159361247</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.852798354037979</v>
+        <v>4.852833151356024</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.830016866257644</v>
+        <v>4.830041917625103</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.837834526138904</v>
+        <v>4.837867480124431</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.890693224739239</v>
+        <v>4.890751526505865</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.917419092150668</v>
+        <v>4.917454142164125</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.926635825737487</v>
+        <v>4.926671344093366</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.916753389849286</v>
+        <v>4.916787711593214</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.897643299518731</v>
+        <v>4.897670907922585</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.895836723243383</v>
+        <v>4.895882716353883</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.896375419378741</v>
+        <v>4.896439714413868</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.893585862378944</v>
+        <v>4.893671453561026</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.878070498067533</v>
+        <v>4.878158654833928</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.854805440763643</v>
+        <v>4.854879806411667</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.828581938274418</v>
+        <v>4.828653232832583</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.819349490378821</v>
+        <v>4.819417562960137</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.789384679547377</v>
+        <v>4.789441867532704</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.761436762805332</v>
+        <v>4.761494359556354</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.750525293397056</v>
+        <v>4.750583161968955</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.754493530964822</v>
+        <v>4.754583460800553</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.749604413649063</v>
+        <v>4.749658227326105</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.750263891889619</v>
+        <v>4.750270860226896</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.756483675407609</v>
+        <v>4.756427797204413</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.762493918915899</v>
+        <v>4.76235206715778</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.761134712514429</v>
+        <v>4.762706030408205</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.757458686877721</v>
+        <v>4.759279844712751</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.754078712877288</v>
+        <v>4.75607397039229</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.752014452962229</v>
+        <v>4.754568023475639</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.74828822102817</v>
+        <v>4.75108796291676</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.749565662687342</v>
+        <v>4.752472836160237</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.754442604290783</v>
+        <v>4.757490985800829</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.776448083028205</v>
+        <v>4.779390667902778</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.788696320507602</v>
+        <v>4.791863423716597</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.799068914609546</v>
+        <v>4.802493090788424</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.800950454554766</v>
+        <v>4.804787237959069</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.833981789039971</v>
+        <v>4.835823024436628</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.843184936494402</v>
+        <v>4.843565335074592</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1306,7 +1306,7 @@
         <v>46360</v>
       </c>
       <c r="B115">
-        <v>4.822895842879978</v>
+        <v>4.826747793769653</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-09-04_20-37-56
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712831932717568</v>
+        <v>4.712831010733122</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711684928649627</v>
+        <v>4.71168922686229</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720202797734502</v>
+        <v>4.720208064482585</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706973068833176</v>
+        <v>4.706983951691935</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694320208137283</v>
+        <v>4.694331214803801</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678395422105249</v>
+        <v>4.678406524431807</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673404592702717</v>
+        <v>4.673415723200804</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686480705934749</v>
+        <v>4.686491836127864</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702436234377547</v>
+        <v>4.702449627220751</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705629512738832</v>
+        <v>4.705638405839541</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694700847568724</v>
+        <v>4.694709914466837</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664732023642367</v>
+        <v>4.664741843426842</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649650248415107</v>
+        <v>4.649651790138763</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.64138704622173</v>
+        <v>4.641390735298822</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636222722398977</v>
+        <v>4.636225020197635</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633984176034289</v>
+        <v>4.633989574086895</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637382861838313</v>
+        <v>4.637384191073489</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634442262902794</v>
+        <v>4.634439253905948</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627599106216516</v>
+        <v>4.627590073894623</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.623858580144033</v>
+        <v>4.62384892776285</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599217889054554</v>
+        <v>4.599208378465404</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.579607363328838</v>
+        <v>4.579586972599858</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.560860348974179</v>
+        <v>4.560827388148739</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.522881887334862</v>
+        <v>4.522833167595262</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.520030948141931</v>
+        <v>4.519961715519432</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.532863908231414</v>
+        <v>4.532787306598124</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.551733379191035</v>
+        <v>4.551655338365308</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.584273863093529</v>
+        <v>4.584186335625192</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.603007841001745</v>
+        <v>4.602896567134333</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.675687130522238</v>
+        <v>4.675559444691533</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.711316376692665</v>
+        <v>4.711180952585503</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.777999183594142</v>
+        <v>4.777872021576647</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.813378362462739</v>
+        <v>4.813303717959564</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.811127528138952</v>
+        <v>4.811054520159869</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.820334344422328</v>
+        <v>4.820261492605191</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862380722714486</v>
+        <v>4.862373474531698</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.85511159361247</v>
+        <v>4.855107470622771</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.852833151356024</v>
+        <v>4.852867194942277</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.830041917625103</v>
+        <v>4.830066410356356</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.837867480124431</v>
+        <v>4.837899707722274</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.890751526505865</v>
+        <v>4.890808557507354</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.917454142164125</v>
+        <v>4.917488402482022</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.926671344093366</v>
+        <v>4.92670606651135</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.916787711593214</v>
+        <v>4.916821288470572</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.897670907922585</v>
+        <v>4.897697913102599</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.895882716353883</v>
+        <v>4.89592772626272</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.896439714413868</v>
+        <v>4.896502658977615</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.893671453561026</v>
+        <v>4.893755232028496</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.878158654833928</v>
+        <v>4.878244938210257</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.854879806411667</v>
+        <v>4.854952574399732</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.828653232832583</v>
+        <v>4.828722964538615</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.819417562960137</v>
+        <v>4.819484135699017</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.789441867532704</v>
+        <v>4.789497765333463</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.761494359556354</v>
+        <v>4.7615506892716</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.750583161968955</v>
+        <v>4.750639805059125</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.754583460800553</v>
+        <v>4.754671626880339</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.749658227326105</v>
+        <v>4.749711140088568</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.750270860226896</v>
+        <v>4.750277940233844</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.756427797204413</v>
+        <v>4.756373356575038</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.76235206715778</v>
+        <v>4.762213304958135</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.762706030408205</v>
+        <v>4.764861523811039</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.759279844712751</v>
+        <v>4.761794693912442</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.75607397039229</v>
+        <v>4.758898169160707</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.754568023475639</v>
+        <v>4.757985660450013</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.75108796291676</v>
+        <v>4.75483262351217</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.752472836160237</v>
+        <v>4.756430265742793</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.757490985800829</v>
+        <v>4.761702236735063</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.779390667902778</v>
+        <v>4.783699518662432</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.791863423716597</v>
+        <v>4.796650124782015</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.802493090788424</v>
+        <v>4.807905318775878</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.804787237959069</v>
+        <v>4.811191674613352</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.835823024436628</v>
+        <v>4.841568139542115</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.843565335074592</v>
+        <v>4.850628546363197</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1306,7 +1306,7 @@
         <v>46360</v>
       </c>
       <c r="B115">
-        <v>4.826747793769653</v>
+        <v>4.845799150211744</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-09-05_09-37-14
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712831010733122</v>
+        <v>4.712830108789425</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.71168922686229</v>
+        <v>4.711693431154625</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720208064482585</v>
+        <v>4.720213216906934</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706983951691935</v>
+        <v>4.706994597721021</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694331214803801</v>
+        <v>4.694341981957095</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678406524431807</v>
+        <v>4.678417385162247</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673415723200804</v>
+        <v>4.673426611557261</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686491836127864</v>
+        <v>4.686502724366725</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702449627220751</v>
+        <v>4.702462730160829</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705638405839541</v>
+        <v>4.705647106722757</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694709914466837</v>
+        <v>4.694718785285693</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664741843426842</v>
+        <v>4.664751450638681</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649651790138763</v>
+        <v>4.649653303440368</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641390735298822</v>
+        <v>4.641394348383652</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636225020197635</v>
+        <v>4.636227268224399</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633989574086895</v>
+        <v>4.633994855987805</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637384191073489</v>
+        <v>4.637385494952849</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634439253905948</v>
+        <v>4.634436311257027</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627590073894623</v>
+        <v>4.627581236064026</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.62384892776285</v>
+        <v>4.623839483966398</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599208378465404</v>
+        <v>4.599199074051894</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.579586972599858</v>
+        <v>4.579567033799932</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.560827388148739</v>
+        <v>4.560795162402552</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.522833167595262</v>
+        <v>4.522785528624352</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.519961715519432</v>
+        <v>4.519894014577181</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.532787306598124</v>
+        <v>4.532712391322333</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.551655338365308</v>
+        <v>4.551579008696388</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.584186335625192</v>
+        <v>4.584100716857585</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.602896567134333</v>
+        <v>4.602787678753149</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.675559444691533</v>
+        <v>4.675434500328937</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.711180952585503</v>
+        <v>4.711048437125814</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.777872021576647</v>
+        <v>4.777747541856348</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.813303717959564</v>
+        <v>4.813230651672624</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.811054520159869</v>
+        <v>4.810983044969187</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.820261492605191</v>
+        <v>4.820190156585491</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862373474531698</v>
+        <v>4.862366364853571</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855107470622771</v>
+        <v>4.855103417264395</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.852867194942277</v>
+        <v>4.852900509006552</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.830066410356356</v>
+        <v>4.830090362910072</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.837899707722274</v>
+        <v>4.837931232653236</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.890808557507354</v>
+        <v>4.890864358816155</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.917488402482022</v>
+        <v>4.917521899414771</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.92670606651135</v>
+        <v>4.926740019357136</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.916821288470572</v>
+        <v>4.91685414439435</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.897697913102599</v>
+        <v>4.897724334536289</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.89592772626272</v>
+        <v>4.895971784070435</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.896502658977615</v>
+        <v>4.896564295025208</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.893755232028496</v>
+        <v>4.89383725459825</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.878244938210257</v>
+        <v>4.878329407160742</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.854952574399732</v>
+        <v>4.855023795599656</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.828722964538615</v>
+        <v>4.828791184167972</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.819484135699017</v>
+        <v>4.81954925757799</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.789497765333463</v>
+        <v>4.789552415981504</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.7615506892716</v>
+        <v>4.761605793005284</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.750639805059125</v>
+        <v>4.750695260754172</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.754671626880339</v>
+        <v>4.754758079680053</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.749711140088568</v>
+        <v>4.749763172470646</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.750277940233844</v>
+        <v>4.750285120638765</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.756373356575038</v>
+        <v>4.756320301667461</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.762213304958135</v>
+        <v>4.762077535098548</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.764861523811039</v>
+        <v>4.766756058081436</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.761794693912442</v>
+        <v>4.764063067463484</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.758898169160707</v>
+        <v>4.761469643844382</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.757985660450013</v>
+        <v>4.761355374445509</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.75483262351217</v>
+        <v>4.758642984572813</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.756430265742793</v>
+        <v>4.760484845355775</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.761702236735063</v>
+        <v>4.765975067827756</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.783699518662432</v>
+        <v>4.787994647781917</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.796650124782015</v>
+        <v>4.801255682457921</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.807905318775878</v>
+        <v>4.813036276748044</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.811191674613352</v>
+        <v>4.817101961757849</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.841568139542115</v>
+        <v>4.846785229862878</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.850628546363197</v>
+        <v>4.856576872747595</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1306,7 +1306,7 @@
         <v>46360</v>
       </c>
       <c r="B115">
-        <v>4.845799150211744</v>
+        <v>4.856901183949825</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forecast data 2026-09-06_21-48-30
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_forecast.xlsx
+++ b/public/data/files/AUDCNH_forecast.xlsx
@@ -722,7 +722,7 @@
         <v>45849</v>
       </c>
       <c r="B42">
-        <v>4.712830108789425</v>
+        <v>4.712829226240098</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -730,7 +730,7 @@
         <v>45856</v>
       </c>
       <c r="B43">
-        <v>4.711693431154625</v>
+        <v>4.711697544571431</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -738,7 +738,7 @@
         <v>45863</v>
       </c>
       <c r="B44">
-        <v>4.720213216906934</v>
+        <v>4.720218258689325</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -746,7 +746,7 @@
         <v>45870</v>
       </c>
       <c r="B45">
-        <v>4.706994597721021</v>
+        <v>4.707005014566412</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -754,7 +754,7 @@
         <v>45877</v>
       </c>
       <c r="B46">
-        <v>4.694341981957095</v>
+        <v>4.694352517329468</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -762,7 +762,7 @@
         <v>45884</v>
       </c>
       <c r="B47">
-        <v>4.678417385162247</v>
+        <v>4.678428012096183</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -770,7 +770,7 @@
         <v>45891</v>
       </c>
       <c r="B48">
-        <v>4.673426611557261</v>
+        <v>4.673437265587149</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -778,7 +778,7 @@
         <v>45898</v>
       </c>
       <c r="B49">
-        <v>4.686502724366725</v>
+        <v>4.686513378454542</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -786,7 +786,7 @@
         <v>45905</v>
       </c>
       <c r="B50">
-        <v>4.702462730160829</v>
+        <v>4.702475552506931</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -794,7 +794,7 @@
         <v>45912</v>
       </c>
       <c r="B51">
-        <v>4.705647106722757</v>
+        <v>4.70565562155251</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -802,7 +802,7 @@
         <v>45919</v>
       </c>
       <c r="B52">
-        <v>4.694718785285693</v>
+        <v>4.694727466316546</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -810,7 +810,7 @@
         <v>45926</v>
       </c>
       <c r="B53">
-        <v>4.664751450638681</v>
+        <v>4.664760852105111</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -818,7 +818,7 @@
         <v>45933</v>
       </c>
       <c r="B54">
-        <v>4.649653303440368</v>
+        <v>4.64965478907347</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -826,7 +826,7 @@
         <v>45940</v>
       </c>
       <c r="B55">
-        <v>4.641394348383652</v>
+        <v>4.641397887793743</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -834,7 +834,7 @@
         <v>45947</v>
       </c>
       <c r="B56">
-        <v>4.636227268224399</v>
+        <v>4.636229468079178</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -842,7 +842,7 @@
         <v>45954</v>
       </c>
       <c r="B57">
-        <v>4.633994855987805</v>
+        <v>4.634000025443999</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -850,7 +850,7 @@
         <v>45961</v>
       </c>
       <c r="B58">
-        <v>4.637385494952849</v>
+        <v>4.637386774180293</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -858,7 +858,7 @@
         <v>45968</v>
       </c>
       <c r="B59">
-        <v>4.634436311257027</v>
+        <v>4.634433432788318</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -866,7 +866,7 @@
         <v>45975</v>
       </c>
       <c r="B60">
-        <v>4.627581236064026</v>
+        <v>4.627572586513217</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -874,7 +874,7 @@
         <v>45982</v>
       </c>
       <c r="B61">
-        <v>4.623839483966398</v>
+        <v>4.623830242067585</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -882,7 +882,7 @@
         <v>45989</v>
       </c>
       <c r="B62">
-        <v>4.599199074051894</v>
+        <v>4.599189969185458</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -890,7 +890,7 @@
         <v>45996</v>
       </c>
       <c r="B63">
-        <v>4.579567033799932</v>
+        <v>4.579547532084061</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -898,7 +898,7 @@
         <v>46003</v>
       </c>
       <c r="B64">
-        <v>4.560795162402552</v>
+        <v>4.560763647454222</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -906,7 +906,7 @@
         <v>46010</v>
       </c>
       <c r="B65">
-        <v>4.522785528624352</v>
+        <v>4.522738934910617</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -914,7 +914,7 @@
         <v>46017</v>
       </c>
       <c r="B66">
-        <v>4.519894014577181</v>
+        <v>4.519827795125801</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46024</v>
       </c>
       <c r="B67">
-        <v>4.532712391322333</v>
+        <v>4.532639107427949</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -930,7 +930,7 @@
         <v>46031</v>
       </c>
       <c r="B68">
-        <v>4.551579008696388</v>
+        <v>4.551504334638937</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -938,7 +938,7 @@
         <v>46038</v>
       </c>
       <c r="B69">
-        <v>4.584100716857585</v>
+        <v>4.584016945188253</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -946,7 +946,7 @@
         <v>46045</v>
       </c>
       <c r="B70">
-        <v>4.602787678753149</v>
+        <v>4.60268110008412</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -954,7 +954,7 @@
         <v>46052</v>
       </c>
       <c r="B71">
-        <v>4.675434500328937</v>
+        <v>4.675312210228611</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -962,7 +962,7 @@
         <v>46059</v>
       </c>
       <c r="B72">
-        <v>4.711048437125814</v>
+        <v>4.710918737755398</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -970,7 +970,7 @@
         <v>46066</v>
       </c>
       <c r="B73">
-        <v>4.777747541856348</v>
+        <v>4.777625660608566</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -978,7 +978,7 @@
         <v>46073</v>
       </c>
       <c r="B74">
-        <v>4.813230651672624</v>
+        <v>4.81315911416908</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -986,7 +986,7 @@
         <v>46080</v>
       </c>
       <c r="B75">
-        <v>4.810983044969187</v>
+        <v>4.810913054911899</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -994,7 +994,7 @@
         <v>46087</v>
       </c>
       <c r="B76">
-        <v>4.820190156585491</v>
+        <v>4.820120289690154</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>46094</v>
       </c>
       <c r="B77">
-        <v>4.862366364853571</v>
+        <v>4.862359389817028</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>46101</v>
       </c>
       <c r="B78">
-        <v>4.855103417264395</v>
+        <v>4.855099431919156</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>46108</v>
       </c>
       <c r="B79">
-        <v>4.852900509006552</v>
+        <v>4.852933116733523</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>46115</v>
       </c>
       <c r="B80">
-        <v>4.830090362910072</v>
+        <v>4.830113792941448</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>46122</v>
       </c>
       <c r="B81">
-        <v>4.837931232653236</v>
+        <v>4.83796207761786</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1042,7 +1042,7 @@
         <v>46129</v>
       </c>
       <c r="B82">
-        <v>4.890864358816155</v>
+        <v>4.89091896975472</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1050,7 +1050,7 @@
         <v>46136</v>
       </c>
       <c r="B83">
-        <v>4.917521899414771</v>
+        <v>4.917554658120146</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1058,7 +1058,7 @@
         <v>46143</v>
       </c>
       <c r="B84">
-        <v>4.926740019357136</v>
+        <v>4.926773227848448</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1066,7 +1066,7 @@
         <v>46150</v>
       </c>
       <c r="B85">
-        <v>4.91685414439435</v>
+        <v>4.916886302267982</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1074,7 +1074,7 @@
         <v>46157</v>
       </c>
       <c r="B86">
-        <v>4.897724334536289</v>
+        <v>4.897750190874862</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1082,7 +1082,7 @@
         <v>46164</v>
       </c>
       <c r="B87">
-        <v>4.895971784070435</v>
+        <v>4.896014919583529</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1090,7 +1090,7 @@
         <v>46171</v>
       </c>
       <c r="B88">
-        <v>4.896564295025208</v>
+        <v>4.896624662798262</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1098,7 +1098,7 @@
         <v>46178</v>
       </c>
       <c r="B89">
-        <v>4.89383725459825</v>
+        <v>4.893917575744304</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1106,7 +1106,7 @@
         <v>46185</v>
       </c>
       <c r="B90">
-        <v>4.878329407160742</v>
+        <v>4.878412118205981</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>46192</v>
       </c>
       <c r="B91">
-        <v>4.855023795599656</v>
+        <v>4.855093518748941</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1122,7 +1122,7 @@
         <v>46199</v>
       </c>
       <c r="B92">
-        <v>4.828791184167972</v>
+        <v>4.828857940322568</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1130,7 +1130,7 @@
         <v>46206</v>
       </c>
       <c r="B93">
-        <v>4.81954925757799</v>
+        <v>4.819612975471641</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1138,7 +1138,7 @@
         <v>46213</v>
       </c>
       <c r="B94">
-        <v>4.789552415981504</v>
+        <v>4.789605860621924</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1146,7 +1146,7 @@
         <v>46220</v>
       </c>
       <c r="B95">
-        <v>4.761605793005284</v>
+        <v>4.761659710069396</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>46227</v>
       </c>
       <c r="B96">
-        <v>4.750695260754172</v>
+        <v>4.750749565597044</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1162,7 +1162,7 @@
         <v>46234</v>
       </c>
       <c r="B97">
-        <v>4.754758079680053</v>
+        <v>4.754842867808298</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1170,7 +1170,7 @@
         <v>46241</v>
       </c>
       <c r="B98">
-        <v>4.749763172470646</v>
+        <v>4.749814344484644</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1178,7 +1178,7 @@
         <v>46248</v>
       </c>
       <c r="B99">
-        <v>4.750285120638765</v>
+        <v>4.750292390937112</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1186,7 +1186,7 @@
         <v>46255</v>
       </c>
       <c r="B100">
-        <v>4.756320301667461</v>
+        <v>4.756268582995891</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1194,7 +1194,7 @@
         <v>46262</v>
       </c>
       <c r="B101">
-        <v>4.762077535098548</v>
+        <v>4.761944664291351</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1202,7 +1202,7 @@
         <v>46269</v>
       </c>
       <c r="B102">
-        <v>4.766756058081436</v>
+        <v>4.768560630600362</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1210,7 +1210,7 @@
         <v>46276</v>
       </c>
       <c r="B103">
-        <v>4.764063067463484</v>
+        <v>4.766262947625982</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1218,7 +1218,7 @@
         <v>46283</v>
       </c>
       <c r="B104">
-        <v>4.761469643844382</v>
+        <v>4.76389122825009</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1226,7 +1226,7 @@
         <v>46290</v>
       </c>
       <c r="B105">
-        <v>4.761355374445509</v>
+        <v>4.764357573874866</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1234,7 +1234,7 @@
         <v>46297</v>
       </c>
       <c r="B106">
-        <v>4.758642984572813</v>
+        <v>4.761886944507113</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1242,7 +1242,7 @@
         <v>46304</v>
       </c>
       <c r="B107">
-        <v>4.760484845355775</v>
+        <v>4.763875716223932</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1250,7 +1250,7 @@
         <v>46311</v>
       </c>
       <c r="B108">
-        <v>4.765975067827756</v>
+        <v>4.769604590455818</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1258,7 +1258,7 @@
         <v>46318</v>
       </c>
       <c r="B109">
-        <v>4.787994647781917</v>
+        <v>4.791818176310524</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1266,7 +1266,7 @@
         <v>46325</v>
       </c>
       <c r="B110">
-        <v>4.801255682457921</v>
+        <v>4.805605718258124</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1274,7 +1274,7 @@
         <v>46332</v>
       </c>
       <c r="B111">
-        <v>4.813036276748044</v>
+        <v>4.817977399660849</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1282,7 +1282,7 @@
         <v>46339</v>
       </c>
       <c r="B112">
-        <v>4.817101961757849</v>
+        <v>4.822561947468646</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1290,7 +1290,7 @@
         <v>46346</v>
       </c>
       <c r="B113">
-        <v>4.846785229862878</v>
+        <v>4.85112151113958</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1298,7 +1298,7 @@
         <v>46353</v>
       </c>
       <c r="B114">
-        <v>4.856576872747595</v>
+        <v>4.861080803518474</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1306,7 +1306,7 @@
         <v>46360</v>
       </c>
       <c r="B115">
-        <v>4.856901183949825</v>
+        <v>4.865269253010146</v>
       </c>
     </row>
   </sheetData>

</xml_diff>